<commit_message>
docs: refresh behavior specification
</commit_message>
<xml_diff>
--- a/docs/pronto-behavior-spec.xlsx
+++ b/docs/pronto-behavior-spec.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R1f8fa74c7e654fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R42a734b2e07b41b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R66d5b493d88a4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="Rb3bfd871e85a44ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R3eedf34938664f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="Rc4858afe2273403b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -720,7 +720,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="Feature ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1019,7 +1019,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot 73c28e5</x:v>
+        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot 885fe1e</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1048,7 +1048,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Status key: Regression-Covered = automated regression; Verified = direct command/build; Needs-Environment = live desktop/provider not exercised; Needs-Product-Decision = deferred by product boundary.</x:v>
+        <x:v>Status key: Regression-Covered = automated regression; Verified = direct command/build; Needs-Environment = live desktop/provider not exercised; Deferred = intentionally outside this slice; Needs-Product-Decision = unresolved product boundary.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -1221,7 +1221,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X5" s="36" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y5" s="36" t="str">
         <x:v>Verify macOS, Windows, and Linux folder permissions when the desktop shell is launched.</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X6" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y6" s="39" t="str">
         <x:v>Add configurable glob-pattern coverage in the provider/durable-state phase.</x:v>
@@ -1358,7 +1358,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X7" s="39" t="str">
         <x:v>Submodule promotion and symlink-root matrix remain for the discovery expansion.</x:v>
@@ -1427,7 +1427,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W8" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X8" s="39" t="str">
         <x:v>Provider and AI payload previews still need their own explicit contract.</x:v>
@@ -1496,7 +1496,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W9" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X9" s="39" t="str">
         <x:v>Add fetched-at evidence after fetch/provider refresh exists.</x:v>
@@ -1565,7 +1565,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W10" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X10" s="39" t="str">
         <x:v>Add staged + unstaged + untracked matrix cases as scan coverage grows.</x:v>
@@ -1634,7 +1634,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W11" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X11" s="39" t="str">
         <x:v>Add a fixture for unreadable paths on each supported OS.</x:v>
@@ -1703,7 +1703,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W12" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X12" s="39" t="str">
         <x:v>Add rebase/cherry-pick/revert/bisect fixtures before action work begins.</x:v>
@@ -1772,7 +1772,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W13" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X13" s="39" t="str">
         <x:v>Add dedicated integration-state fixture matrix and user correction persistence.</x:v>
@@ -1841,7 +1841,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W14" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X14" s="39" t="str">
         <x:v>Implement fetch freshness and policy controls in Phase 2.</x:v>
@@ -1910,7 +1910,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X15" s="39" t="str">
         <x:v>Add provider-backed conditions only after permission/freshness contracts exist.</x:v>
@@ -1979,7 +1979,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W16" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X16" s="39" t="str">
         <x:v>Add UI interaction verification once the Tauri shell is launched.</x:v>
@@ -2048,7 +2048,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W17" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X17" s="39" t="str">
         <x:v>Expose retention configuration and current-state independence in Phase 2.</x:v>
@@ -2117,7 +2117,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W18" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X18" s="39" t="str">
         <x:v>Verify crash recovery and migrate to SQLite when durable state expands.</x:v>
@@ -2193,7 +2193,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X19" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y19" s="39" t="str">
         <x:v>Run a human visual pass in the Tauri window and record screenshots/interaction outcomes.</x:v>
@@ -2268,7 +2268,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X20" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y20" s="39" t="str">
         <x:v>Verify evidence drawer content, expected-state action, and close behavior manually.</x:v>
@@ -2343,7 +2343,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X21" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y21" s="39" t="str">
         <x:v>Provider install/auth and refresh evidence are Phase 2 work.</x:v>
@@ -2351,85 +2351,91 @@
     </x:row>
     <x:row r="22" ht="70" customHeight="1">
       <x:c r="A22" s="51" t="str">
-        <x:v>CLI-001</x:v>
+        <x:v>UI-004</x:v>
       </x:c>
       <x:c r="B22" s="39" t="str">
-        <x:v>Companion CLI</x:v>
+        <x:v>Navigation</x:v>
       </x:c>
       <x:c r="C22" s="39" t="str">
-        <x:v>Terminal</x:v>
+        <x:v>Local and deferred navigation</x:v>
       </x:c>
       <x:c r="D22" s="39" t="str">
-        <x:v>As an operator, I can read a concise status or structured JSON snapshot from the same local registry.</x:v>
+        <x:v>As an operator, I can tell which workspace surfaces are available locally and which are deferred.</x:v>
       </x:c>
       <x:c r="E22" s="39" t="str">
         <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F22" s="39" t="str">
-        <x:v>Local-only</x:v>
+        <x:v>Local-only / no provider auth</x:v>
       </x:c>
       <x:c r="G22" s="39" t="str">
-        <x:v>Registry exists or is empty</x:v>
+        <x:v>Snapshot loaded or empty registry</x:v>
       </x:c>
       <x:c r="H22" s="39" t="str">
-        <x:v>Terminal</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I22" s="39" t="str">
-        <x:v>`status` and `status --json` call the same Rust core and return human-readable or machine-readable output.</x:v>
+        <x:v>Command center, Activity, and Settings render local content; Products, Groups, and Remote catalog render explicit deferred boundaries.</x:v>
       </x:c>
       <x:c r="J22" s="39" t="str">
-        <x:v>CLI output is useful for scripts and agrees with the desktop snapshot model.</x:v>
+        <x:v>Navigation never implies provider data or hides an unimplemented capability.</x:v>
       </x:c>
       <x:c r="K22" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:1469-1526; src-tauri/src/bin/pronto_cli.rs:1-3; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
+        <x:v>src/renderer/src/App.tsx; src/renderer/src/components/WorkspaceSurfaces.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:215-227, 304-306</x:v>
       </x:c>
       <x:c r="L22" s="39" t="str">
-        <x:v>CLI smoke</x:v>
+        <x:v>Typecheck/build + live desktop review</x:v>
       </x:c>
       <x:c r="M22" s="39" t="str">
-        <x:v>pnpm cli:json; cargo run --manifest-path src-tauri/Cargo.toml --bin pronto_cli -- status</x:v>
+        <x:v>pnpm typecheck; pnpm build:web; click each navigation item in the Tauri window</x:v>
       </x:c>
       <x:c r="N22" s="39" t="str">
-        <x:v>JSON status exits successfully and uses the shared portfolio snapshot contract.</x:v>
+        <x:v>Renderer source and build are green; live navigation and deferred-copy review remain environment checks.</x:v>
       </x:c>
       <x:c r="O22" s="39" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P22" s="39" t="str"/>
-      <x:c r="Q22" s="39" t="str"/>
-      <x:c r="R22" s="39" t="str"/>
+      <x:c r="Q22" s="39" t="str">
+        <x:v>Environment</x:v>
+      </x:c>
+      <x:c r="R22" s="39" t="str">
+        <x:v>The live Tauri window and interaction state are not exercised by static checks.</x:v>
+      </x:c>
       <x:c r="S22" s="39" t="str">
-        <x:v>No: direct command smoke.</x:v>
+        <x:v>Navigation now maps each item to a truthful local or deferred surface.</x:v>
       </x:c>
       <x:c r="T22" s="39" t="str">
-        <x:v>CLI is a thin entry point; policy remains in shared core.</x:v>
+        <x:v>No; static presentation is covered by build gates.</x:v>
       </x:c>
       <x:c r="U22" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:1498-1526; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
+        <x:v>Navigation boundaries remain data-independent and do not add provider state.</x:v>
       </x:c>
       <x:c r="V22" s="39" t="str">
+        <x:v>src/renderer/src/App.tsx; src/renderer/src/components/WorkspaceSurfaces.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:304-306</x:v>
+      </x:c>
+      <x:c r="W22" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W22" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
       <x:c r="X22" s="39" t="str">
-        <x:v>Implement desktop focus behavior for `pronto .` when the app lifecycle is available.</x:v>
-      </x:c>
-      <x:c r="Y22" s="39"/>
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y22" s="39" t="str">
+        <x:v>Verify active navigation, deferred copy, and Activity/Settings content manually.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="70" customHeight="1">
       <x:c r="A23" s="51" t="str">
-        <x:v>CLI-002</x:v>
+        <x:v>UI-005</x:v>
       </x:c>
       <x:c r="B23" s="39" t="str">
-        <x:v>Companion CLI</x:v>
+        <x:v>Accessibility</x:v>
       </x:c>
       <x:c r="C23" s="39" t="str">
-        <x:v>Executable wrapper</x:v>
+        <x:v>Keyboard focus and dismissal</x:v>
       </x:c>
       <x:c r="D23" s="39" t="str">
-        <x:v>As an operator, I can invoke `pronto` through the package-installed wrapper.</x:v>
+        <x:v>As an operator, I can focus search and dismiss open drawers with the keyboard.</x:v>
       </x:c>
       <x:c r="E23" s="39" t="str">
         <x:v>Local operator</x:v>
@@ -2438,136 +2444,148 @@
         <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G23" s="39" t="str">
-        <x:v>Rust toolchain available</x:v>
+        <x:v>A focused desktop window with search or a drawer available</x:v>
       </x:c>
       <x:c r="H23" s="39" t="str">
-        <x:v>Terminal</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I23" s="39" t="str">
-        <x:v>The Node wrapper forwards arguments to the native CLI without shell interpolation.</x:v>
+        <x:v>Cmd/Ctrl-K focuses global search and Escape closes evidence or repository drawers.</x:v>
       </x:c>
       <x:c r="J23" s="39" t="str">
-        <x:v>CLI arguments are forwarded safely and output remains the shared Rust output.</x:v>
+        <x:v>Keyboard shortcuts provide a fast path without invoking provider or modifying operations.</x:v>
       </x:c>
       <x:c r="K23" s="39" t="str">
-        <x:v>bin/pronto.mjs:1-22; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
+        <x:v>src/renderer/src/App.tsx; src/renderer/src/components/Drawers.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:356-380, 419-433</x:v>
       </x:c>
       <x:c r="L23" s="39" t="str">
-        <x:v>CLI smoke + source review</x:v>
+        <x:v>Typecheck/build + live keyboard review</x:v>
       </x:c>
       <x:c r="M23" s="39" t="str">
-        <x:v>node bin/pronto.mjs status --json</x:v>
+        <x:v>pnpm typecheck; pnpm build:web; use Cmd/Ctrl-K and Escape in the Tauri window</x:v>
       </x:c>
       <x:c r="N23" s="39" t="str">
-        <x:v>Wrapper exits successfully and returns JSON from the Rust binary.</x:v>
+        <x:v>Shortcut and dismissal handlers are present and compile; live focus behavior remains environment verification.</x:v>
       </x:c>
       <x:c r="O23" s="39" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P23" s="39" t="str"/>
-      <x:c r="Q23" s="39" t="str"/>
-      <x:c r="R23" s="39" t="str"/>
+      <x:c r="Q23" s="39" t="str">
+        <x:v>Environment</x:v>
+      </x:c>
+      <x:c r="R23" s="39" t="str">
+        <x:v>Static checks cannot prove native window focus or focus-return behavior.</x:v>
+      </x:c>
       <x:c r="S23" s="39" t="str">
-        <x:v>No: direct command smoke.</x:v>
+        <x:v>Added global search focus and drawer dismissal without expanding the action surface.</x:v>
       </x:c>
       <x:c r="T23" s="39" t="str">
-        <x:v>Wrapper is intentionally minimal; no duplicate business logic.</x:v>
+        <x:v>No; static interaction wiring is covered by build gates.</x:v>
       </x:c>
       <x:c r="U23" s="39" t="str">
-        <x:v>bin/pronto.mjs:1-22; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
+        <x:v>Keyboard handling stays in the renderer and is independent of provider state.</x:v>
       </x:c>
       <x:c r="V23" s="39" t="str">
+        <x:v>src/renderer/src/App.tsx; src/renderer/src/components/Drawers.tsx</x:v>
+      </x:c>
+      <x:c r="W23" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W23" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
       <x:c r="X23" s="39" t="str">
-        <x:v>Package installation and `pronto .` focus behavior remain to be verified.</x:v>
-      </x:c>
-      <x:c r="Y23" s="39"/>
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y23" s="39" t="str">
+        <x:v>Verify search focus, Escape dismissal, and focus behavior manually.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="70" customHeight="1">
       <x:c r="A24" s="51" t="str">
-        <x:v>BUILD-001</x:v>
+        <x:v>UI-006</x:v>
       </x:c>
       <x:c r="B24" s="39" t="str">
-        <x:v>Distribution</x:v>
+        <x:v>Local workspace</x:v>
       </x:c>
       <x:c r="C24" s="39" t="str">
-        <x:v>Tauri app bundle</x:v>
+        <x:v>Settings and Activity</x:v>
       </x:c>
       <x:c r="D24" s="39" t="str">
-        <x:v>As an operator, I can build a desktop app bundle and DMG from the repository.</x:v>
+        <x:v>As an operator, I can inspect local roots, storage, freshness, privacy, and transition history.</x:v>
       </x:c>
       <x:c r="E24" s="39" t="str">
-        <x:v>Maintainer</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F24" s="39" t="str">
         <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G24" s="39" t="str">
-        <x:v>Rust toolchain and pnpm dependencies installed</x:v>
+        <x:v>Snapshot metadata and optional transition events</x:v>
       </x:c>
       <x:c r="H24" s="39" t="str">
-        <x:v>Build system</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I24" s="39" t="str">
-        <x:v>The Tauri release build produces a macOS app bundle and DMG from the React renderer and Rust core.</x:v>
+        <x:v>Settings shows local roots, storage location, freshness, and privacy; Activity shows transition events or a truthful empty state.</x:v>
       </x:c>
       <x:c r="J24" s="39" t="str">
-        <x:v>A reproducible build artifact exists without relying on a web-only preview.</x:v>
+        <x:v>Local configuration and history are understandable without a server account or provider refresh.</x:v>
       </x:c>
       <x:c r="K24" s="39" t="str">
-        <x:v>src-tauri/tauri.conf.json:1-40; package.json:1-53; /Users/jakyeamos/Downloads/pronto_prd.md:196-210, 926-934</x:v>
+        <x:v>src/renderer/src/components/WorkspaceSurfaces.tsx; src/renderer/src/App.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:699-717, 859-900</x:v>
       </x:c>
       <x:c r="L24" s="39" t="str">
-        <x:v>Production build</x:v>
+        <x:v>Typecheck/build + live desktop review</x:v>
       </x:c>
       <x:c r="M24" s="39" t="str">
-        <x:v>pnpm build</x:v>
+        <x:v>pnpm typecheck; pnpm build:web; open Settings and Activity in the Tauri window</x:v>
       </x:c>
       <x:c r="N24" s="39" t="str">
-        <x:v>Release build previously produced `Pronto.app` and `Pronto_0.1.0_aarch64.dmg`; final incremental build is rerun below.</x:v>
+        <x:v>Surface content is wired to the local snapshot contract and builds successfully; live rendering remains environment verification.</x:v>
       </x:c>
       <x:c r="O24" s="39" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P24" s="39" t="str"/>
-      <x:c r="Q24" s="39" t="str"/>
-      <x:c r="R24" s="39" t="str"/>
+      <x:c r="Q24" s="39" t="str">
+        <x:v>Environment</x:v>
+      </x:c>
+      <x:c r="R24" s="39" t="str">
+        <x:v>The Tauri runtime and platform data directory are not exercised by static checks.</x:v>
+      </x:c>
       <x:c r="S24" s="39" t="str">
-        <x:v>No: direct build output.</x:v>
+        <x:v>Added local Settings and Activity surfaces with explicit freshness and privacy copy.</x:v>
       </x:c>
       <x:c r="T24" s="39" t="str">
-        <x:v>Tauri keeps native access behind Rust commands and avoids a Node renderer runtime.</x:v>
+        <x:v>No; static presentation is covered by build gates.</x:v>
       </x:c>
       <x:c r="U24" s="39" t="str">
-        <x:v>package.json; /Users/jakyeamos/Downloads/pronto_prd.md:926-934</x:v>
+        <x:v>The surfaces expose metadata and transition records without exposing source or diff content.</x:v>
       </x:c>
       <x:c r="V24" s="39" t="str">
+        <x:v>src/renderer/src/components/WorkspaceSurfaces.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
+      </x:c>
+      <x:c r="W24" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W24" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
       <x:c r="X24" s="39" t="str">
-        <x:v>Code signing/notarization is outside this local implementation.</x:v>
-      </x:c>
-      <x:c r="Y24" s="39"/>
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y24" s="39" t="str">
+        <x:v>Verify roots, storage path, freshness, privacy, event rows, and empty state manually.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="70" customHeight="1">
       <x:c r="A25" s="51" t="str">
-        <x:v>SAFE-001</x:v>
+        <x:v>UI-007</x:v>
       </x:c>
       <x:c r="B25" s="39" t="str">
-        <x:v>Safety</x:v>
+        <x:v>Filtering</x:v>
       </x:c>
       <x:c r="C25" s="39" t="str">
-        <x:v>Native command boundary</x:v>
+        <x:v>Filtered empty state</x:v>
       </x:c>
       <x:c r="D25" s="39" t="str">
-        <x:v>As an operator, I trust that the local scan cannot execute a user-controlled shell string or prohibited destructive Git action.</x:v>
+        <x:v>As an operator, I can tell the difference between an empty portfolio and filters that match nothing.</x:v>
       </x:c>
       <x:c r="E25" s="39" t="str">
         <x:v>Local operator</x:v>
@@ -2576,397 +2594,379 @@
         <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G25" s="39" t="str">
-        <x:v>Any repository path or branch name may contain shell-special characters</x:v>
+        <x:v>At least one repository or condition exists</x:v>
       </x:c>
       <x:c r="H25" s="39" t="str">
-        <x:v>Native core</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I25" s="39" t="str">
-        <x:v>Git calls use structured argument arrays and the current slice exposes only scan, persistence, and expected-state mutations.</x:v>
+        <x:v>When filters remove every row, the command center explains that no matches were found and offers Clear filters; no-repository states remain distinct.</x:v>
       </x:c>
       <x:c r="J25" s="39" t="str">
-        <x:v>No force push, hard reset, destructive checkout, branch deletion, or history rewrite is reachable in the implemented surface.</x:v>
+        <x:v>Filtering is recoverable and does not make local evidence appear missing.</x:v>
       </x:c>
       <x:c r="K25" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:251-297, 1434-1467; /Users/jakyeamos/Downloads/pronto_prd.md:541-551, 1175-1183</x:v>
+        <x:v>src/renderer/src/components/CommandCenterSurface.tsx; src/renderer/src/components/ConsolePrimitives.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:356-380</x:v>
       </x:c>
       <x:c r="L25" s="39" t="str">
-        <x:v>Static safety audit + hook-mode tests</x:v>
+        <x:v>Typecheck/build + live desktop review</x:v>
       </x:c>
       <x:c r="M25" s="39" t="str">
-        <x:v>rg 'Command::new|git ' src-tauri/src; GIT_INDEX_FILE=.git/index pnpm test; pre-cr run --workspace .</x:v>
+        <x:v>pnpm typecheck; pnpm build:web; apply filters until no rows match in the Tauri window</x:v>
       </x:c>
       <x:c r="N25" s="39" t="str">
-        <x:v>Structured process invocation is the only Git boundary; hook-mode tests pass after inherited Git env sanitization.</x:v>
+        <x:v>Filtered-empty and no-data states are represented separately in the renderer; live visual behavior remains environment verification.</x:v>
       </x:c>
       <x:c r="O25" s="39" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P25" s="39" t="str"/>
-      <x:c r="Q25" s="39" t="str"/>
-      <x:c r="R25" s="39" t="str"/>
+      <x:c r="Q25" s="39" t="str">
+        <x:v>Environment</x:v>
+      </x:c>
+      <x:c r="R25" s="39" t="str">
+        <x:v>Static checks cannot prove the visual distinction or Clear filters interaction.</x:v>
+      </x:c>
       <x:c r="S25" s="39" t="str">
-        <x:v>Yes: regression protects hook environment contamination; no destructive action test needed for absent commands.</x:v>
+        <x:v>Added a dedicated no-match state and recoverable Clear filters action.</x:v>
       </x:c>
       <x:c r="T25" s="39" t="str">
-        <x:v>Safety gate is explicit and small; adding actions requires a separate preflight/audit phase.</x:v>
+        <x:v>No; static presentation is covered by build gates.</x:v>
       </x:c>
       <x:c r="U25" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:251-297; /Users/jakyeamos/Downloads/pronto_prd.md:541-551, 1175-1183</x:v>
+        <x:v>The empty-state distinction is local renderer behavior and does not alter scan truth.</x:v>
       </x:c>
       <x:c r="V25" s="39" t="str">
+        <x:v>src/renderer/src/components/CommandCenterSurface.tsx; src/renderer/src/components/ConsolePrimitives.tsx</x:v>
+      </x:c>
+      <x:c r="W25" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W25" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
       <x:c r="X25" s="39" t="str">
-        <x:v>Add action-tier audit tests only when modifying actions are authorized and implemented.</x:v>
-      </x:c>
-      <x:c r="Y25" s="39"/>
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y25" s="39" t="str">
+        <x:v>Verify no-data, no-match, and Clear filters states manually.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="70" customHeight="1">
       <x:c r="A26" s="51" t="str">
-        <x:v>PROV-001</x:v>
+        <x:v>CLI-001</x:v>
       </x:c>
       <x:c r="B26" s="39" t="str">
-        <x:v>Provider</x:v>
+        <x:v>Companion CLI</x:v>
       </x:c>
       <x:c r="C26" s="39" t="str">
-        <x:v>GitHub identities / refresh</x:v>
+        <x:v>Terminal</x:v>
       </x:c>
       <x:c r="D26" s="39" t="str">
-        <x:v>As an operator, I can connect multiple identities and see permission degradation explicitly.</x:v>
+        <x:v>As an operator, I can read a concise status or structured JSON snapshot from the same local registry.</x:v>
       </x:c>
       <x:c r="E26" s="39" t="str">
-        <x:v>Provider-connected operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F26" s="39" t="str">
-        <x:v>Provider auth required</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G26" s="39" t="str">
-        <x:v>GitHub account and OS credential-store permissions</x:v>
+        <x:v>Registry exists or is empty</x:v>
       </x:c>
       <x:c r="H26" s="39" t="str">
-        <x:v>Desktop + provider API</x:v>
+        <x:v>Terminal</x:v>
       </x:c>
       <x:c r="I26" s="39" t="str">
-        <x:v>No provider adapter is enabled in this slice; the app does not claim GitHub identity, refresh, or permission results.</x:v>
+        <x:v>`status` and `status --json` call the same Rust core and return human-readable or machine-readable output.</x:v>
       </x:c>
       <x:c r="J26" s="39" t="str">
-        <x:v>No provider state is shown as current until identity and permission evidence exist.</x:v>
+        <x:v>CLI output is useful for scripts and agrees with the desktop snapshot model.</x:v>
       </x:c>
       <x:c r="K26" s="39" t="str">
-        <x:v>docs/implementation-plan.md:19-24; /Users/jakyeamos/Downloads/pronto_prd.md:296-306, 974-987</x:v>
+        <x:v>src-tauri/src/core.rs:1469-1526; src-tauri/src/bin/pronto_cli.rs:1-3; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
       </x:c>
       <x:c r="L26" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>CLI smoke</x:v>
       </x:c>
       <x:c r="M26" s="39" t="str">
-        <x:v>Deferred: requires explicit provider authority and credentials</x:v>
+        <x:v>pnpm cli:json; cargo run --manifest-path src-tauri/Cargo.toml --bin pronto_cli -- status</x:v>
       </x:c>
       <x:c r="N26" s="39" t="str">
-        <x:v>Provider identity, credential separation, and permission degradation are not implemented.</x:v>
+        <x:v>JSON status exits successfully and uses the shared portfolio snapshot contract.</x:v>
       </x:c>
       <x:c r="O26" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="P26" s="39" t="str"/>
-      <x:c r="Q26" s="39" t="str">
-        <x:v>Dependency</x:v>
-      </x:c>
-      <x:c r="R26" s="39" t="str">
-        <x:v>Requires network, provider auth, OS credential store, and a durable identity mapping.</x:v>
-      </x:c>
+      <x:c r="Q26" s="39" t="str"/>
+      <x:c r="R26" s="39" t="str"/>
       <x:c r="S26" s="39" t="str">
-        <x:v>Kept as an explicit deferred boundary; no fake adapter or mock provider result is added.</x:v>
+        <x:v>No: direct command smoke.</x:v>
       </x:c>
       <x:c r="T26" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>CLI is a thin entry point; policy remains in shared core.</x:v>
       </x:c>
       <x:c r="U26" s="39" t="str">
-        <x:v>Provider work is separated from local Git evidence by design.</x:v>
+        <x:v>src-tauri/src/core.rs:1498-1526; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
       </x:c>
       <x:c r="V26" s="39" t="str">
-        <x:v>pronto_prd.md:296-306, 974-987; docs/implementation-plan.md:49-54</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W26" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X26" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
-      <x:c r="Y26" s="39" t="str">
-        <x:v>Define provider permission and freshness contracts before implementation.</x:v>
-      </x:c>
+        <x:v>Implement desktop focus behavior for `pronto .` when the app lifecycle is available.</x:v>
+      </x:c>
+      <x:c r="Y26" s="39"/>
     </x:row>
     <x:row r="27" ht="70" customHeight="1">
       <x:c r="A27" s="51" t="str">
-        <x:v>REMOTE-001</x:v>
+        <x:v>CLI-002</x:v>
       </x:c>
       <x:c r="B27" s="39" t="str">
-        <x:v>Remote catalog</x:v>
+        <x:v>Companion CLI</x:v>
       </x:c>
       <x:c r="C27" s="39" t="str">
-        <x:v>Remote-only / clone</x:v>
+        <x:v>Executable wrapper</x:v>
       </x:c>
       <x:c r="D27" s="39" t="str">
-        <x:v>As an operator, I can import or clone a remote-only repository into a selected root.</x:v>
+        <x:v>As an operator, I can invoke `pronto` through the package-installed wrapper.</x:v>
       </x:c>
       <x:c r="E27" s="39" t="str">
-        <x:v>Provider-connected operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F27" s="39" t="str">
-        <x:v>Provider auth required</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G27" s="39" t="str">
-        <x:v>Remote repository catalog and clone permission</x:v>
+        <x:v>Rust toolchain available</x:v>
       </x:c>
       <x:c r="H27" s="39" t="str">
-        <x:v>Desktop + network</x:v>
+        <x:v>Terminal</x:v>
       </x:c>
       <x:c r="I27" s="39" t="str">
-        <x:v>Remote catalog and clone are not exposed by the local-first slice.</x:v>
+        <x:v>The Node wrapper forwards arguments to the native CLI without shell interpolation.</x:v>
       </x:c>
       <x:c r="J27" s="39" t="str">
-        <x:v>A remote repository is not represented as local until clone succeeds and the local scan registers it.</x:v>
+        <x:v>CLI arguments are forwarded safely and output remains the shared Rust output.</x:v>
       </x:c>
       <x:c r="K27" s="39" t="str">
-        <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:280-286, 849-857</x:v>
+        <x:v>bin/pronto.mjs:1-22; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
       </x:c>
       <x:c r="L27" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>CLI smoke + source review</x:v>
       </x:c>
       <x:c r="M27" s="39" t="str">
-        <x:v>Deferred: requires provider auth, network, clone preflight, and selected root</x:v>
+        <x:v>node bin/pronto.mjs status --json</x:v>
       </x:c>
       <x:c r="N27" s="39" t="str">
-        <x:v>No remote-only or clone path is implemented.</x:v>
+        <x:v>Wrapper exits successfully and returns JSON from the Rust binary.</x:v>
       </x:c>
       <x:c r="O27" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="P27" s="39" t="str"/>
-      <x:c r="Q27" s="39" t="str">
-        <x:v>Dependency</x:v>
-      </x:c>
-      <x:c r="R27" s="39" t="str">
-        <x:v>Requires network and exact destination authorization.</x:v>
-      </x:c>
+      <x:c r="Q27" s="39" t="str"/>
+      <x:c r="R27" s="39" t="str"/>
       <x:c r="S27" s="39" t="str">
-        <x:v>Deferred explicitly rather than pretending provider access exists.</x:v>
+        <x:v>No: direct command smoke.</x:v>
       </x:c>
       <x:c r="T27" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Wrapper is intentionally minimal; no duplicate business logic.</x:v>
       </x:c>
       <x:c r="U27" s="39" t="str">
-        <x:v>Clone is a modifying action and must arrive with fresh preflight/audit contracts.</x:v>
+        <x:v>bin/pronto.mjs:1-22; /Users/jakyeamos/Downloads/pronto_prd.md:723-743</x:v>
       </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>pronto_prd.md:280-286, 849-857</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X27" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
-      <x:c r="Y27" s="39" t="str">
-        <x:v>Define clone destination and audit semantics before adding the action.</x:v>
-      </x:c>
+        <x:v>Package installation and `pronto .` focus behavior remain to be verified.</x:v>
+      </x:c>
+      <x:c r="Y27" s="39"/>
     </x:row>
     <x:row r="28" ht="70" customHeight="1">
       <x:c r="A28" s="51" t="str">
-        <x:v>ACTION-001</x:v>
+        <x:v>BUILD-001</x:v>
       </x:c>
       <x:c r="B28" s="39" t="str">
-        <x:v>Safe actions</x:v>
+        <x:v>Distribution</x:v>
       </x:c>
       <x:c r="C28" s="39" t="str">
-        <x:v>Preflight / audit</x:v>
+        <x:v>Tauri app bundle</x:v>
       </x:c>
       <x:c r="D28" s="39" t="str">
-        <x:v>As an operator, I can see exact targets and fresh preflight evidence before a modifying action runs.</x:v>
+        <x:v>As an operator, I can build a desktop app bundle and DMG from the repository.</x:v>
       </x:c>
       <x:c r="E28" s="39" t="str">
-        <x:v>Local operator</x:v>
+        <x:v>Maintainer</x:v>
       </x:c>
       <x:c r="F28" s="39" t="str">
-        <x:v>Local-only or provider auth</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G28" s="39" t="str">
-        <x:v>A bounded modifying action is explicitly authorized</x:v>
+        <x:v>Rust toolchain and pnpm dependencies installed</x:v>
       </x:c>
       <x:c r="H28" s="39" t="str">
-        <x:v>Desktop + native core</x:v>
+        <x:v>Build system</x:v>
       </x:c>
       <x:c r="I28" s="39" t="str">
-        <x:v>The current slice exposes no modifying Git action, so preflight and audit are not falsely represented as complete.</x:v>
+        <x:v>The Tauri release build produces a macOS app bundle and DMG from the React renderer and Rust core.</x:v>
       </x:c>
       <x:c r="J28" s="39" t="str">
-        <x:v>No action is available without a fresh preflight, exact target, audit record, and post-action rescan.</x:v>
+        <x:v>A reproducible build artifact exists without relying on a web-only preview.</x:v>
       </x:c>
       <x:c r="K28" s="39" t="str">
-        <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:529-551, 1173-1183</x:v>
+        <x:v>src-tauri/tauri.conf.json:1-40; package.json:1-53; /Users/jakyeamos/Downloads/pronto_prd.md:196-210, 926-934</x:v>
       </x:c>
       <x:c r="L28" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Production build</x:v>
       </x:c>
       <x:c r="M28" s="39" t="str">
-        <x:v>Deferred until action policy is implemented</x:v>
+        <x:v>pnpm build</x:v>
       </x:c>
       <x:c r="N28" s="39" t="str">
-        <x:v>No modifying action adapter exists in this implementation.</x:v>
+        <x:v>Release build previously produced `Pronto.app` and `Pronto_0.1.0_aarch64.dmg`; final incremental build is rerun below.</x:v>
       </x:c>
       <x:c r="O28" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="P28" s="39" t="str"/>
-      <x:c r="Q28" s="39" t="str">
-        <x:v>Dependency</x:v>
-      </x:c>
-      <x:c r="R28" s="39" t="str">
-        <x:v>Requires action tiers, permission policy, audit schema, and failure semantics.</x:v>
-      </x:c>
+      <x:c r="Q28" s="39" t="str"/>
+      <x:c r="R28" s="39" t="str"/>
       <x:c r="S28" s="39" t="str">
-        <x:v>Read-only slice keeps the action surface absent.</x:v>
+        <x:v>No: direct build output.</x:v>
       </x:c>
       <x:c r="T28" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Tauri keeps native access behind Rust commands and avoids a Node renderer runtime.</x:v>
       </x:c>
       <x:c r="U28" s="39" t="str">
-        <x:v>Do not add action buttons before the preflight/audit contract is testable.</x:v>
+        <x:v>package.json; /Users/jakyeamos/Downloads/pronto_prd.md:926-934</x:v>
       </x:c>
       <x:c r="V28" s="39" t="str">
-        <x:v>pronto_prd.md:529-551</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W28" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X28" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
-      <x:c r="Y28" s="39" t="str">
-        <x:v>Phase 2 must add preflight tests before any modifying command.</x:v>
-      </x:c>
+        <x:v>Code signing/notarization is outside this local implementation.</x:v>
+      </x:c>
+      <x:c r="Y28" s="39"/>
     </x:row>
     <x:row r="29" ht="70" customHeight="1">
       <x:c r="A29" s="51" t="str">
-        <x:v>PR-001</x:v>
+        <x:v>SAFE-001</x:v>
       </x:c>
       <x:c r="B29" s="39" t="str">
-        <x:v>Pull requests</x:v>
+        <x:v>Safety</x:v>
       </x:c>
       <x:c r="C29" s="39" t="str">
-        <x:v>Provider lifecycle</x:v>
+        <x:v>Native command boundary</x:v>
       </x:c>
       <x:c r="D29" s="39" t="str">
-        <x:v>As an operator, I can create or merge a PR only when provider facts and permissions are verifiable.</x:v>
+        <x:v>As an operator, I trust that the local scan cannot execute a user-controlled shell string or prohibited destructive Git action.</x:v>
       </x:c>
       <x:c r="E29" s="39" t="str">
-        <x:v>Provider-connected operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F29" s="39" t="str">
-        <x:v>Provider auth required</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G29" s="39" t="str">
-        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
+        <x:v>Any repository path or branch name may contain shell-special characters</x:v>
       </x:c>
       <x:c r="H29" s="39" t="str">
-        <x:v>Desktop + provider API</x:v>
+        <x:v>Native core</x:v>
       </x:c>
       <x:c r="I29" s="39" t="str">
-        <x:v>PR creation, review evidence, and merge actions are explicit deferred boundaries.</x:v>
+        <x:v>Git calls use structured argument arrays and the current slice exposes only scan, persistence, and expected-state mutations.</x:v>
       </x:c>
       <x:c r="J29" s="39" t="str">
-        <x:v>Unknown checks or reviews never become a merge-eligible state.</x:v>
+        <x:v>No force push, hard reset, destructive checkout, branch deletion, or history rewrite is reachable in the implemented surface.</x:v>
       </x:c>
       <x:c r="K29" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>src-tauri/src/core.rs:251-297, 1434-1467; /Users/jakyeamos/Downloads/pronto_prd.md:541-551, 1175-1183</x:v>
       </x:c>
       <x:c r="L29" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Static safety audit + hook-mode tests</x:v>
       </x:c>
       <x:c r="M29" s="39" t="str">
-        <x:v>Deferred: provider permission and PR API required</x:v>
+        <x:v>rg 'Command::new|git ' src-tauri/src; GIT_INDEX_FILE=.git/index pnpm test; pre-cr run --workspace .</x:v>
       </x:c>
       <x:c r="N29" s="39" t="str">
-        <x:v>No PR lifecycle implementation is present.</x:v>
+        <x:v>Structured process invocation is the only Git boundary; hook-mode tests pass after inherited Git env sanitization.</x:v>
       </x:c>
       <x:c r="O29" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="P29" s="39" t="str"/>
-      <x:c r="Q29" s="39" t="str">
-        <x:v>Dependency</x:v>
-      </x:c>
-      <x:c r="R29" s="39" t="str">
-        <x:v>Requires provider adapter, permission degradation, and action audit.</x:v>
-      </x:c>
+      <x:c r="Q29" s="39" t="str"/>
+      <x:c r="R29" s="39" t="str"/>
       <x:c r="S29" s="39" t="str">
-        <x:v>Deferred with explicit unknown/unavailable semantics.</x:v>
+        <x:v>Yes: regression protects hook environment contamination; no destructive action test needed for absent commands.</x:v>
       </x:c>
       <x:c r="T29" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Safety gate is explicit and small; adding actions requires a separate preflight/audit phase.</x:v>
       </x:c>
       <x:c r="U29" s="39" t="str">
-        <x:v>PR work depends on provider state and cannot be safely inferred from local Git alone.</x:v>
+        <x:v>src-tauri/src/core.rs:251-297; /Users/jakyeamos/Downloads/pronto_prd.md:541-551, 1175-1183</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="X29" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
-      <x:c r="Y29" s="39" t="str">
-        <x:v>Add provider-backed evidence before adding any merge control.</x:v>
-      </x:c>
+        <x:v>Add action-tier audit tests only when modifying actions are authorized and implemented.</x:v>
+      </x:c>
+      <x:c r="Y29" s="39"/>
     </x:row>
     <x:row r="30" ht="70" customHeight="1">
       <x:c r="A30" s="51" t="str">
-        <x:v>REL-001</x:v>
+        <x:v>PROV-001</x:v>
       </x:c>
       <x:c r="B30" s="39" t="str">
-        <x:v>Releases</x:v>
+        <x:v>Provider</x:v>
       </x:c>
       <x:c r="C30" s="39" t="str">
-        <x:v>Release preparation</x:v>
+        <x:v>GitHub identities / refresh</x:v>
       </x:c>
       <x:c r="D30" s="39" t="str">
-        <x:v>As an operator, I can prepare a deterministic release draft without publishing it automatically.</x:v>
+        <x:v>As an operator, I can connect multiple identities and see permission degradation explicitly.</x:v>
       </x:c>
       <x:c r="E30" s="39" t="str">
-        <x:v>Release maintainer</x:v>
+        <x:v>Provider-connected operator</x:v>
       </x:c>
       <x:c r="F30" s="39" t="str">
         <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G30" s="39" t="str">
-        <x:v>Published release baseline, configured rule, clean isolated worktree</x:v>
+        <x:v>GitHub account and OS credential-store permissions</x:v>
       </x:c>
       <x:c r="H30" s="39" t="str">
         <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I30" s="39" t="str">
-        <x:v>Release baseline, deterministic rules, isolated worktrees, and draft handoff are deferred.</x:v>
+        <x:v>No provider adapter is enabled in this slice; the app does not claim GitHub identity, refresh, or permission results.</x:v>
       </x:c>
       <x:c r="J30" s="39" t="str">
-        <x:v>No release threshold or version recommendation appears until its configured evidence exists.</x:v>
+        <x:v>No provider state is shown as current until identity and permission evidence exist.</x:v>
       </x:c>
       <x:c r="K30" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>docs/implementation-plan.md:19-24; /Users/jakyeamos/Downloads/pronto_prd.md:296-306, 974-987</x:v>
       </x:c>
       <x:c r="L30" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M30" s="39" t="str">
-        <x:v>Deferred: provider, release recipe, and isolated worktree gates required</x:v>
+        <x:v>Deferred: requires explicit provider authority and credentials</x:v>
       </x:c>
       <x:c r="N30" s="39" t="str">
-        <x:v>No release preparation or publication path is implemented.</x:v>
+        <x:v>Provider identity, credential separation, and permission degradation are not implemented.</x:v>
       </x:c>
       <x:c r="O30" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -2976,72 +2976,72 @@
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R30" s="39" t="str">
-        <x:v>Requires exact diff review, validation gates, and publication boundary.</x:v>
+        <x:v>Requires network, provider auth, OS credential store, and a durable identity mapping.</x:v>
       </x:c>
       <x:c r="S30" s="39" t="str">
-        <x:v>Phase 3 plan preserves the no-publish rule.</x:v>
+        <x:v>Kept as an explicit deferred boundary; no fake adapter or mock provider result is added.</x:v>
       </x:c>
       <x:c r="T30" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U30" s="39" t="str">
-        <x:v>Release automation is intentionally not inferred from local commit counts.</x:v>
+        <x:v>Provider work is separated from local Git evidence by design.</x:v>
       </x:c>
       <x:c r="V30" s="39" t="str">
-        <x:v>pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>pronto_prd.md:296-306, 974-987; docs/implementation-plan.md:49-54</x:v>
       </x:c>
       <x:c r="W30" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X30" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y30" s="39" t="str">
-        <x:v>Define recipe state and audit events before implementation.</x:v>
+        <x:v>Define provider permission and freshness contracts before implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="70" customHeight="1">
       <x:c r="A31" s="51" t="str">
-        <x:v>PROC-001</x:v>
+        <x:v>REMOTE-001</x:v>
       </x:c>
       <x:c r="B31" s="39" t="str">
-        <x:v>Agent workspaces</x:v>
+        <x:v>Remote catalog</x:v>
       </x:c>
       <x:c r="C31" s="39" t="str">
-        <x:v>Process / terminal evidence</x:v>
+        <x:v>Remote-only / clone</x:v>
       </x:c>
       <x:c r="D31" s="39" t="str">
-        <x:v>As an operator, I can tell whether an agent workspace has process evidence without exposing terminal contents.</x:v>
+        <x:v>As an operator, I can import or clone a remote-only repository into a selected root.</x:v>
       </x:c>
       <x:c r="E31" s="39" t="str">
-        <x:v>Local operator</x:v>
+        <x:v>Provider-connected operator</x:v>
       </x:c>
       <x:c r="F31" s="39" t="str">
-        <x:v>Local permission required</x:v>
+        <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G31" s="39" t="str">
-        <x:v>OS process inspection permission and optional manifest</x:v>
+        <x:v>Remote repository catalog and clone permission</x:v>
       </x:c>
       <x:c r="H31" s="39" t="str">
-        <x:v>Desktop + native adapters</x:v>
+        <x:v>Desktop + network</x:v>
       </x:c>
       <x:c r="I31" s="39" t="str">
-        <x:v>Process, terminal, and generic agent adapters are deferred; no certainty is claimed from their absence.</x:v>
+        <x:v>Remote catalog and clone are not exposed by the local-first slice.</x:v>
       </x:c>
       <x:c r="J31" s="39" t="str">
-        <x:v>Unknown process evidence remains unknown rather than being classified as inactive or safe to clean.</x:v>
+        <x:v>A remote repository is not represented as local until clone succeeds and the local scan registers it.</x:v>
       </x:c>
       <x:c r="K31" s="39" t="str">
-        <x:v>docs/implementation-plan.md:51-54; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
+        <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:280-286, 849-857</x:v>
       </x:c>
       <x:c r="L31" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M31" s="39" t="str">
-        <x:v>Deferred: OS adapter and permission boundary required</x:v>
+        <x:v>Deferred: requires provider auth, network, clone preflight, and selected root</x:v>
       </x:c>
       <x:c r="N31" s="39" t="str">
-        <x:v>No process or terminal capture is implemented.</x:v>
+        <x:v>No remote-only or clone path is implemented.</x:v>
       </x:c>
       <x:c r="O31" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -3051,248 +3051,548 @@
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R31" s="39" t="str">
-        <x:v>Cross-platform process APIs and privacy review are required.</x:v>
+        <x:v>Requires network and exact destination authorization.</x:v>
       </x:c>
       <x:c r="S31" s="39" t="str">
-        <x:v>The current slice only models linked worktrees as local workspaces.</x:v>
+        <x:v>Deferred explicitly rather than pretending provider access exists.</x:v>
       </x:c>
       <x:c r="T31" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U31" s="39" t="str">
-        <x:v>Never capture terminal contents, prompts, source text, or keystrokes.</x:v>
+        <x:v>Clone is a modifying action and must arrive with fresh preflight/audit contracts.</x:v>
       </x:c>
       <x:c r="V31" s="39" t="str">
-        <x:v>pronto_prd.md:489-525</x:v>
+        <x:v>pronto_prd.md:280-286, 849-857</x:v>
       </x:c>
       <x:c r="W31" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X31" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y31" s="39" t="str">
-        <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
+        <x:v>Define clone destination and audit semantics before adding the action.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="70" customHeight="1">
       <x:c r="A32" s="51" t="str">
-        <x:v>GROUP-001</x:v>
+        <x:v>ACTION-001</x:v>
       </x:c>
       <x:c r="B32" s="39" t="str">
-        <x:v>Products</x:v>
+        <x:v>Safe actions</x:v>
       </x:c>
       <x:c r="C32" s="39" t="str">
-        <x:v>Products / groups</x:v>
+        <x:v>Preflight / audit</x:v>
       </x:c>
       <x:c r="D32" s="39" t="str">
-        <x:v>As an operator, I can aggregate multiple repositories without hiding repository-level evidence.</x:v>
+        <x:v>As an operator, I can see exact targets and fresh preflight evidence before a modifying action runs.</x:v>
       </x:c>
       <x:c r="E32" s="39" t="str">
-        <x:v>Portfolio operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F32" s="39" t="str">
         <x:v>Local-only or provider auth</x:v>
       </x:c>
       <x:c r="G32" s="39" t="str">
-        <x:v>Product/group configuration and participating repositories</x:v>
+        <x:v>A bounded modifying action is explicitly authorized</x:v>
       </x:c>
       <x:c r="H32" s="39" t="str">
-        <x:v>Desktop 1280×800</x:v>
+        <x:v>Desktop + native core</x:v>
       </x:c>
       <x:c r="I32" s="39" t="str">
-        <x:v>Products, groups, and coordinated release are deferred; the current portfolio remains repository-first.</x:v>
+        <x:v>The current slice exposes no modifying Git action, so preflight and audit are not falsely represented as complete.</x:v>
       </x:c>
       <x:c r="J32" s="39" t="str">
-        <x:v>No aggregate product status is shown until its repository-level provenance and release policy are defined.</x:v>
+        <x:v>No action is available without a fresh preflight, exact target, audit record, and post-action rescan.</x:v>
       </x:c>
       <x:c r="K32" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:529-551, 1173-1183</x:v>
       </x:c>
       <x:c r="L32" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M32" s="39" t="str">
-        <x:v>Deferred: product model and coordination policy required</x:v>
+        <x:v>Deferred until action policy is implemented</x:v>
       </x:c>
       <x:c r="N32" s="39" t="str">
-        <x:v>No product/group mutation or coordinated release logic is implemented.</x:v>
+        <x:v>No modifying action adapter exists in this implementation.</x:v>
       </x:c>
       <x:c r="O32" s="39" t="str">
-        <x:v>Needs-Product-Decision</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P32" s="39" t="str"/>
       <x:c r="Q32" s="39" t="str">
-        <x:v>Product</x:v>
+        <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R32" s="39" t="str">
-        <x:v>Requires decisions about composition, release modes, dependency order, and partial failure.</x:v>
+        <x:v>Requires action tiers, permission policy, audit schema, and failure semantics.</x:v>
       </x:c>
       <x:c r="S32" s="39" t="str">
-        <x:v>Repository-first UI avoids a premature aggregate abstraction.</x:v>
+        <x:v>Read-only slice keeps the action surface absent.</x:v>
       </x:c>
       <x:c r="T32" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U32" s="39" t="str">
-        <x:v>This is intentionally a product decision boundary, not an implementation defect.</x:v>
+        <x:v>Do not add action buttons before the preflight/audit contract is testable.</x:v>
       </x:c>
       <x:c r="V32" s="39" t="str">
-        <x:v>pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>pronto_prd.md:529-551</x:v>
       </x:c>
       <x:c r="W32" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X32" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y32" s="39" t="str">
-        <x:v>Confirm product/group semantics before Phase 3.</x:v>
+        <x:v>Phase 2 must add preflight tests before any modifying command.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="70" customHeight="1">
       <x:c r="A33" s="51" t="str">
-        <x:v>AI-001</x:v>
+        <x:v>PR-001</x:v>
       </x:c>
       <x:c r="B33" s="39" t="str">
-        <x:v>AI and privacy</x:v>
+        <x:v>Pull requests</x:v>
       </x:c>
       <x:c r="C33" s="39" t="str">
-        <x:v>Privacy boundary</x:v>
+        <x:v>Provider lifecycle</x:v>
       </x:c>
       <x:c r="D33" s="39" t="str">
-        <x:v>As an operator, I can keep AI disabled and prevent uncommitted source from leaving the machine.</x:v>
+        <x:v>As an operator, I can create or merge a PR only when provider facts and permissions are verifiable.</x:v>
       </x:c>
       <x:c r="E33" s="39" t="str">
-        <x:v>Privacy-conscious operator</x:v>
+        <x:v>Provider-connected operator</x:v>
       </x:c>
       <x:c r="F33" s="39" t="str">
-        <x:v>AI disabled by default</x:v>
+        <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G33" s="39" t="str">
-        <x:v>Explicit provider/model permission and approved payload</x:v>
+        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
       </x:c>
       <x:c r="H33" s="39" t="str">
-        <x:v>Desktop + provider/local model</x:v>
+        <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I33" s="39" t="str">
-        <x:v>No AI request path exists in this slice; local snapshots contain metadata and no uncommitted diff content.</x:v>
+        <x:v>PR creation, review evidence, and merge actions are explicit deferred boundaries.</x:v>
       </x:c>
       <x:c r="J33" s="39" t="str">
-        <x:v>No AI claim or payload is possible until the user opts in and reviews the exact payload categories.</x:v>
+        <x:v>Unknown checks or reviews never become a merge-eligible state.</x:v>
       </x:c>
       <x:c r="K33" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:32-188; src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
       </x:c>
       <x:c r="L33" s="39" t="str">
-        <x:v>Static safety review + privacy regression</x:v>
+        <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M33" s="39" t="str">
-        <x:v>rg 'diff|filename|content' src-tauri/src/core.rs src/renderer/src; cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+        <x:v>Deferred: provider permission and PR API required</x:v>
       </x:c>
       <x:c r="N33" s="39" t="str">
-        <x:v>No external AI call is implemented; snapshot privacy test passes and UI states the local/private boundary.</x:v>
+        <x:v>No PR lifecycle implementation is present.</x:v>
       </x:c>
       <x:c r="O33" s="39" t="str">
-        <x:v>Needs-Product-Decision</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P33" s="39" t="str"/>
       <x:c r="Q33" s="39" t="str">
-        <x:v>Product</x:v>
+        <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R33" s="39" t="str">
-        <x:v>AI payload categories, local endpoint, provider credentials, and traceability need explicit product decisions.</x:v>
+        <x:v>Requires provider adapter, permission degradation, and action audit.</x:v>
       </x:c>
       <x:c r="S33" s="39" t="str">
-        <x:v>Deferred AI authority; local metadata-only evidence remains available.</x:v>
+        <x:v>Deferred with explicit unknown/unavailable semantics.</x:v>
       </x:c>
       <x:c r="T33" s="39" t="str">
-        <x:v>Yes: snapshot excludes source/diff content.</x:v>
+        <x:v>No.</x:v>
       </x:c>
       <x:c r="U33" s="39" t="str">
-        <x:v>AI is not introduced as a shortcut for missing provider evidence.</x:v>
+        <x:v>PR work depends on provider state and cannot be safely inferred from local Git alone.</x:v>
       </x:c>
       <x:c r="V33" s="39" t="str">
-        <x:v>pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>pronto_prd.md:555-571, 1185-1189</x:v>
       </x:c>
       <x:c r="W33" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X33" s="39" t="str">
-        <x:v>73c28e5</x:v>
+        <x:v>885fe1e</x:v>
       </x:c>
       <x:c r="Y33" s="39" t="str">
-        <x:v>Define per-repository permissions and payload preview before any provider call.</x:v>
+        <x:v>Add provider-backed evidence before adding any merge control.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="70" customHeight="1">
       <x:c r="A34" s="51" t="str">
+        <x:v>REL-001</x:v>
+      </x:c>
+      <x:c r="B34" s="39" t="str">
+        <x:v>Releases</x:v>
+      </x:c>
+      <x:c r="C34" s="39" t="str">
+        <x:v>Release preparation</x:v>
+      </x:c>
+      <x:c r="D34" s="39" t="str">
+        <x:v>As an operator, I can prepare a deterministic release draft without publishing it automatically.</x:v>
+      </x:c>
+      <x:c r="E34" s="39" t="str">
+        <x:v>Release maintainer</x:v>
+      </x:c>
+      <x:c r="F34" s="39" t="str">
+        <x:v>Provider auth required</x:v>
+      </x:c>
+      <x:c r="G34" s="39" t="str">
+        <x:v>Published release baseline, configured rule, clean isolated worktree</x:v>
+      </x:c>
+      <x:c r="H34" s="39" t="str">
+        <x:v>Desktop + provider API</x:v>
+      </x:c>
+      <x:c r="I34" s="39" t="str">
+        <x:v>Release baseline, deterministic rules, isolated worktrees, and draft handoff are deferred.</x:v>
+      </x:c>
+      <x:c r="J34" s="39" t="str">
+        <x:v>No release threshold or version recommendation appears until its configured evidence exists.</x:v>
+      </x:c>
+      <x:c r="K34" s="39" t="str">
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
+      </x:c>
+      <x:c r="L34" s="39" t="str">
+        <x:v>Boundary review</x:v>
+      </x:c>
+      <x:c r="M34" s="39" t="str">
+        <x:v>Deferred: provider, release recipe, and isolated worktree gates required</x:v>
+      </x:c>
+      <x:c r="N34" s="39" t="str">
+        <x:v>No release preparation or publication path is implemented.</x:v>
+      </x:c>
+      <x:c r="O34" s="39" t="str">
+        <x:v>Needs-Environment</x:v>
+      </x:c>
+      <x:c r="P34" s="39" t="str"/>
+      <x:c r="Q34" s="39" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="R34" s="39" t="str">
+        <x:v>Requires exact diff review, validation gates, and publication boundary.</x:v>
+      </x:c>
+      <x:c r="S34" s="39" t="str">
+        <x:v>Phase 3 plan preserves the no-publish rule.</x:v>
+      </x:c>
+      <x:c r="T34" s="39" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="U34" s="39" t="str">
+        <x:v>Release automation is intentionally not inferred from local commit counts.</x:v>
+      </x:c>
+      <x:c r="V34" s="39" t="str">
+        <x:v>pronto_prd.md:575-655, 1191-1203</x:v>
+      </x:c>
+      <x:c r="W34" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X34" s="39" t="str">
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y34" s="39" t="str">
+        <x:v>Define recipe state and audit events before implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="70" customHeight="1">
+      <x:c r="A35" s="51" t="str">
+        <x:v>PROC-001</x:v>
+      </x:c>
+      <x:c r="B35" s="39" t="str">
+        <x:v>Agent workspaces</x:v>
+      </x:c>
+      <x:c r="C35" s="39" t="str">
+        <x:v>Process / terminal evidence</x:v>
+      </x:c>
+      <x:c r="D35" s="39" t="str">
+        <x:v>As an operator, I can tell whether an agent workspace has process evidence without exposing terminal contents.</x:v>
+      </x:c>
+      <x:c r="E35" s="39" t="str">
+        <x:v>Local operator</x:v>
+      </x:c>
+      <x:c r="F35" s="39" t="str">
+        <x:v>Local permission required</x:v>
+      </x:c>
+      <x:c r="G35" s="39" t="str">
+        <x:v>OS process inspection permission and optional manifest</x:v>
+      </x:c>
+      <x:c r="H35" s="39" t="str">
+        <x:v>Desktop + native adapters</x:v>
+      </x:c>
+      <x:c r="I35" s="39" t="str">
+        <x:v>Process, terminal, and generic agent adapters are deferred; no certainty is claimed from their absence.</x:v>
+      </x:c>
+      <x:c r="J35" s="39" t="str">
+        <x:v>Unknown process evidence remains unknown rather than being classified as inactive or safe to clean.</x:v>
+      </x:c>
+      <x:c r="K35" s="39" t="str">
+        <x:v>docs/implementation-plan.md:51-54; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
+      </x:c>
+      <x:c r="L35" s="39" t="str">
+        <x:v>Boundary review</x:v>
+      </x:c>
+      <x:c r="M35" s="39" t="str">
+        <x:v>Deferred: OS adapter and permission boundary required</x:v>
+      </x:c>
+      <x:c r="N35" s="39" t="str">
+        <x:v>No process or terminal capture is implemented.</x:v>
+      </x:c>
+      <x:c r="O35" s="39" t="str">
+        <x:v>Needs-Environment</x:v>
+      </x:c>
+      <x:c r="P35" s="39" t="str"/>
+      <x:c r="Q35" s="39" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="R35" s="39" t="str">
+        <x:v>Cross-platform process APIs and privacy review are required.</x:v>
+      </x:c>
+      <x:c r="S35" s="39" t="str">
+        <x:v>The current slice only models linked worktrees as local workspaces.</x:v>
+      </x:c>
+      <x:c r="T35" s="39" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="U35" s="39" t="str">
+        <x:v>Never capture terminal contents, prompts, source text, or keystrokes.</x:v>
+      </x:c>
+      <x:c r="V35" s="39" t="str">
+        <x:v>pronto_prd.md:489-525</x:v>
+      </x:c>
+      <x:c r="W35" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X35" s="39" t="str">
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y35" s="39" t="str">
+        <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="70" customHeight="1">
+      <x:c r="A36" s="51" t="str">
+        <x:v>GROUP-001</x:v>
+      </x:c>
+      <x:c r="B36" s="39" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="C36" s="39" t="str">
+        <x:v>Products / groups</x:v>
+      </x:c>
+      <x:c r="D36" s="39" t="str">
+        <x:v>As an operator, I can aggregate multiple repositories without hiding repository-level evidence.</x:v>
+      </x:c>
+      <x:c r="E36" s="39" t="str">
+        <x:v>Portfolio operator</x:v>
+      </x:c>
+      <x:c r="F36" s="39" t="str">
+        <x:v>Local-only or provider auth</x:v>
+      </x:c>
+      <x:c r="G36" s="39" t="str">
+        <x:v>Product/group configuration and participating repositories</x:v>
+      </x:c>
+      <x:c r="H36" s="39" t="str">
+        <x:v>Desktop 1280×800</x:v>
+      </x:c>
+      <x:c r="I36" s="39" t="str">
+        <x:v>Products, groups, and coordinated release are deferred; the current portfolio remains repository-first.</x:v>
+      </x:c>
+      <x:c r="J36" s="39" t="str">
+        <x:v>No aggregate product status is shown until its repository-level provenance and release policy are defined.</x:v>
+      </x:c>
+      <x:c r="K36" s="39" t="str">
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
+      </x:c>
+      <x:c r="L36" s="39" t="str">
+        <x:v>Boundary review</x:v>
+      </x:c>
+      <x:c r="M36" s="39" t="str">
+        <x:v>Deferred: product model and coordination policy required</x:v>
+      </x:c>
+      <x:c r="N36" s="39" t="str">
+        <x:v>No product/group mutation or coordinated release logic is implemented.</x:v>
+      </x:c>
+      <x:c r="O36" s="39" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="P36" s="39" t="str"/>
+      <x:c r="Q36" s="39" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="R36" s="39" t="str">
+        <x:v>Manual product/group configuration is accepted; implementation still needs the durable state and coordination model.</x:v>
+      </x:c>
+      <x:c r="S36" s="39" t="str">
+        <x:v>Repository-first UI avoids a premature inferred aggregate abstraction.</x:v>
+      </x:c>
+      <x:c r="T36" s="39" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="U36" s="39" t="str">
+        <x:v>This is an accepted delivery boundary, not an unresolved product decision.</x:v>
+      </x:c>
+      <x:c r="V36" s="39" t="str">
+        <x:v>pronto_prd.md:227-238, 659-677</x:v>
+      </x:c>
+      <x:c r="W36" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X36" s="39" t="str">
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y36" s="39" t="str">
+        <x:v>Implement manual product/group configuration after the SQLite contract is stable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="70" customHeight="1">
+      <x:c r="A37" s="51" t="str">
+        <x:v>AI-001</x:v>
+      </x:c>
+      <x:c r="B37" s="39" t="str">
+        <x:v>AI and privacy</x:v>
+      </x:c>
+      <x:c r="C37" s="39" t="str">
+        <x:v>Privacy boundary</x:v>
+      </x:c>
+      <x:c r="D37" s="39" t="str">
+        <x:v>As an operator, I can keep AI disabled and prevent uncommitted source from leaving the machine.</x:v>
+      </x:c>
+      <x:c r="E37" s="39" t="str">
+        <x:v>Privacy-conscious operator</x:v>
+      </x:c>
+      <x:c r="F37" s="39" t="str">
+        <x:v>AI disabled by default</x:v>
+      </x:c>
+      <x:c r="G37" s="39" t="str">
+        <x:v>Explicit provider/model permission and approved payload</x:v>
+      </x:c>
+      <x:c r="H37" s="39" t="str">
+        <x:v>Desktop + provider/local model</x:v>
+      </x:c>
+      <x:c r="I37" s="39" t="str">
+        <x:v>No AI request path exists in this slice; local snapshots contain metadata and no uncommitted diff content.</x:v>
+      </x:c>
+      <x:c r="J37" s="39" t="str">
+        <x:v>No AI claim or payload is possible until the user opts in and reviews the exact payload categories.</x:v>
+      </x:c>
+      <x:c r="K37" s="39" t="str">
+        <x:v>src-tauri/src/core.rs:32-188; src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
+      </x:c>
+      <x:c r="L37" s="39" t="str">
+        <x:v>Static safety review + privacy regression</x:v>
+      </x:c>
+      <x:c r="M37" s="39" t="str">
+        <x:v>rg 'diff|filename|content' src-tauri/src/core.rs src/renderer/src; cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+      </x:c>
+      <x:c r="N37" s="39" t="str">
+        <x:v>No external AI call is implemented; snapshot privacy test passes and UI states the local/private boundary.</x:v>
+      </x:c>
+      <x:c r="O37" s="39" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="P37" s="39" t="str"/>
+      <x:c r="Q37" s="39" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="R37" s="39" t="str">
+        <x:v>AI remains disabled by the accepted product direction; payload categories and provider permissions are outside this slice.</x:v>
+      </x:c>
+      <x:c r="S37" s="39" t="str">
+        <x:v>Deferred AI authority; local metadata-only evidence remains available.</x:v>
+      </x:c>
+      <x:c r="T37" s="39" t="str">
+        <x:v>Yes: snapshot excludes source/diff content.</x:v>
+      </x:c>
+      <x:c r="U37" s="39" t="str">
+        <x:v>AI is not introduced as a shortcut for missing provider evidence.</x:v>
+      </x:c>
+      <x:c r="V37" s="39" t="str">
+        <x:v>pronto_prd.md:679-695, 1205-1211</x:v>
+      </x:c>
+      <x:c r="W37" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X37" s="39" t="str">
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="Y37" s="39" t="str">
+        <x:v>Keep AI disabled until per-repository permissions and payload preview are explicitly designed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="70" customHeight="1">
+      <x:c r="A38" s="51" t="str">
         <x:v>HIST-001</x:v>
       </x:c>
-      <x:c r="B34" s="39" t="str">
+      <x:c r="B38" s="39" t="str">
         <x:v>History</x:v>
       </x:c>
-      <x:c r="C34" s="39" t="str">
+      <x:c r="C38" s="39" t="str">
         <x:v>Event retention</x:v>
       </x:c>
-      <x:c r="D34" s="39" t="str">
+      <x:c r="D38" s="39" t="str">
         <x:v>As an operator, I can retain bounded transition history without losing current state.</x:v>
       </x:c>
-      <x:c r="E34" s="39" t="str">
+      <x:c r="E38" s="39" t="str">
         <x:v>Local operator</x:v>
       </x:c>
-      <x:c r="F34" s="39" t="str">
+      <x:c r="F38" s="39" t="str">
         <x:v>Local-only</x:v>
       </x:c>
-      <x:c r="G34" s="39" t="str">
+      <x:c r="G38" s="39" t="str">
         <x:v>Transition events persisted in local store</x:v>
       </x:c>
-      <x:c r="H34" s="39" t="str">
+      <x:c r="H38" s="39" t="str">
         <x:v>Native core</x:v>
       </x:c>
-      <x:c r="I34" s="39" t="str">
+      <x:c r="I38" s="39" t="str">
         <x:v>Events are transition-only, retained for a default bounded window, and pruned independently of current snapshots.</x:v>
       </x:c>
-      <x:c r="J34" s="39" t="str">
+      <x:c r="J38" s="39" t="str">
         <x:v>History is useful without growing indefinitely or becoming a source-content archive.</x:v>
       </x:c>
-      <x:c r="K34" s="39" t="str">
+      <x:c r="K38" s="39" t="str">
         <x:v>src-tauri/src/core.rs:110-149, 1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
       </x:c>
-      <x:c r="L34" s="39" t="str">
+      <x:c r="L38" s="39" t="str">
         <x:v>Rust repeated-scan regression + source review</x:v>
       </x:c>
-      <x:c r="M34" s="39" t="str">
+      <x:c r="M38" s="39" t="str">
         <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
       </x:c>
-      <x:c r="N34" s="39" t="str">
+      <x:c r="N38" s="39" t="str">
         <x:v>Transition persistence passes; the 90-day default and configurable retention are represented in the core constants/logic for this slice.</x:v>
       </x:c>
-      <x:c r="O34" s="39" t="str">
+      <x:c r="O38" s="39" t="str">
         <x:v>Regression-Covered</x:v>
       </x:c>
-      <x:c r="P34" s="39" t="str"/>
-      <x:c r="Q34" s="39" t="str"/>
-      <x:c r="R34" s="39" t="str"/>
-      <x:c r="S34" s="39" t="str">
+      <x:c r="P38" s="39" t="str"/>
+      <x:c r="Q38" s="39" t="str"/>
+      <x:c r="R38" s="39" t="str"/>
+      <x:c r="S38" s="39" t="str">
         <x:v>Yes: repeated-scan event regression.</x:v>
       </x:c>
-      <x:c r="T34" s="39" t="str">
+      <x:c r="T38" s="39" t="str">
         <x:v>Bounded event history is a small persistence concern; durable configuration remains Phase 2.</x:v>
       </x:c>
-      <x:c r="U34" s="39" t="str">
+      <x:c r="U38" s="39" t="str">
         <x:v>src-tauri/src/core.rs:1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
       </x:c>
-      <x:c r="V34" s="39" t="str">
+      <x:c r="V38" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W34" s="39" t="str">
-        <x:v>73c28e5</x:v>
-      </x:c>
-      <x:c r="X34" s="39" t="str">
+      <x:c r="W38" s="39" t="str">
+        <x:v>885fe1e</x:v>
+      </x:c>
+      <x:c r="X38" s="39" t="str">
         <x:v>Expose retention settings and add date-boundary tests.</x:v>
       </x:c>
-      <x:c r="Y34" s="39"/>
+      <x:c r="Y38" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3300,7 +3600,7 @@
     <x:mergeCell ref="A2:Y2"/>
     <x:mergeCell ref="A3:Y3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="O5:O34">
+  <x:conditionalFormatting sqref="O5:O38">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Regression-Covered"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Verified"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Build verified"/>
@@ -3310,13 +3610,13 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="O5:O34">
+    <x:dataValidation type="list" sqref="O5:O38">
       <x:formula1>"Regression-Covered,Verified,Needs-Environment,Needs-Product-Decision,Deferred"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R625301352f4240fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e30cca6ebe849e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3441,13 +3741,13 @@
         <x:v>FR-027–031</x:v>
       </x:c>
       <x:c r="C8" s="39" t="str">
-        <x:v>UI-001</x:v>
+        <x:v>UI-001; UI-004–007</x:v>
       </x:c>
       <x:c r="D8" s="39" t="str">
         <x:v>Environment</x:v>
       </x:c>
       <x:c r="E8" s="39" t="str">
-        <x:v>Portfolio-first renderer exists with filters and local layout; live Tauri interaction remains to be verified.</x:v>
+        <x:v>Portfolio-first renderer now includes truthful navigation, freshness, keyboard access, settings/activity surfaces, filters, and local empty states; live Tauri interaction remains to be verified.</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
         <x:v>Phase 1 desktop verification</x:v>
@@ -3461,13 +3761,13 @@
         <x:v>FR-032–039; AC-008–010</x:v>
       </x:c>
       <x:c r="C9" s="39" t="str">
-        <x:v>COND-001–002; UI-002</x:v>
+        <x:v>COND-001–002; UI-002; UI-007</x:v>
       </x:c>
       <x:c r="D9" s="39" t="str">
         <x:v>Partial / environment</x:v>
       </x:c>
       <x:c r="E9" s="39" t="str">
-        <x:v>Deterministic grouped queue, evidence drawer, expected fingerprints, and empty states exist; live interaction still needs a desktop pass.</x:v>
+        <x:v>Deterministic grouped queue, evidence drawer, expected fingerprints, and distinct no-data/no-match states exist; live interaction still needs a desktop pass.</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>Phase 1 desktop verification</x:v>
@@ -3584,13 +3884,13 @@
         <x:v>GROUP-001</x:v>
       </x:c>
       <x:c r="D15" s="39" t="str">
-        <x:v>Product decision</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E15" s="39" t="str">
-        <x:v>Aggregation and coordinated release need product decisions before implementation.</x:v>
+        <x:v>Manual product/group configuration is the accepted direction; aggregation and coordinated release remain deferred until the durable state model is implemented.</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>Phase 3 decision gate</x:v>
+        <x:v>Phase 2 design gate</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
@@ -3607,7 +3907,7 @@
         <x:v>Privacy boundary</x:v>
       </x:c>
       <x:c r="E16" s="39" t="str">
-        <x:v>AI is absent/disabled by default; local snapshots avoid filenames and diff content. Provider payload preview and per-repository permission remain deferred.</x:v>
+        <x:v>AI is disabled by default; local snapshots avoid filenames and diff content. Provider payload preview and per-repository permission remain intentionally absent.</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
         <x:v>Phase 2 decision gate</x:v>
@@ -3621,13 +3921,13 @@
         <x:v>FR-109–112; AC-031–032</x:v>
       </x:c>
       <x:c r="C17" s="39" t="str">
-        <x:v>AUD-001; HIST-001</x:v>
+        <x:v>AUD-001; HIST-001; UI-006</x:v>
       </x:c>
       <x:c r="D17" s="39" t="str">
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E17" s="39" t="str">
-        <x:v>Transition-only metadata history and bounded pruning are implemented; configurable retention and durable database migration remain deferred.</x:v>
+        <x:v>Transition-only metadata history and bounded pruning are implemented and surfaced in Activity; configurable retention and durable database migration remain deferred.</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
         <x:v>Phase 2</x:v>
@@ -3694,7 +3994,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R573969b18903461b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5966e3c4e65245cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3735,7 +4035,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Implementation commit: 73c28e5 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
+        <x:v>Implementation commit: 885fe1e | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -3777,33 +4077,33 @@
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="61" t="n">
-        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$34)</x:f>
-        <x:v>30</x:v>
+        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$38)</x:f>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B5" s="62"/>
       <x:c r="C5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$34,"Regression-Covered")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Regression-Covered")</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="62"/>
       <x:c r="E5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$34,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$34,"Build verified")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$38,"Build verified")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F5" s="62"/>
       <x:c r="G5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$34,"Needs-Environment")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Needs-Environment")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H5" s="62"/>
       <x:c r="I5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$34,"Needs-Product-Decision")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Needs-Product-Decision")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J5" s="62"/>
       <x:c r="K5" s="63" t="n">
         <x:f>(C5+E5+G5)/(A5)</x:f>
-        <x:v>0.9333333333333333</x:v>
+        <x:v>0.9411764705882353</x:v>
       </x:c>
       <x:c r="L5" s="64"/>
     </x:row>
@@ -3845,16 +4145,16 @@
         <x:v>Local evidence foundation</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:v>Discovery, structured Git facts, explainable conditions, expected fingerprints, transition history, portfolio UI, read-only CLI</x:v>
+        <x:v>Discovery, structured Git facts, explainable conditions, expected fingerprints, transition history, portfolio UI, truthful local navigation, read-only CLI</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
-        <x:v>cargo test; typecheck; lint; build; CLI smoke; Pre-CR</x:v>
+        <x:v>cargo test; typecheck; lint; build:web; CLI smoke; Pre-CR</x:v>
       </x:c>
       <x:c r="E10" s="36" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F10" s="37" t="str">
-        <x:v>Current implementation commit is 1817527; workbook review is this iteration.</x:v>
+        <x:v>Local UX slice is implemented at 885fe1e; workbook review is this iteration.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -3865,16 +4165,16 @@
         <x:v>Provider and durable state expansion</x:v>
       </x:c>
       <x:c r="C11" s="39" t="str">
-        <x:v>SQLite contract, GitHub identities, fetch/refresh freshness, remote catalog/clone, process adapters, action preflight/audit</x:v>
+        <x:v>Versioned SQLite contract, GitHub identities, fetch/refresh freshness, remote catalog/clone, process adapters, action preflight/audit</x:v>
       </x:c>
       <x:c r="D11" s="39" t="str">
-        <x:v>Provider permission and persistence design review</x:v>
+        <x:v>SQLite migration and provider permission design review</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>Requires explicit auth, destination, and action authority.</x:v>
+        <x:v>SQLite comes before provider data; read-only GitHub and safe local actions follow explicit contracts.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -4014,7 +4314,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>Vite production bundle emitted</x:v>
+        <x:v>Vite production bundle emitted after the local UX slice</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
@@ -4077,7 +4377,7 @@
     </x:row>
     <x:row r="31" ht="26" customHeight="1">
       <x:c r="A31" s="8" t="str">
-        <x:v>The implementation is intentionally a local-first vertical slice. The main residual risk is not missing code breadth; it is unverified live desktop/provider behavior. The next safe expansion is a provider/durable-state contract with explicit permissions, freshness, and action preflight before adding remote or modifying operations.</x:v>
+        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX slice is implemented; the next safe expansion is versioned SQLite while preserving renderer and CLI snapshot contracts, followed by action preflight/audit and then provider context.</x:v>
       </x:c>
       <x:c r="B31" s="8"/>
       <x:c r="C31" s="8"/>

</xml_diff>

<commit_message>
docs: refresh behavior spec for sqlite
</commit_message>
<xml_diff>
--- a/docs/pronto-behavior-spec.xlsx
+++ b/docs/pronto-behavior-spec.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="Rb3bfd871e85a44ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R3eedf34938664f4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="Rc4858afe2273403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R9a0984223ffb4a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R60852c5a949448e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R5846143b9ab14ee0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1019,7 +1019,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot 885fe1e</x:v>
+        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot d332573</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1221,7 +1221,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X5" s="36" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y5" s="36" t="str">
         <x:v>Verify macOS, Windows, and Linux folder permissions when the desktop shell is launched.</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X6" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y6" s="39" t="str">
         <x:v>Add configurable glob-pattern coverage in the provider/durable-state phase.</x:v>
@@ -1358,7 +1358,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X7" s="39" t="str">
         <x:v>Submodule promotion and symlink-root matrix remain for the discovery expansion.</x:v>
@@ -1427,7 +1427,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W8" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X8" s="39" t="str">
         <x:v>Provider and AI payload previews still need their own explicit contract.</x:v>
@@ -1496,7 +1496,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W9" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X9" s="39" t="str">
         <x:v>Add fetched-at evidence after fetch/provider refresh exists.</x:v>
@@ -1565,7 +1565,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W10" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X10" s="39" t="str">
         <x:v>Add staged + unstaged + untracked matrix cases as scan coverage grows.</x:v>
@@ -1634,7 +1634,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W11" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X11" s="39" t="str">
         <x:v>Add a fixture for unreadable paths on each supported OS.</x:v>
@@ -1703,7 +1703,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W12" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X12" s="39" t="str">
         <x:v>Add rebase/cherry-pick/revert/bisect fixtures before action work begins.</x:v>
@@ -1772,7 +1772,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W13" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X13" s="39" t="str">
         <x:v>Add dedicated integration-state fixture matrix and user correction persistence.</x:v>
@@ -1841,7 +1841,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W14" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X14" s="39" t="str">
         <x:v>Implement fetch freshness and policy controls in Phase 2.</x:v>
@@ -1910,7 +1910,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X15" s="39" t="str">
         <x:v>Add provider-backed conditions only after permission/freshness contracts exist.</x:v>
@@ -1979,7 +1979,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W16" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X16" s="39" t="str">
         <x:v>Add UI interaction verification once the Tauri shell is launched.</x:v>
@@ -2048,7 +2048,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W17" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X17" s="39" t="str">
         <x:v>Expose retention configuration and current-state independence in Phase 2.</x:v>
@@ -2063,7 +2063,7 @@
         <x:v>Persistence</x:v>
       </x:c>
       <x:c r="C18" s="39" t="str">
-        <x:v>Local registry</x:v>
+        <x:v>Versioned SQLite registry</x:v>
       </x:c>
       <x:c r="D18" s="39" t="str">
         <x:v>As an operator, I can close and reopen Pronto without losing registered roots or current snapshots.</x:v>
@@ -2081,13 +2081,13 @@
         <x:v>Native core</x:v>
       </x:c>
       <x:c r="I18" s="39" t="str">
-        <x:v>Registry state is loaded from the platform data directory and saved through a temporary file rename.</x:v>
+        <x:v>Registry state is loaded from a versioned SQLite database under the platform data directory and saved in transactions; a legacy JSON registry is imported non-destructively when present.</x:v>
       </x:c>
       <x:c r="J18" s="39" t="str">
         <x:v>Persistence is local and recoverable without a server account.</x:v>
       </x:c>
       <x:c r="K18" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:193-249, 1322-1358; /Users/jakyeamos/Downloads/pronto_prd.md:926-954</x:v>
+        <x:v>src-tauri/src/core.rs:214-545, 1621-1655, 2006-2090; /Users/jakyeamos/Downloads/pronto_prd.md:926-954</x:v>
       </x:c>
       <x:c r="L18" s="39" t="str">
         <x:v>Rust persistence regression + source review</x:v>
@@ -2096,7 +2096,7 @@
         <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
       </x:c>
       <x:c r="N18" s="39" t="str">
-        <x:v>Persistence fixture reads the stored state after scan and confirms transition history survives.</x:v>
+        <x:v>Six Rust tests cover transactional persistence, transition history, schema metadata, and legacy JSON migration.</x:v>
       </x:c>
       <x:c r="O18" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -2105,22 +2105,22 @@
       <x:c r="Q18" s="39" t="str"/>
       <x:c r="R18" s="39" t="str"/>
       <x:c r="S18" s="39" t="str">
-        <x:v>Yes: JSON store persistence test.</x:v>
+        <x:v>Yes: SQLite persistence and legacy migration tests.</x:v>
       </x:c>
       <x:c r="T18" s="39" t="str">
-        <x:v>Atomic JSON is intentionally a Phase 1 foundation; SQLite migration is planned before multi-provider state.</x:v>
+        <x:v>The schema is versioned, uses separate roots/repositories/expected/events tables, and keeps complex snapshot payloads behind the existing Rust contract.</x:v>
       </x:c>
       <x:c r="U18" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:217-239; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
+        <x:v>src-tauri/src/core.rs:242-545, 2006-2090; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
       </x:c>
       <x:c r="V18" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W18" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X18" s="39" t="str">
-        <x:v>Verify crash recovery and migrate to SQLite when durable state expands.</x:v>
+        <x:v>Add explicit schema migration steps before introducing schema version 2 and verify crash recovery on the target desktop runtime.</x:v>
       </x:c>
       <x:c r="Y18" s="39"/>
     </x:row>
@@ -2193,7 +2193,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X19" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y19" s="39" t="str">
         <x:v>Run a human visual pass in the Tauri window and record screenshots/interaction outcomes.</x:v>
@@ -2268,7 +2268,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X20" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y20" s="39" t="str">
         <x:v>Verify evidence drawer content, expected-state action, and close behavior manually.</x:v>
@@ -2343,7 +2343,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X21" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y21" s="39" t="str">
         <x:v>Provider install/auth and refresh evidence are Phase 2 work.</x:v>
@@ -2418,7 +2418,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X22" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y22" s="39" t="str">
         <x:v>Verify active navigation, deferred copy, and Activity/Settings content manually.</x:v>
@@ -2493,7 +2493,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X23" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y23" s="39" t="str">
         <x:v>Verify search focus, Escape dismissal, and focus behavior manually.</x:v>
@@ -2568,7 +2568,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X24" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y24" s="39" t="str">
         <x:v>Verify roots, storage path, freshness, privacy, event rows, and empty state manually.</x:v>
@@ -2643,7 +2643,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X25" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y25" s="39" t="str">
         <x:v>Verify no-data, no-match, and Clear filters states manually.</x:v>
@@ -2711,7 +2711,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W26" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X26" s="39" t="str">
         <x:v>Implement desktop focus behavior for `pronto .` when the app lifecycle is available.</x:v>
@@ -2780,7 +2780,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X27" s="39" t="str">
         <x:v>Package installation and `pronto .` focus behavior remain to be verified.</x:v>
@@ -2849,7 +2849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W28" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X28" s="39" t="str">
         <x:v>Code signing/notarization is outside this local implementation.</x:v>
@@ -2918,7 +2918,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X29" s="39" t="str">
         <x:v>Add action-tier audit tests only when modifying actions are authorized and implemented.</x:v>
@@ -2994,7 +2994,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X30" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y30" s="39" t="str">
         <x:v>Define provider permission and freshness contracts before implementation.</x:v>
@@ -3069,7 +3069,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X31" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y31" s="39" t="str">
         <x:v>Define clone destination and audit semantics before adding the action.</x:v>
@@ -3144,7 +3144,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X32" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y32" s="39" t="str">
         <x:v>Phase 2 must add preflight tests before any modifying command.</x:v>
@@ -3219,7 +3219,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X33" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y33" s="39" t="str">
         <x:v>Add provider-backed evidence before adding any merge control.</x:v>
@@ -3294,7 +3294,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X34" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y34" s="39" t="str">
         <x:v>Define recipe state and audit events before implementation.</x:v>
@@ -3369,7 +3369,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X35" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y35" s="39" t="str">
         <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
@@ -3444,7 +3444,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X36" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y36" s="39" t="str">
         <x:v>Implement manual product/group configuration after the SQLite contract is stable.</x:v>
@@ -3519,7 +3519,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X37" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="Y37" s="39" t="str">
         <x:v>Keep AI disabled until per-repository permissions and payload preview are explicitly designed.</x:v>
@@ -3587,7 +3587,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W38" s="39" t="str">
-        <x:v>885fe1e</x:v>
+        <x:v>d332573</x:v>
       </x:c>
       <x:c r="X38" s="39" t="str">
         <x:v>Expose retention settings and add date-boundary tests.</x:v>
@@ -3616,7 +3616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e30cca6ebe849e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c7dcdb113f467a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3927,7 +3927,7 @@
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E17" s="39" t="str">
-        <x:v>Transition-only metadata history and bounded pruning are implemented and surfaced in Activity; configurable retention and durable database migration remain deferred.</x:v>
+        <x:v>Transition-only metadata history and bounded pruning are implemented and surfaced in Activity; configurable retention and future schema migrations remain deferred.</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
         <x:v>Phase 2</x:v>
@@ -3994,7 +3994,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5966e3c4e65245cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff6a473fff6b4fa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4035,7 +4035,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Implementation commit: 885fe1e | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
+        <x:v>Implementation commit: d332573 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -4162,19 +4162,19 @@
         <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="B11" s="39" t="str">
-        <x:v>Provider and durable state expansion</x:v>
+        <x:v>Provider and safe action expansion</x:v>
       </x:c>
       <x:c r="C11" s="39" t="str">
-        <x:v>Versioned SQLite contract, GitHub identities, fetch/refresh freshness, remote catalog/clone, process adapters, action preflight/audit</x:v>
+        <x:v>GitHub identities, fetch/refresh freshness, remote catalog/clone, process adapters, action preflight/audit</x:v>
       </x:c>
       <x:c r="D11" s="39" t="str">
-        <x:v>SQLite migration and provider permission design review</x:v>
+        <x:v>Provider permission and action audit design review</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>SQLite comes before provider data; read-only GitHub and safe local actions follow explicit contracts.</x:v>
+        <x:v>Versioned SQLite is complete; read-only GitHub and safe local actions follow explicit contracts.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -4272,7 +4272,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D21" s="40" t="str">
-        <x:v>5 Rust tests; Vitest no test files</x:v>
+        <x:v>6 Rust tests; Vitest no test files</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
@@ -4377,7 +4377,7 @@
     </x:row>
     <x:row r="31" ht="26" customHeight="1">
       <x:c r="A31" s="8" t="str">
-        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX slice is implemented; the next safe expansion is versioned SQLite while preserving renderer and CLI snapshot contracts, followed by action preflight/audit and then provider context.</x:v>
+        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX and durable-state slices are implemented; the next safe expansion is action preflight/audit, followed by read-only provider context.</x:v>
       </x:c>
       <x:c r="B31" s="8"/>
       <x:c r="C31" s="8"/>

</xml_diff>

<commit_message>
docs: refresh action behavior coverage
</commit_message>
<xml_diff>
--- a/docs/pronto-behavior-spec.xlsx
+++ b/docs/pronto-behavior-spec.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R9a0984223ffb4a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R60852c5a949448e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R5846143b9ab14ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R3059b3698dac4cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R5a543ef32eba4011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R9b1ed6bb24504c9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -720,7 +720,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="Feature ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1019,7 +1019,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot d332573</x:v>
+        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot b13de08</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1221,7 +1221,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X5" s="36" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y5" s="36" t="str">
         <x:v>Verify macOS, Windows, and Linux folder permissions when the desktop shell is launched.</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X6" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y6" s="39" t="str">
         <x:v>Add configurable glob-pattern coverage in the provider/durable-state phase.</x:v>
@@ -1358,7 +1358,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X7" s="39" t="str">
         <x:v>Submodule promotion and symlink-root matrix remain for the discovery expansion.</x:v>
@@ -1427,7 +1427,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W8" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X8" s="39" t="str">
         <x:v>Provider and AI payload previews still need their own explicit contract.</x:v>
@@ -1496,7 +1496,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W9" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X9" s="39" t="str">
         <x:v>Add fetched-at evidence after fetch/provider refresh exists.</x:v>
@@ -1565,7 +1565,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W10" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X10" s="39" t="str">
         <x:v>Add staged + unstaged + untracked matrix cases as scan coverage grows.</x:v>
@@ -1634,7 +1634,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W11" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X11" s="39" t="str">
         <x:v>Add a fixture for unreadable paths on each supported OS.</x:v>
@@ -1703,7 +1703,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W12" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X12" s="39" t="str">
         <x:v>Add rebase/cherry-pick/revert/bisect fixtures before action work begins.</x:v>
@@ -1772,7 +1772,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W13" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X13" s="39" t="str">
         <x:v>Add dedicated integration-state fixture matrix and user correction persistence.</x:v>
@@ -1841,7 +1841,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W14" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X14" s="39" t="str">
         <x:v>Implement fetch freshness and policy controls in Phase 2.</x:v>
@@ -1910,7 +1910,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X15" s="39" t="str">
         <x:v>Add provider-backed conditions only after permission/freshness contracts exist.</x:v>
@@ -1979,7 +1979,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W16" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X16" s="39" t="str">
         <x:v>Add UI interaction verification once the Tauri shell is launched.</x:v>
@@ -2012,7 +2012,7 @@
         <x:v>Desktop + native core</x:v>
       </x:c>
       <x:c r="I17" s="39" t="str">
-        <x:v>Transition fingerprints suppress duplicate unchanged events and retain bounded history.</x:v>
+        <x:v>Transition fingerprints suppress duplicate unchanged events, retain bounded history, and add a process-local sequence to same-second event IDs.</x:v>
       </x:c>
       <x:c r="J17" s="39" t="str">
         <x:v>Timeline shows meaningful change, not noise.</x:v>
@@ -2024,10 +2024,10 @@
         <x:v>Rust repeated-scan regression</x:v>
       </x:c>
       <x:c r="M17" s="39" t="str">
-        <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline</x:v>
       </x:c>
       <x:c r="N17" s="39" t="str">
-        <x:v>Repeated unchanged scans do not add duplicate events; changed state adds one transition event.</x:v>
+        <x:v>Repeated unchanged scans do not add duplicate events; changed state adds one transition event, including when scans share a timestamp.</x:v>
       </x:c>
       <x:c r="O17" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -2042,13 +2042,13 @@
         <x:v>History logic is isolated from current state and prunes to configured bounds.</x:v>
       </x:c>
       <x:c r="U17" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:1650-1728; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
+        <x:v>src-tauri/src/core.rs:1671-1695, 2205-2250; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
       </x:c>
       <x:c r="V17" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W17" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X17" s="39" t="str">
         <x:v>Expose retention configuration and current-state independence in Phase 2.</x:v>
@@ -2096,7 +2096,7 @@
         <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
       </x:c>
       <x:c r="N18" s="39" t="str">
-        <x:v>Six Rust tests cover transactional persistence, transition history, schema metadata, and legacy JSON migration.</x:v>
+        <x:v>Nine Rust tests cover transactional persistence, transition history, schema metadata, legacy JSON migration, action audits, and same-second event IDs.</x:v>
       </x:c>
       <x:c r="O18" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -2108,19 +2108,19 @@
         <x:v>Yes: SQLite persistence and legacy migration tests.</x:v>
       </x:c>
       <x:c r="T18" s="39" t="str">
-        <x:v>The schema is versioned, uses separate roots/repositories/expected/events tables, and keeps complex snapshot payloads behind the existing Rust contract.</x:v>
+        <x:v>The schema is versioned at v2, explicitly migrates v1, uses separate roots/repositories/expected/events/action_audits tables, and keeps complex snapshot payloads behind the existing Rust contract.</x:v>
       </x:c>
       <x:c r="U18" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:242-545, 2006-2090; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
+        <x:v>src-tauri/src/core.rs:269-345, 483-522, 535-665; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
       </x:c>
       <x:c r="V18" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W18" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X18" s="39" t="str">
-        <x:v>Add explicit schema migration steps before introducing schema version 2 and verify crash recovery on the target desktop runtime.</x:v>
+        <x:v>Verify crash recovery on the target desktop runtime before introducing provider data or a modifying action contract.</x:v>
       </x:c>
       <x:c r="Y18" s="39"/>
     </x:row>
@@ -2193,7 +2193,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X19" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y19" s="39" t="str">
         <x:v>Run a human visual pass in the Tauri window and record screenshots/interaction outcomes.</x:v>
@@ -2268,7 +2268,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X20" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y20" s="39" t="str">
         <x:v>Verify evidence drawer content, expected-state action, and close behavior manually.</x:v>
@@ -2343,7 +2343,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X21" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y21" s="39" t="str">
         <x:v>Provider install/auth and refresh evidence are Phase 2 work.</x:v>
@@ -2418,7 +2418,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X22" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y22" s="39" t="str">
         <x:v>Verify active navigation, deferred copy, and Activity/Settings content manually.</x:v>
@@ -2493,7 +2493,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X23" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y23" s="39" t="str">
         <x:v>Verify search focus, Escape dismissal, and focus behavior manually.</x:v>
@@ -2525,7 +2525,7 @@
         <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I24" s="39" t="str">
-        <x:v>Settings shows local roots, storage location, freshness, and privacy; Activity shows transition events or a truthful empty state.</x:v>
+        <x:v>Settings shows local roots, storage location, freshness, and privacy; Activity shows safe local action audits, transition events, or a truthful empty state.</x:v>
       </x:c>
       <x:c r="J24" s="39" t="str">
         <x:v>Local configuration and history are understandable without a server account or provider refresh.</x:v>
@@ -2540,7 +2540,7 @@
         <x:v>pnpm typecheck; pnpm build:web; open Settings and Activity in the Tauri window</x:v>
       </x:c>
       <x:c r="N24" s="39" t="str">
-        <x:v>Surface content is wired to the local snapshot contract and builds successfully; live rendering remains environment verification.</x:v>
+        <x:v>Surface content is wired to the local snapshot contract, including bounded action-audit rows, and builds successfully; live rendering remains environment verification.</x:v>
       </x:c>
       <x:c r="O24" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -2553,7 +2553,7 @@
         <x:v>The Tauri runtime and platform data directory are not exercised by static checks.</x:v>
       </x:c>
       <x:c r="S24" s="39" t="str">
-        <x:v>Added local Settings and Activity surfaces with explicit freshness and privacy copy.</x:v>
+        <x:v>Added local Settings and Activity surfaces with explicit freshness, privacy, safe-action, and transition-history copy.</x:v>
       </x:c>
       <x:c r="T24" s="39" t="str">
         <x:v>No; static presentation is covered by build gates.</x:v>
@@ -2568,7 +2568,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X24" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y24" s="39" t="str">
         <x:v>Verify roots, storage path, freshness, privacy, event rows, and empty state manually.</x:v>
@@ -2643,7 +2643,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X25" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y25" s="39" t="str">
         <x:v>Verify no-data, no-match, and Clear filters states manually.</x:v>
@@ -2711,7 +2711,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W26" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X26" s="39" t="str">
         <x:v>Implement desktop focus behavior for `pronto .` when the app lifecycle is available.</x:v>
@@ -2780,7 +2780,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X27" s="39" t="str">
         <x:v>Package installation and `pronto .` focus behavior remain to be verified.</x:v>
@@ -2849,7 +2849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W28" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X28" s="39" t="str">
         <x:v>Code signing/notarization is outside this local implementation.</x:v>
@@ -2918,7 +2918,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="X29" s="39" t="str">
         <x:v>Add action-tier audit tests only when modifying actions are authorized and implemented.</x:v>
@@ -2994,7 +2994,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X30" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y30" s="39" t="str">
         <x:v>Define provider permission and freshness contracts before implementation.</x:v>
@@ -3069,7 +3069,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X31" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y31" s="39" t="str">
         <x:v>Define clone destination and audit semantics before adding the action.</x:v>
@@ -3101,10 +3101,10 @@
         <x:v>Desktop + native core</x:v>
       </x:c>
       <x:c r="I32" s="39" t="str">
-        <x:v>The current slice exposes no modifying Git action, so preflight and audit are not falsely represented as complete.</x:v>
+        <x:v>The current slice exposes no modifying Git action; read-only refresh/inspect preflights and durable audits are implemented without overstating modifying-action support.</x:v>
       </x:c>
       <x:c r="J32" s="39" t="str">
-        <x:v>No action is available without a fresh preflight, exact target, audit record, and post-action rescan.</x:v>
+        <x:v>No modifying action is available without a fresh preflight, exact target, audit record, and post-action rescan; unsupported actions are recorded as blocked.</x:v>
       </x:c>
       <x:c r="K32" s="39" t="str">
         <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:529-551, 1173-1183</x:v>
@@ -3116,7 +3116,7 @@
         <x:v>Deferred until action policy is implemented</x:v>
       </x:c>
       <x:c r="N32" s="39" t="str">
-        <x:v>No modifying action adapter exists in this implementation.</x:v>
+        <x:v>No modifying action adapter exists in this implementation; the read-only foundation is covered by ACTION-002.</x:v>
       </x:c>
       <x:c r="O32" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -3129,13 +3129,13 @@
         <x:v>Requires action tiers, permission policy, audit schema, and failure semantics.</x:v>
       </x:c>
       <x:c r="S32" s="39" t="str">
-        <x:v>Read-only slice keeps the action surface absent.</x:v>
+        <x:v>Read-only slice keeps modifying operations absent while recording explicit safe-action boundaries.</x:v>
       </x:c>
       <x:c r="T32" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U32" s="39" t="str">
-        <x:v>Do not add action buttons before the preflight/audit contract is testable.</x:v>
+        <x:v>Do not add modifying action buttons before the preflight/audit contract is testable.</x:v>
       </x:c>
       <x:c r="V32" s="39" t="str">
         <x:v>pronto_prd.md:529-551</x:v>
@@ -3144,129 +3144,125 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X32" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y32" s="39" t="str">
-        <x:v>Phase 2 must add preflight tests before any modifying command.</x:v>
+        <x:v>Phase 2 must add destination-specific permission and post-action verification before any modifying command.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="70" customHeight="1">
       <x:c r="A33" s="51" t="str">
-        <x:v>PR-001</x:v>
+        <x:v>ACTION-002</x:v>
       </x:c>
       <x:c r="B33" s="39" t="str">
-        <x:v>Pull requests</x:v>
+        <x:v>Safe actions</x:v>
       </x:c>
       <x:c r="C33" s="39" t="str">
-        <x:v>Provider lifecycle</x:v>
+        <x:v>Preflight / Activity</x:v>
       </x:c>
       <x:c r="D33" s="39" t="str">
-        <x:v>As an operator, I can create or merge a PR only when provider facts and permissions are verifiable.</x:v>
+        <x:v>As an operator, I can preflight a read-only local action and review its durable audit outcome.</x:v>
       </x:c>
       <x:c r="E33" s="39" t="str">
-        <x:v>Provider-connected operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F33" s="39" t="str">
-        <x:v>Provider auth required</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G33" s="39" t="str">
-        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
+        <x:v>Registered roots or scanned repositories</x:v>
       </x:c>
       <x:c r="H33" s="39" t="str">
-        <x:v>Desktop + provider API</x:v>
+        <x:v>Desktop + native core</x:v>
       </x:c>
       <x:c r="I33" s="39" t="str">
-        <x:v>PR creation, review evidence, and merge actions are explicit deferred boundaries.</x:v>
+        <x:v>The native allowlist permits refresh and inspect as read-only actions, resolves exact root/repository target IDs, records rejected unsupported actions, and completes refresh audits after the local scan.</x:v>
       </x:c>
       <x:c r="J33" s="39" t="str">
-        <x:v>Unknown checks or reviews never become a merge-eligible state.</x:v>
+        <x:v>I can see what local action was considered, its risk/status, and the exact target boundary without any Git mutation or provider write.</x:v>
       </x:c>
       <x:c r="K33" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>src-tauri/src/core.rs:1739-1924, 2050-2063, 2205-2250; src-tauri/src/lib.rs:18-26; src/renderer/src/api.ts; src/renderer/src/components/WorkspaceSurfaces.tsx:45-99; /Users/jakyeamos/Downloads/pronto_prd.md:529-551, 1173-1183</x:v>
       </x:c>
       <x:c r="L33" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust regression + typecheck/build + Activity source review</x:v>
       </x:c>
       <x:c r="M33" s="39" t="str">
-        <x:v>Deferred: provider permission and PR API required</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; pnpm typecheck; pnpm build:web</x:v>
       </x:c>
       <x:c r="N33" s="39" t="str">
-        <x:v>No PR lifecycle implementation is present.</x:v>
+        <x:v>Nine Rust tests pass, including allowed/rejected preflights, completed refresh audit, schema-v1 migration, and same-second transition persistence; Activity renders audit rows.</x:v>
       </x:c>
       <x:c r="O33" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P33" s="39" t="str"/>
-      <x:c r="Q33" s="39" t="str">
-        <x:v>Dependency</x:v>
-      </x:c>
-      <x:c r="R33" s="39" t="str">
-        <x:v>Requires provider adapter, permission degradation, and action audit.</x:v>
-      </x:c>
+      <x:c r="Q33" s="39" t="str"/>
+      <x:c r="R33" s="39" t="str"/>
       <x:c r="S33" s="39" t="str">
-        <x:v>Deferred with explicit unknown/unavailable semantics.</x:v>
+        <x:v>Yes: preflight, rejected-action, completed-refresh, migration, and collision regression tests.</x:v>
       </x:c>
       <x:c r="T33" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Explicit allowlist and one persistence path keep action policy out of display components; modifying operations remain absent.</x:v>
       </x:c>
       <x:c r="U33" s="39" t="str">
-        <x:v>PR work depends on provider state and cannot be safely inferred from local Git alone.</x:v>
+        <x:v>Yes: native Rust regression coverage.</x:v>
       </x:c>
       <x:c r="V33" s="39" t="str">
-        <x:v>pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>b13de08 source/test output</x:v>
       </x:c>
       <x:c r="W33" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="X33" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y33" s="39" t="str">
-        <x:v>Add provider-backed evidence before adding any merge control.</x:v>
+        <x:v>Read-only inspect is preflight-only; add modifying actions only with destination-specific permission and post-action verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="70" customHeight="1">
       <x:c r="A34" s="51" t="str">
-        <x:v>REL-001</x:v>
+        <x:v>PR-001</x:v>
       </x:c>
       <x:c r="B34" s="39" t="str">
-        <x:v>Releases</x:v>
+        <x:v>Pull requests</x:v>
       </x:c>
       <x:c r="C34" s="39" t="str">
-        <x:v>Release preparation</x:v>
+        <x:v>Provider lifecycle</x:v>
       </x:c>
       <x:c r="D34" s="39" t="str">
-        <x:v>As an operator, I can prepare a deterministic release draft without publishing it automatically.</x:v>
+        <x:v>As an operator, I can create or merge a PR only when provider facts and permissions are verifiable.</x:v>
       </x:c>
       <x:c r="E34" s="39" t="str">
-        <x:v>Release maintainer</x:v>
+        <x:v>Provider-connected operator</x:v>
       </x:c>
       <x:c r="F34" s="39" t="str">
         <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G34" s="39" t="str">
-        <x:v>Published release baseline, configured rule, clean isolated worktree</x:v>
+        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
       </x:c>
       <x:c r="H34" s="39" t="str">
         <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I34" s="39" t="str">
-        <x:v>Release baseline, deterministic rules, isolated worktrees, and draft handoff are deferred.</x:v>
+        <x:v>PR creation, review evidence, and merge actions are explicit deferred boundaries.</x:v>
       </x:c>
       <x:c r="J34" s="39" t="str">
-        <x:v>No release threshold or version recommendation appears until its configured evidence exists.</x:v>
+        <x:v>Unknown checks or reviews never become a merge-eligible state.</x:v>
       </x:c>
       <x:c r="K34" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
       </x:c>
       <x:c r="L34" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M34" s="39" t="str">
-        <x:v>Deferred: provider, release recipe, and isolated worktree gates required</x:v>
+        <x:v>Deferred: provider permission and PR API required</x:v>
       </x:c>
       <x:c r="N34" s="39" t="str">
-        <x:v>No release preparation or publication path is implemented.</x:v>
+        <x:v>No PR lifecycle implementation is present.</x:v>
       </x:c>
       <x:c r="O34" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -3276,72 +3272,72 @@
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R34" s="39" t="str">
-        <x:v>Requires exact diff review, validation gates, and publication boundary.</x:v>
+        <x:v>Requires provider adapter, permission degradation, and action audit.</x:v>
       </x:c>
       <x:c r="S34" s="39" t="str">
-        <x:v>Phase 3 plan preserves the no-publish rule.</x:v>
+        <x:v>Deferred with explicit unknown/unavailable semantics.</x:v>
       </x:c>
       <x:c r="T34" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U34" s="39" t="str">
-        <x:v>Release automation is intentionally not inferred from local commit counts.</x:v>
+        <x:v>PR work depends on provider state and cannot be safely inferred from local Git alone.</x:v>
       </x:c>
       <x:c r="V34" s="39" t="str">
-        <x:v>pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>pronto_prd.md:555-571, 1185-1189</x:v>
       </x:c>
       <x:c r="W34" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X34" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y34" s="39" t="str">
-        <x:v>Define recipe state and audit events before implementation.</x:v>
+        <x:v>Add provider-backed evidence before adding any merge control.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="70" customHeight="1">
       <x:c r="A35" s="51" t="str">
-        <x:v>PROC-001</x:v>
+        <x:v>REL-001</x:v>
       </x:c>
       <x:c r="B35" s="39" t="str">
-        <x:v>Agent workspaces</x:v>
+        <x:v>Releases</x:v>
       </x:c>
       <x:c r="C35" s="39" t="str">
-        <x:v>Process / terminal evidence</x:v>
+        <x:v>Release preparation</x:v>
       </x:c>
       <x:c r="D35" s="39" t="str">
-        <x:v>As an operator, I can tell whether an agent workspace has process evidence without exposing terminal contents.</x:v>
+        <x:v>As an operator, I can prepare a deterministic release draft without publishing it automatically.</x:v>
       </x:c>
       <x:c r="E35" s="39" t="str">
-        <x:v>Local operator</x:v>
+        <x:v>Release maintainer</x:v>
       </x:c>
       <x:c r="F35" s="39" t="str">
-        <x:v>Local permission required</x:v>
+        <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G35" s="39" t="str">
-        <x:v>OS process inspection permission and optional manifest</x:v>
+        <x:v>Published release baseline, configured rule, clean isolated worktree</x:v>
       </x:c>
       <x:c r="H35" s="39" t="str">
-        <x:v>Desktop + native adapters</x:v>
+        <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I35" s="39" t="str">
-        <x:v>Process, terminal, and generic agent adapters are deferred; no certainty is claimed from their absence.</x:v>
+        <x:v>Release baseline, deterministic rules, isolated worktrees, and draft handoff are deferred.</x:v>
       </x:c>
       <x:c r="J35" s="39" t="str">
-        <x:v>Unknown process evidence remains unknown rather than being classified as inactive or safe to clean.</x:v>
+        <x:v>No release threshold or version recommendation appears until its configured evidence exists.</x:v>
       </x:c>
       <x:c r="K35" s="39" t="str">
-        <x:v>docs/implementation-plan.md:51-54; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
       </x:c>
       <x:c r="L35" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M35" s="39" t="str">
-        <x:v>Deferred: OS adapter and permission boundary required</x:v>
+        <x:v>Deferred: provider, release recipe, and isolated worktree gates required</x:v>
       </x:c>
       <x:c r="N35" s="39" t="str">
-        <x:v>No process or terminal capture is implemented.</x:v>
+        <x:v>No release preparation or publication path is implemented.</x:v>
       </x:c>
       <x:c r="O35" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -3351,147 +3347,147 @@
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R35" s="39" t="str">
-        <x:v>Cross-platform process APIs and privacy review are required.</x:v>
+        <x:v>Requires exact diff review, validation gates, and publication boundary.</x:v>
       </x:c>
       <x:c r="S35" s="39" t="str">
-        <x:v>The current slice only models linked worktrees as local workspaces.</x:v>
+        <x:v>Phase 3 plan preserves the no-publish rule.</x:v>
       </x:c>
       <x:c r="T35" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U35" s="39" t="str">
-        <x:v>Never capture terminal contents, prompts, source text, or keystrokes.</x:v>
+        <x:v>Release automation is intentionally not inferred from local commit counts.</x:v>
       </x:c>
       <x:c r="V35" s="39" t="str">
-        <x:v>pronto_prd.md:489-525</x:v>
+        <x:v>pronto_prd.md:575-655, 1191-1203</x:v>
       </x:c>
       <x:c r="W35" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X35" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y35" s="39" t="str">
-        <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
+        <x:v>Define recipe state and audit events before implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="70" customHeight="1">
       <x:c r="A36" s="51" t="str">
-        <x:v>GROUP-001</x:v>
+        <x:v>PROC-001</x:v>
       </x:c>
       <x:c r="B36" s="39" t="str">
-        <x:v>Products</x:v>
+        <x:v>Agent workspaces</x:v>
       </x:c>
       <x:c r="C36" s="39" t="str">
-        <x:v>Products / groups</x:v>
+        <x:v>Process / terminal evidence</x:v>
       </x:c>
       <x:c r="D36" s="39" t="str">
-        <x:v>As an operator, I can aggregate multiple repositories without hiding repository-level evidence.</x:v>
+        <x:v>As an operator, I can tell whether an agent workspace has process evidence without exposing terminal contents.</x:v>
       </x:c>
       <x:c r="E36" s="39" t="str">
-        <x:v>Portfolio operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F36" s="39" t="str">
-        <x:v>Local-only or provider auth</x:v>
+        <x:v>Local permission required</x:v>
       </x:c>
       <x:c r="G36" s="39" t="str">
-        <x:v>Product/group configuration and participating repositories</x:v>
+        <x:v>OS process inspection permission and optional manifest</x:v>
       </x:c>
       <x:c r="H36" s="39" t="str">
-        <x:v>Desktop 1280×800</x:v>
+        <x:v>Desktop + native adapters</x:v>
       </x:c>
       <x:c r="I36" s="39" t="str">
-        <x:v>Products, groups, and coordinated release are deferred; the current portfolio remains repository-first.</x:v>
+        <x:v>Process, terminal, and generic agent adapters are deferred; no certainty is claimed from their absence.</x:v>
       </x:c>
       <x:c r="J36" s="39" t="str">
-        <x:v>No aggregate product status is shown until its repository-level provenance and release policy are defined.</x:v>
+        <x:v>Unknown process evidence remains unknown rather than being classified as inactive or safe to clean.</x:v>
       </x:c>
       <x:c r="K36" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>docs/implementation-plan.md:51-54; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
       </x:c>
       <x:c r="L36" s="39" t="str">
         <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M36" s="39" t="str">
-        <x:v>Deferred: product model and coordination policy required</x:v>
+        <x:v>Deferred: OS adapter and permission boundary required</x:v>
       </x:c>
       <x:c r="N36" s="39" t="str">
-        <x:v>No product/group mutation or coordinated release logic is implemented.</x:v>
+        <x:v>No process or terminal capture is implemented.</x:v>
       </x:c>
       <x:c r="O36" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Needs-Environment</x:v>
       </x:c>
       <x:c r="P36" s="39" t="str"/>
       <x:c r="Q36" s="39" t="str">
-        <x:v>Product</x:v>
+        <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R36" s="39" t="str">
-        <x:v>Manual product/group configuration is accepted; implementation still needs the durable state and coordination model.</x:v>
+        <x:v>Cross-platform process APIs and privacy review are required.</x:v>
       </x:c>
       <x:c r="S36" s="39" t="str">
-        <x:v>Repository-first UI avoids a premature inferred aggregate abstraction.</x:v>
+        <x:v>The current slice only models linked worktrees as local workspaces.</x:v>
       </x:c>
       <x:c r="T36" s="39" t="str">
         <x:v>No.</x:v>
       </x:c>
       <x:c r="U36" s="39" t="str">
-        <x:v>This is an accepted delivery boundary, not an unresolved product decision.</x:v>
+        <x:v>Never capture terminal contents, prompts, source text, or keystrokes.</x:v>
       </x:c>
       <x:c r="V36" s="39" t="str">
-        <x:v>pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>pronto_prd.md:489-525</x:v>
       </x:c>
       <x:c r="W36" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X36" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y36" s="39" t="str">
-        <x:v>Implement manual product/group configuration after the SQLite contract is stable.</x:v>
+        <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="70" customHeight="1">
       <x:c r="A37" s="51" t="str">
-        <x:v>AI-001</x:v>
+        <x:v>GROUP-001</x:v>
       </x:c>
       <x:c r="B37" s="39" t="str">
-        <x:v>AI and privacy</x:v>
+        <x:v>Products</x:v>
       </x:c>
       <x:c r="C37" s="39" t="str">
-        <x:v>Privacy boundary</x:v>
+        <x:v>Products / groups</x:v>
       </x:c>
       <x:c r="D37" s="39" t="str">
-        <x:v>As an operator, I can keep AI disabled and prevent uncommitted source from leaving the machine.</x:v>
+        <x:v>As an operator, I can aggregate multiple repositories without hiding repository-level evidence.</x:v>
       </x:c>
       <x:c r="E37" s="39" t="str">
-        <x:v>Privacy-conscious operator</x:v>
+        <x:v>Portfolio operator</x:v>
       </x:c>
       <x:c r="F37" s="39" t="str">
-        <x:v>AI disabled by default</x:v>
+        <x:v>Local-only or provider auth</x:v>
       </x:c>
       <x:c r="G37" s="39" t="str">
-        <x:v>Explicit provider/model permission and approved payload</x:v>
+        <x:v>Product/group configuration and participating repositories</x:v>
       </x:c>
       <x:c r="H37" s="39" t="str">
-        <x:v>Desktop + provider/local model</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I37" s="39" t="str">
-        <x:v>No AI request path exists in this slice; local snapshots contain metadata and no uncommitted diff content.</x:v>
+        <x:v>Products, groups, and coordinated release are deferred; the current portfolio remains repository-first.</x:v>
       </x:c>
       <x:c r="J37" s="39" t="str">
-        <x:v>No AI claim or payload is possible until the user opts in and reviews the exact payload categories.</x:v>
+        <x:v>No aggregate product status is shown until its repository-level provenance and release policy are defined.</x:v>
       </x:c>
       <x:c r="K37" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:32-188; src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
       </x:c>
       <x:c r="L37" s="39" t="str">
-        <x:v>Static safety review + privacy regression</x:v>
+        <x:v>Boundary review</x:v>
       </x:c>
       <x:c r="M37" s="39" t="str">
-        <x:v>rg 'diff|filename|content' src-tauri/src/core.rs src/renderer/src; cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+        <x:v>Deferred: product model and coordination policy required</x:v>
       </x:c>
       <x:c r="N37" s="39" t="str">
-        <x:v>No external AI call is implemented; snapshot privacy test passes and UI states the local/private boundary.</x:v>
+        <x:v>No product/group mutation or coordinated release logic is implemented.</x:v>
       </x:c>
       <x:c r="O37" s="39" t="str">
         <x:v>Deferred</x:v>
@@ -3501,98 +3497,173 @@
         <x:v>Product</x:v>
       </x:c>
       <x:c r="R37" s="39" t="str">
-        <x:v>AI remains disabled by the accepted product direction; payload categories and provider permissions are outside this slice.</x:v>
+        <x:v>Manual product/group configuration is accepted; implementation still needs the durable state and coordination model.</x:v>
       </x:c>
       <x:c r="S37" s="39" t="str">
-        <x:v>Deferred AI authority; local metadata-only evidence remains available.</x:v>
+        <x:v>Repository-first UI avoids a premature inferred aggregate abstraction.</x:v>
       </x:c>
       <x:c r="T37" s="39" t="str">
-        <x:v>Yes: snapshot excludes source/diff content.</x:v>
+        <x:v>No.</x:v>
       </x:c>
       <x:c r="U37" s="39" t="str">
-        <x:v>AI is not introduced as a shortcut for missing provider evidence.</x:v>
+        <x:v>This is an accepted delivery boundary, not an unresolved product decision.</x:v>
       </x:c>
       <x:c r="V37" s="39" t="str">
-        <x:v>pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>pronto_prd.md:227-238, 659-677</x:v>
       </x:c>
       <x:c r="W37" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X37" s="39" t="str">
-        <x:v>d332573</x:v>
+        <x:v>b13de08</x:v>
       </x:c>
       <x:c r="Y37" s="39" t="str">
-        <x:v>Keep AI disabled until per-repository permissions and payload preview are explicitly designed.</x:v>
+        <x:v>Implement manual product/group configuration after the SQLite contract is stable.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
       <x:c r="A38" s="51" t="str">
+        <x:v>AI-001</x:v>
+      </x:c>
+      <x:c r="B38" s="39" t="str">
+        <x:v>AI and privacy</x:v>
+      </x:c>
+      <x:c r="C38" s="39" t="str">
+        <x:v>Privacy boundary</x:v>
+      </x:c>
+      <x:c r="D38" s="39" t="str">
+        <x:v>As an operator, I can keep AI disabled and prevent uncommitted source from leaving the machine.</x:v>
+      </x:c>
+      <x:c r="E38" s="39" t="str">
+        <x:v>Privacy-conscious operator</x:v>
+      </x:c>
+      <x:c r="F38" s="39" t="str">
+        <x:v>AI disabled by default</x:v>
+      </x:c>
+      <x:c r="G38" s="39" t="str">
+        <x:v>Explicit provider/model permission and approved payload</x:v>
+      </x:c>
+      <x:c r="H38" s="39" t="str">
+        <x:v>Desktop + provider/local model</x:v>
+      </x:c>
+      <x:c r="I38" s="39" t="str">
+        <x:v>No AI request path exists in this slice; local snapshots contain metadata and no uncommitted diff content.</x:v>
+      </x:c>
+      <x:c r="J38" s="39" t="str">
+        <x:v>No AI claim or payload is possible until the user opts in and reviews the exact payload categories.</x:v>
+      </x:c>
+      <x:c r="K38" s="39" t="str">
+        <x:v>src-tauri/src/core.rs:32-188; src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
+      </x:c>
+      <x:c r="L38" s="39" t="str">
+        <x:v>Static safety review + privacy regression</x:v>
+      </x:c>
+      <x:c r="M38" s="39" t="str">
+        <x:v>rg 'diff|filename|content' src-tauri/src/core.rs src/renderer/src; cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+      </x:c>
+      <x:c r="N38" s="39" t="str">
+        <x:v>No external AI call is implemented; snapshot privacy test passes and UI states the local/private boundary.</x:v>
+      </x:c>
+      <x:c r="O38" s="39" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="P38" s="39" t="str"/>
+      <x:c r="Q38" s="39" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="R38" s="39" t="str">
+        <x:v>AI remains disabled by the accepted product direction; payload categories and provider permissions are outside this slice.</x:v>
+      </x:c>
+      <x:c r="S38" s="39" t="str">
+        <x:v>Deferred AI authority; local metadata-only evidence remains available.</x:v>
+      </x:c>
+      <x:c r="T38" s="39" t="str">
+        <x:v>Yes: snapshot excludes source/diff content.</x:v>
+      </x:c>
+      <x:c r="U38" s="39" t="str">
+        <x:v>AI is not introduced as a shortcut for missing provider evidence.</x:v>
+      </x:c>
+      <x:c r="V38" s="39" t="str">
+        <x:v>pronto_prd.md:679-695, 1205-1211</x:v>
+      </x:c>
+      <x:c r="W38" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X38" s="39" t="str">
+        <x:v>b13de08</x:v>
+      </x:c>
+      <x:c r="Y38" s="39" t="str">
+        <x:v>Keep AI disabled until per-repository permissions and payload preview are explicitly designed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="70" customHeight="1">
+      <x:c r="A39" s="51" t="str">
         <x:v>HIST-001</x:v>
       </x:c>
-      <x:c r="B38" s="39" t="str">
+      <x:c r="B39" s="39" t="str">
         <x:v>History</x:v>
       </x:c>
-      <x:c r="C38" s="39" t="str">
+      <x:c r="C39" s="39" t="str">
         <x:v>Event retention</x:v>
       </x:c>
-      <x:c r="D38" s="39" t="str">
+      <x:c r="D39" s="39" t="str">
         <x:v>As an operator, I can retain bounded transition history without losing current state.</x:v>
       </x:c>
-      <x:c r="E38" s="39" t="str">
+      <x:c r="E39" s="39" t="str">
         <x:v>Local operator</x:v>
       </x:c>
-      <x:c r="F38" s="39" t="str">
+      <x:c r="F39" s="39" t="str">
         <x:v>Local-only</x:v>
       </x:c>
-      <x:c r="G38" s="39" t="str">
+      <x:c r="G39" s="39" t="str">
         <x:v>Transition events persisted in local store</x:v>
       </x:c>
-      <x:c r="H38" s="39" t="str">
+      <x:c r="H39" s="39" t="str">
         <x:v>Native core</x:v>
       </x:c>
-      <x:c r="I38" s="39" t="str">
-        <x:v>Events are transition-only, retained for a default bounded window, and pruned independently of current snapshots.</x:v>
-      </x:c>
-      <x:c r="J38" s="39" t="str">
+      <x:c r="I39" s="39" t="str">
+        <x:v>Events are transition-only with sequence-safe IDs, retained for a default bounded window, and action audits are bounded and pruned independently of current snapshots.</x:v>
+      </x:c>
+      <x:c r="J39" s="39" t="str">
         <x:v>History is useful without growing indefinitely or becoming a source-content archive.</x:v>
       </x:c>
-      <x:c r="K38" s="39" t="str">
+      <x:c r="K39" s="39" t="str">
         <x:v>src-tauri/src/core.rs:110-149, 1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
       </x:c>
-      <x:c r="L38" s="39" t="str">
+      <x:c r="L39" s="39" t="str">
         <x:v>Rust repeated-scan regression + source review</x:v>
       </x:c>
-      <x:c r="M38" s="39" t="str">
-        <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
-      </x:c>
-      <x:c r="N38" s="39" t="str">
-        <x:v>Transition persistence passes; the 90-day default and configurable retention are represented in the core constants/logic for this slice.</x:v>
-      </x:c>
-      <x:c r="O38" s="39" t="str">
+      <x:c r="M39" s="39" t="str">
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline</x:v>
+      </x:c>
+      <x:c r="N39" s="39" t="str">
+        <x:v>Transition persistence passes, including same-second IDs; the 90-day default and configurable retention are represented in the core constants/logic for this slice, with action audits bounded to recent records.</x:v>
+      </x:c>
+      <x:c r="O39" s="39" t="str">
         <x:v>Regression-Covered</x:v>
       </x:c>
-      <x:c r="P38" s="39" t="str"/>
-      <x:c r="Q38" s="39" t="str"/>
-      <x:c r="R38" s="39" t="str"/>
-      <x:c r="S38" s="39" t="str">
+      <x:c r="P39" s="39" t="str"/>
+      <x:c r="Q39" s="39" t="str"/>
+      <x:c r="R39" s="39" t="str"/>
+      <x:c r="S39" s="39" t="str">
         <x:v>Yes: repeated-scan event regression.</x:v>
       </x:c>
-      <x:c r="T38" s="39" t="str">
-        <x:v>Bounded event history is a small persistence concern; durable configuration remains Phase 2.</x:v>
-      </x:c>
-      <x:c r="U38" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
-      </x:c>
-      <x:c r="V38" s="39" t="str">
+      <x:c r="T39" s="39" t="str">
+        <x:v>Bounded event and action-audit history is a small persistence concern; durable configuration remains Phase 2.</x:v>
+      </x:c>
+      <x:c r="U39" s="39" t="str">
+        <x:v>src-tauri/src/core.rs:1671-1695, 1739-1780, 1900-1924; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
+      </x:c>
+      <x:c r="V39" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W38" s="39" t="str">
-        <x:v>d332573</x:v>
-      </x:c>
-      <x:c r="X38" s="39" t="str">
-        <x:v>Expose retention settings and add date-boundary tests.</x:v>
-      </x:c>
-      <x:c r="Y38" s="39"/>
+      <x:c r="W39" s="39" t="str">
+        <x:v>b13de08</x:v>
+      </x:c>
+      <x:c r="X39" s="39" t="str">
+        <x:v>Expose retention settings and add date-boundary tests for action audits.</x:v>
+      </x:c>
+      <x:c r="Y39" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3600,7 +3671,7 @@
     <x:mergeCell ref="A2:Y2"/>
     <x:mergeCell ref="A3:Y3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="O5:O38">
+  <x:conditionalFormatting sqref="O5:O39">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Regression-Covered"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Verified"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Build verified"/>
@@ -3610,13 +3681,13 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="O5:O38">
+    <x:dataValidation type="list" sqref="O5:O39">
       <x:formula1>"Regression-Covered,Verified,Needs-Environment,Needs-Product-Decision,Deferred"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c7dcdb113f467a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54b1e35410444d39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3821,13 +3892,13 @@
         <x:v>FR-065–070; AC-015–018</x:v>
       </x:c>
       <x:c r="C12" s="39" t="str">
-        <x:v>SAFE-001; ACTION-001</x:v>
+        <x:v>SAFE-001; ACTION-001–002</x:v>
       </x:c>
       <x:c r="D12" s="39" t="str">
-        <x:v>Read-only only</x:v>
+        <x:v>Read-only audited</x:v>
       </x:c>
       <x:c r="E12" s="39" t="str">
-        <x:v>Structured Git boundary and prohibited-action absence are verified. Modifying actions require fresh preflight, audit, and exact-target contracts.</x:v>
+        <x:v>Explicit allowlist permits refresh/inspect, resolves exact root/repository IDs, records rejected unsupported actions, and completes refresh audits. Modifying actions remain deferred behind fresh preflight, audit, and exact-target contracts.</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
         <x:v>Phase 2</x:v>
@@ -3921,13 +3992,13 @@
         <x:v>FR-109–112; AC-031–032</x:v>
       </x:c>
       <x:c r="C17" s="39" t="str">
-        <x:v>AUD-001; HIST-001; UI-006</x:v>
+        <x:v>AUD-001; HIST-001; UI-006; ACTION-002</x:v>
       </x:c>
       <x:c r="D17" s="39" t="str">
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E17" s="39" t="str">
-        <x:v>Transition-only metadata history and bounded pruning are implemented and surfaced in Activity; configurable retention and future schema migrations remain deferred.</x:v>
+        <x:v>Transition-only metadata history and bounded action-audit history are implemented and surfaced in Activity; configurable retention and future schema migrations remain deferred.</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
         <x:v>Phase 2</x:v>
@@ -3947,7 +4018,7 @@
         <x:v>Read-only verified</x:v>
       </x:c>
       <x:c r="E18" s="39" t="str">
-        <x:v>Shared Rust core powers human/JSON status and the Node wrapper; desktop focus and policy expansion await action work.</x:v>
+        <x:v>Shared Rust core powers human/JSON status and the Node wrapper; completed refresh audits persist in the shared registry, while desktop focus and policy expansion await action work.</x:v>
       </x:c>
       <x:c r="F18" s="40" t="str">
         <x:v>Phase 1</x:v>
@@ -3994,7 +4065,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff6a473fff6b4fa8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recb18da0c7d64480"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4035,7 +4106,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Implementation commit: d332573 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
+        <x:v>Implementation commit: b13de08 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -4077,33 +4148,33 @@
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="61" t="n">
-        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$38)</x:f>
-        <x:v>34</x:v>
+        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$39)</x:f>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B5" s="62"/>
       <x:c r="C5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Regression-Covered")</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Regression-Covered")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D5" s="62"/>
       <x:c r="E5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$38,"Build verified")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$39,"Build verified")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F5" s="62"/>
       <x:c r="G5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Needs-Environment")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Needs-Environment")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="H5" s="62"/>
       <x:c r="I5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$38,"Needs-Product-Decision")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Needs-Product-Decision")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J5" s="62"/>
       <x:c r="K5" s="63" t="n">
         <x:f>(C5+E5+G5)/(A5)</x:f>
-        <x:v>0.9411764705882353</x:v>
+        <x:v>0.9428571428571428</x:v>
       </x:c>
       <x:c r="L5" s="64"/>
     </x:row>
@@ -4154,7 +4225,7 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F10" s="37" t="str">
-        <x:v>Local UX slice is implemented at 885fe1e; workbook review is this iteration.</x:v>
+        <x:v>Local UX, durable SQLite state, and read-only action audit foundation are implemented at b13de08; workbook review is this iteration.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -4171,10 +4242,10 @@
         <x:v>Provider permission and action audit design review</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>Versioned SQLite is complete; read-only GitHub and safe local actions follow explicit contracts.</x:v>
+        <x:v>Versioned SQLite and the read-only action-audit foundation are complete; read-only GitHub follows explicit identity/freshness contracts; modifying actions remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -4272,12 +4343,12 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D21" s="40" t="str">
-        <x:v>6 Rust tests; Vitest no test files</x:v>
+        <x:v>9 Rust tests; Vitest no test files</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
       <x:c r="A22" s="38" t="str">
-        <x:v>cargo check --manifest-path src-tauri/Cargo.toml</x:v>
+        <x:v>cargo check --manifest-path src-tauri/Cargo.toml --offline</x:v>
       </x:c>
       <x:c r="B22" s="39" t="str">
         <x:v>Native compilation</x:v>
@@ -4300,7 +4371,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D23" s="40" t="str">
-        <x:v>JSON output</x:v>
+        <x:v>JSON output includes the shared action_audits field</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="32" customHeight="1">
@@ -4314,7 +4385,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>Vite production bundle emitted after the local UX slice</x:v>
+        <x:v>Vite production bundle emitted with safe action history wiring</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
@@ -4328,21 +4399,21 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D25" s="40" t="str">
-        <x:v>Pronto.app and Pronto_0.1.0_aarch64.dmg emitted</x:v>
+        <x:v>Pronto.app and Pronto_0.1.0_aarch64.dmg emitted after the action-audit slice</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="38" t="str">
-        <x:v>pre-cr run --workspace .</x:v>
+        <x:v>pre-cr run --json --workspace .</x:v>
       </x:c>
       <x:c r="B26" s="39" t="str">
         <x:v>Commit readiness / anti-slop</x:v>
       </x:c>
       <x:c r="C26" s="39" t="str">
-        <x:v>Pass</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="D26" s="40" t="str">
-        <x:v>0% threshold; no-instrumentation adapter explicit</x:v>
+        <x:v>Docs/workbook-only changes are ignored by the configured source surfaces; no changed-line coverage result was produced. Source commit b13de08 passed its commit-time gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="32" customHeight="1">
@@ -4377,7 +4448,7 @@
     </x:row>
     <x:row r="31" ht="26" customHeight="1">
       <x:c r="A31" s="8" t="str">
-        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX and durable-state slices are implemented; the next safe expansion is action preflight/audit, followed by read-only provider context.</x:v>
+        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX, durable-state, and read-only action preflight/audit slices are implemented at b13de08; the next safe expansion is read-only provider context.</x:v>
       </x:c>
       <x:c r="B31" s="8"/>
       <x:c r="C31" s="8"/>

</xml_diff>

<commit_message>
docs: refresh prd behavior workbook
</commit_message>
<xml_diff>
--- a/docs/pronto-behavior-spec.xlsx
+++ b/docs/pronto-behavior-spec.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R3059b3698dac4cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="R5a543ef32eba4011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R9b1ed6bb24504c9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behavior Inventory" sheetId="1" r:id="R7e99967b88404b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Boundaries" sheetId="2" r:id="Rdc4aaf7d49614ff6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Plan" sheetId="3" r:id="R1f9dd747f18b4a7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -720,7 +720,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BehaviorInventoryTable" displayName="BehaviorInventoryTable" ref="A4:Y40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="25">
     <x:tableColumn id="1" name="Feature ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1019,7 +1019,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot b13de08</x:v>
+        <x:v>Source: /Users/jakyeamos/Downloads/pronto_prd.md | reviewed 2026-07-25 | implementation snapshot c0bf758</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1221,7 +1221,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X5" s="36" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y5" s="36" t="str">
         <x:v>Verify macOS, Windows, and Linux folder permissions when the desktop shell is launched.</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X6" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y6" s="39" t="str">
         <x:v>Add configurable glob-pattern coverage in the provider/durable-state phase.</x:v>
@@ -1358,7 +1358,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W7" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X7" s="39" t="str">
         <x:v>Submodule promotion and symlink-root matrix remain for the discovery expansion.</x:v>
@@ -1391,22 +1391,22 @@
         <x:v>Desktop + CLI</x:v>
       </x:c>
       <x:c r="I8" s="39" t="str">
-        <x:v>The snapshot exposes counts and aggregate line totals, not filenames, patch text, or source content.</x:v>
+        <x:v>The portfolio snapshot exposes counts and aggregate line totals, not filenames, patch text, or source content; the separate AI preview only includes committed metadata or committed diff content after repository permission is selected.</x:v>
       </x:c>
       <x:c r="J8" s="39" t="str">
-        <x:v>Portfolio evidence is useful for triage while remaining metadata-only.</x:v>
+        <x:v>Portfolio evidence is useful for triage while the privacy boundary makes every AI payload category explicit and excludes uncommitted content.</x:v>
       </x:c>
       <x:c r="K8" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:32-188, 443-516; /Users/jakyeamos/Downloads/pronto_prd.md:314-328, 906-920</x:v>
+        <x:v>src-tauri/src/core.rs:32-188, 443-516, 2880-3065; /Users/jakyeamos/Downloads/pronto_prd.md:314-328, 679-695, 906-920</x:v>
       </x:c>
       <x:c r="L8" s="39" t="str">
-        <x:v>Rust serialized snapshot assertion + source review</x:v>
+        <x:v>Rust serialized snapshot and AI payload regression assertions + source review</x:v>
       </x:c>
       <x:c r="M8" s="39" t="str">
-        <x:v>cargo test --manifest-path src-tauri/Cargo.toml; pnpm cli:json</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; pnpm cli:json</x:v>
       </x:c>
       <x:c r="N8" s="39" t="str">
-        <x:v>Fixture assertions inspect serialized JSON and confirm no filename or diff payload is returned.</x:v>
+        <x:v>Fixture assertions confirm base snapshots contain no filename/diff payload and AI previews exclude uncommitted.txt while exposing only the permitted committed categories.</x:v>
       </x:c>
       <x:c r="O8" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -1415,22 +1415,22 @@
       <x:c r="Q8" s="39" t="str"/>
       <x:c r="R8" s="39" t="str"/>
       <x:c r="S8" s="39" t="str">
-        <x:v>Yes: snapshot privacy assertion.</x:v>
+        <x:v>Yes: snapshot privacy and AI payload regression assertions.</x:v>
       </x:c>
       <x:c r="T8" s="39" t="str">
-        <x:v>Privacy is encoded at the data contract rather than hidden only in presentation.</x:v>
+        <x:v>Privacy is encoded at the data contract and permissioned preview rather than hidden only in presentation.</x:v>
       </x:c>
       <x:c r="U8" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:1602-1644; /Users/jakyeamos/Downloads/pronto_prd.md:314-328</x:v>
+        <x:v>src-tauri/src/core.rs:1602-1644, 6293-6375; /Users/jakyeamos/Downloads/pronto_prd.md:314-328, 679-695</x:v>
       </x:c>
       <x:c r="V8" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W8" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X8" s="39" t="str">
-        <x:v>Provider and AI payload previews still need their own explicit contract.</x:v>
+        <x:v>External AI request execution remains intentionally absent; local payload preview is the evidence boundary.</x:v>
       </x:c>
       <x:c r="Y8" s="39"/>
     </x:row>
@@ -1496,7 +1496,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W9" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X9" s="39" t="str">
         <x:v>Add fetched-at evidence after fetch/provider refresh exists.</x:v>
@@ -1565,7 +1565,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W10" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X10" s="39" t="str">
         <x:v>Add staged + unstaged + untracked matrix cases as scan coverage grows.</x:v>
@@ -1634,7 +1634,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W11" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X11" s="39" t="str">
         <x:v>Add a fixture for unreadable paths on each supported OS.</x:v>
@@ -1703,7 +1703,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W12" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X12" s="39" t="str">
         <x:v>Add rebase/cherry-pick/revert/bisect fixtures before action work begins.</x:v>
@@ -1772,7 +1772,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W13" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X13" s="39" t="str">
         <x:v>Add dedicated integration-state fixture matrix and user correction persistence.</x:v>
@@ -1841,7 +1841,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W14" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X14" s="39" t="str">
         <x:v>Implement fetch freshness and policy controls in Phase 2.</x:v>
@@ -1910,7 +1910,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X15" s="39" t="str">
         <x:v>Add provider-backed conditions only after permission/freshness contracts exist.</x:v>
@@ -1979,7 +1979,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W16" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X16" s="39" t="str">
         <x:v>Add UI interaction verification once the Tauri shell is launched.</x:v>
@@ -2048,7 +2048,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W17" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X17" s="39" t="str">
         <x:v>Expose retention configuration and current-state independence in Phase 2.</x:v>
@@ -2096,7 +2096,7 @@
         <x:v>cargo test --manifest-path src-tauri/Cargo.toml</x:v>
       </x:c>
       <x:c r="N18" s="39" t="str">
-        <x:v>Nine Rust tests cover transactional persistence, transition history, schema metadata, legacy JSON migration, action audits, and same-second event IDs.</x:v>
+        <x:v>Twenty Rust tests cover transactional persistence, transition history, schema metadata, legacy JSON migration, provider snapshots, local configuration, action audits, AI privacy, release preparation, and same-second event IDs.</x:v>
       </x:c>
       <x:c r="O18" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -2108,16 +2108,16 @@
         <x:v>Yes: SQLite persistence and legacy migration tests.</x:v>
       </x:c>
       <x:c r="T18" s="39" t="str">
-        <x:v>The schema is versioned at v2, explicitly migrates v1, uses separate roots/repositories/expected/events/action_audits tables, and keeps complex snapshot payloads behind the existing Rust contract.</x:v>
+        <x:v>The schema is versioned at v4, explicitly migrates earlier versions, and persists roots, repositories, products, groups, expected state, events, action audits, provider identities, and provider snapshots behind the existing Rust contract.</x:v>
       </x:c>
       <x:c r="U18" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:269-345, 483-522, 535-665; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
+        <x:v>src-tauri/src/core.rs:12-13, 269-345, 483-522, 535-665, 680-783; /Users/jakyeamos/Downloads/pronto_prd.md:936-954</x:v>
       </x:c>
       <x:c r="V18" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="W18" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X18" s="39" t="str">
         <x:v>Verify crash recovery on the target desktop runtime before introducing provider data or a modifying action contract.</x:v>
@@ -2193,7 +2193,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X19" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y19" s="39" t="str">
         <x:v>Run a human visual pass in the Tauri window and record screenshots/interaction outcomes.</x:v>
@@ -2268,7 +2268,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X20" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y20" s="39" t="str">
         <x:v>Verify evidence drawer content, expected-state action, and close behavior manually.</x:v>
@@ -2294,19 +2294,19 @@
         <x:v>No provider auth</x:v>
       </x:c>
       <x:c r="G21" s="39" t="str">
-        <x:v>Provider/release data unavailable</x:v>
+        <x:v>Provider, release, process, or AI data may be unavailable or permission-limited</x:v>
       </x:c>
       <x:c r="H21" s="39" t="str">
         <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I21" s="39" t="str">
-        <x:v>The renderer labels provider refresh, remote catalog, PR, release, process, and AI capabilities as unavailable/deferred.</x:v>
+        <x:v>The renderer labels GitHub refresh, remote catalog, PR/release evidence, process uncertainty, AI permission, and non-implemented mutations with explicit status/copy.</x:v>
       </x:c>
       <x:c r="J21" s="39" t="str">
-        <x:v>Missing permission or unimplemented capability is explicit and never silently inferred as healthy.</x:v>
+        <x:v>Missing permission, stale provider data, or an intentionally preview-only capability is explicit and never silently inferred as healthy.</x:v>
       </x:c>
       <x:c r="K21" s="39" t="str">
-        <x:v>src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:151-159, 304-306, 605-607, 1121-1133</x:v>
+        <x:v>src/renderer/src/App.tsx:180-309, 432-466; src/renderer/src/components/RemoteCatalogSurface.tsx; src/renderer/src/components/AiSummaryPreview.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:151-159, 304-306, 605-607, 1121-1133</x:v>
       </x:c>
       <x:c r="L21" s="39" t="str">
         <x:v>Build + source review</x:v>
@@ -2315,7 +2315,7 @@
         <x:v>pnpm build:web; pnpm build</x:v>
       </x:c>
       <x:c r="N21" s="39" t="str">
-        <x:v>Unavailable boundary is compiled into the app; provider-backed runtime is intentionally not claimed.</x:v>
+        <x:v>The app exposes a read-only GitHub provider boundary when authenticated and preserves unavailable/deferred states for missing credentials, mutations, publication, and AI requests.</x:v>
       </x:c>
       <x:c r="O21" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -2328,13 +2328,13 @@
         <x:v>Provider credentials and network authority are not available or requested for this slice.</x:v>
       </x:c>
       <x:c r="S21" s="39" t="str">
-        <x:v>UI states are explicit and kept outside local scan truth.</x:v>
+        <x:v>UI states are explicit and kept outside local scan truth; provider snapshots retain fetched-at evidence.</x:v>
       </x:c>
       <x:c r="T21" s="39" t="str">
         <x:v>No; boundary is represented by source and build.</x:v>
       </x:c>
       <x:c r="U21" s="39" t="str">
-        <x:v>No provider adapter abstraction is added until its permission contract is defined.</x:v>
+        <x:v>Provider adapter and local payload preview contracts are explicit; mutation and external AI contracts remain closed.</x:v>
       </x:c>
       <x:c r="V21" s="39" t="str">
         <x:v>docs/implementation-plan.md; /Users/jakyeamos/Downloads/pronto_prd.md:304-306, 1121-1133</x:v>
@@ -2343,10 +2343,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X21" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y21" s="39" t="str">
-        <x:v>Provider install/auth and refresh evidence are Phase 2 work.</x:v>
+        <x:v>Live authenticated refresh and desktop interaction remain environment checks; provider mutations and external AI execution remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="70" customHeight="1">
@@ -2418,7 +2418,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X22" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y22" s="39" t="str">
         <x:v>Verify active navigation, deferred copy, and Activity/Settings content manually.</x:v>
@@ -2493,7 +2493,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X23" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y23" s="39" t="str">
         <x:v>Verify search focus, Escape dismissal, and focus behavior manually.</x:v>
@@ -2525,13 +2525,13 @@
         <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I24" s="39" t="str">
-        <x:v>Settings shows local roots, storage location, freshness, and privacy; Activity shows safe local action audits, transition events, or a truthful empty state.</x:v>
+        <x:v>Settings shows local roots, storage location, freshness, privacy, ignore policy, refresh policy, background monitoring, and bounded retention; Activity shows safe local action audits, transition events, or a truthful empty state.</x:v>
       </x:c>
       <x:c r="J24" s="39" t="str">
-        <x:v>Local configuration and history are understandable without a server account or provider refresh.</x:v>
+        <x:v>Local configuration and history are understandable without a server account or provider refresh, and retention changes stay local and bounded.</x:v>
       </x:c>
       <x:c r="K24" s="39" t="str">
-        <x:v>src/renderer/src/components/WorkspaceSurfaces.tsx; src/renderer/src/App.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:699-717, 859-900</x:v>
+        <x:v>src/renderer/src/components/WorkspaceSurfaces.tsx; src/renderer/src/App.tsx; src-tauri/src/core.rs:5058-5068; /Users/jakyeamos/Downloads/pronto_prd.md:699-717, 859-900</x:v>
       </x:c>
       <x:c r="L24" s="39" t="str">
         <x:v>Typecheck/build + live desktop review</x:v>
@@ -2540,7 +2540,7 @@
         <x:v>pnpm typecheck; pnpm build:web; open Settings and Activity in the Tauri window</x:v>
       </x:c>
       <x:c r="N24" s="39" t="str">
-        <x:v>Surface content is wired to the local snapshot contract, including bounded action-audit rows, and builds successfully; live rendering remains environment verification.</x:v>
+        <x:v>Surface content is wired to the local snapshot contract, including bounded action-audit rows and configurable retention, and builds successfully; live rendering remains environment verification.</x:v>
       </x:c>
       <x:c r="O24" s="39" t="str">
         <x:v>Needs-Environment</x:v>
@@ -2568,7 +2568,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X24" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y24" s="39" t="str">
         <x:v>Verify roots, storage path, freshness, privacy, event rows, and empty state manually.</x:v>
@@ -2643,7 +2643,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X25" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y25" s="39" t="str">
         <x:v>Verify no-data, no-match, and Clear filters states manually.</x:v>
@@ -2711,7 +2711,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W26" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X26" s="39" t="str">
         <x:v>Implement desktop focus behavior for `pronto .` when the app lifecycle is available.</x:v>
@@ -2780,7 +2780,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X27" s="39" t="str">
         <x:v>Package installation and `pronto .` focus behavior remain to be verified.</x:v>
@@ -2849,7 +2849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W28" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X28" s="39" t="str">
         <x:v>Code signing/notarization is outside this local implementation.</x:v>
@@ -2918,7 +2918,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="X29" s="39" t="str">
         <x:v>Add action-tier audit tests only when modifying actions are authorized and implemented.</x:v>
@@ -2936,7 +2936,7 @@
         <x:v>GitHub identities / refresh</x:v>
       </x:c>
       <x:c r="D30" s="39" t="str">
-        <x:v>As an operator, I can connect multiple identities and see permission degradation explicitly.</x:v>
+        <x:v>As an operator, I can refresh a read-only GitHub identity and repository snapshot and see unavailable authentication explicitly.</x:v>
       </x:c>
       <x:c r="E30" s="39" t="str">
         <x:v>Provider-connected operator</x:v>
@@ -2951,53 +2951,53 @@
         <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I30" s="39" t="str">
-        <x:v>No provider adapter is enabled in this slice; the app does not claim GitHub identity, refresh, or permission results.</x:v>
+        <x:v>The GitHub CLI adapter reads the authenticated user, paginated repositories, pull requests, and releases; refresh persists sanitized snapshots and changes to Unavailable without destroying the last known snapshot when auth is missing.</x:v>
       </x:c>
       <x:c r="J30" s="39" t="str">
-        <x:v>No provider state is shown as current until identity and permission evidence exist.</x:v>
+        <x:v>A read-only provider refresh can explain identity, locality, freshness, and unavailable credentials without claiming clone, write, or merge authority.</x:v>
       </x:c>
       <x:c r="K30" s="39" t="str">
-        <x:v>docs/implementation-plan.md:19-24; /Users/jakyeamos/Downloads/pronto_prd.md:296-306, 974-987</x:v>
+        <x:v>src-tauri/src/core.rs:1355-1464, 1676-1765, 6400-6539; src/renderer/src/components/RemoteCatalogSurface.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:296-306, 974-987</x:v>
       </x:c>
       <x:c r="L30" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust parser/provider refresh regression + source review + authenticated desktop check</x:v>
       </x:c>
       <x:c r="M30" s="39" t="str">
-        <x:v>Deferred: requires explicit provider authority and credentials</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; click Remote catalog → Refresh GitHub</x:v>
       </x:c>
       <x:c r="N30" s="39" t="str">
-        <x:v>Provider identity, credential separation, and permission degradation are not implemented.</x:v>
+        <x:v>Provider parsing, local/remote matching, persistence, and unavailable-state transitions are regression-covered; live refresh requires an authenticated gh environment.</x:v>
       </x:c>
       <x:c r="O30" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P30" s="39" t="str"/>
       <x:c r="Q30" s="39" t="str">
-        <x:v>Dependency</x:v>
+        <x:v>Environment</x:v>
       </x:c>
       <x:c r="R30" s="39" t="str">
-        <x:v>Requires network, provider auth, OS credential store, and a durable identity mapping.</x:v>
+        <x:v>The repository uses the existing gh credential path; live auth and permission scope cannot be proven by offline fixtures.</x:v>
       </x:c>
       <x:c r="S30" s="39" t="str">
-        <x:v>Kept as an explicit deferred boundary; no fake adapter or mock provider result is added.</x:v>
+        <x:v>Implemented a provider-neutral refresh contract with GitHub CLI adapter, sanitized identity/repository snapshots, explicit unavailable state, and no provider mutations.</x:v>
       </x:c>
       <x:c r="T30" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: parser and provider-refresh fixture assertions.</x:v>
       </x:c>
       <x:c r="U30" s="39" t="str">
-        <x:v>Provider work is separated from local Git evidence by design.</x:v>
+        <x:v>Provider state remains a timestamped snapshot and never overwrites local Git truth.</x:v>
       </x:c>
       <x:c r="V30" s="39" t="str">
-        <x:v>pronto_prd.md:296-306, 974-987; docs/implementation-plan.md:49-54</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:296-306, 974-987; src-tauri/src/core.rs:1355-1765</x:v>
       </x:c>
       <x:c r="W30" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X30" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y30" s="39" t="str">
-        <x:v>Define provider permission and freshness contracts before implementation.</x:v>
+        <x:v>Multiple-provider identity selection and richer organization permissions remain outside this read-only GitHub adapter.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="70" customHeight="1">
@@ -3011,7 +3011,7 @@
         <x:v>Remote-only / clone</x:v>
       </x:c>
       <x:c r="D31" s="39" t="str">
-        <x:v>As an operator, I can import or clone a remote-only repository into a selected root.</x:v>
+        <x:v>As an operator, I can inspect a remote-only GitHub repository and see whether it matches a local checkout.</x:v>
       </x:c>
       <x:c r="E31" s="39" t="str">
         <x:v>Provider-connected operator</x:v>
@@ -3020,59 +3020,59 @@
         <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G31" s="39" t="str">
-        <x:v>Remote repository catalog and clone permission</x:v>
+        <x:v>Read-only GitHub repository snapshot</x:v>
       </x:c>
       <x:c r="H31" s="39" t="str">
         <x:v>Desktop + network</x:v>
       </x:c>
       <x:c r="I31" s="39" t="str">
-        <x:v>Remote catalog and clone are not exposed by the local-first slice.</x:v>
+        <x:v>The read-only Remote catalog persists remote-only and local-and-remote labels, default branch, archive state, URL, identity, and refresh time; clone remains absent.</x:v>
       </x:c>
       <x:c r="J31" s="39" t="str">
-        <x:v>A remote repository is not represented as local until clone succeeds and the local scan registers it.</x:v>
+        <x:v>A remote repository is not represented as local until a separately authorized clone succeeds and a local scan registers it.</x:v>
       </x:c>
       <x:c r="K31" s="39" t="str">
-        <x:v>docs/implementation-plan.md:49-54; /Users/jakyeamos/Downloads/pronto_prd.md:280-286, 849-857</x:v>
+        <x:v>src-tauri/src/core.rs:1466-1656, 1676-1743, 6400-6539; src/renderer/src/components/RemoteCatalogSurface.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:280-286, 849-857</x:v>
       </x:c>
       <x:c r="L31" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust parser/provider fixture + renderer build + authenticated desktop check</x:v>
       </x:c>
       <x:c r="M31" s="39" t="str">
-        <x:v>Deferred: requires provider auth, network, clone preflight, and selected root</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; open Remote catalog</x:v>
       </x:c>
       <x:c r="N31" s="39" t="str">
-        <x:v>No remote-only or clone path is implemented.</x:v>
+        <x:v>Remote-only parsing and local/remote matching are regression-covered; live catalog refresh requires authenticated gh; no clone command is exposed.</x:v>
       </x:c>
       <x:c r="O31" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P31" s="39" t="str"/>
       <x:c r="Q31" s="39" t="str">
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R31" s="39" t="str">
-        <x:v>Requires network and exact destination authorization.</x:v>
+        <x:v>Clone still requires network, exact destination authorization, fresh preflight, and post-scan audit.</x:v>
       </x:c>
       <x:c r="S31" s="39" t="str">
-        <x:v>Deferred explicitly rather than pretending provider access exists.</x:v>
+        <x:v>Implemented the read-only remote catalog and kept clone explicitly outside the allowed action surface.</x:v>
       </x:c>
       <x:c r="T31" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: remote parser and local-match assertions.</x:v>
       </x:c>
       <x:c r="U31" s="39" t="str">
-        <x:v>Clone is a modifying action and must arrive with fresh preflight/audit contracts.</x:v>
+        <x:v>Remote state is a provider snapshot and cannot imply a local working copy.</x:v>
       </x:c>
       <x:c r="V31" s="39" t="str">
-        <x:v>pronto_prd.md:280-286, 849-857</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:280-286, 849-857; src-tauri/src/core.rs:1676-1743</x:v>
       </x:c>
       <x:c r="W31" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X31" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y31" s="39" t="str">
-        <x:v>Define clone destination and audit semantics before adding the action.</x:v>
+        <x:v>Define clone destination and audit semantics before adding the modifying action.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="70" customHeight="1">
@@ -3144,7 +3144,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="X32" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y32" s="39" t="str">
         <x:v>Phase 2 must add destination-specific permission and post-action verification before any modifying command.</x:v>
@@ -3191,7 +3191,7 @@
         <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; pnpm typecheck; pnpm build:web</x:v>
       </x:c>
       <x:c r="N33" s="39" t="str">
-        <x:v>Nine Rust tests pass, including allowed/rejected preflights, completed refresh audit, schema-v1 migration, and same-second transition persistence; Activity renders audit rows.</x:v>
+        <x:v>Twenty Rust tests pass, including allowed/rejected preflights, completed scoped refresh audits, schema migration, provider snapshots, local configuration, AI privacy, release preparation, and same-second transition persistence; Activity renders audit rows.</x:v>
       </x:c>
       <x:c r="O33" s="39" t="str">
         <x:v>Regression-Covered</x:v>
@@ -3200,7 +3200,7 @@
       <x:c r="Q33" s="39" t="str"/>
       <x:c r="R33" s="39" t="str"/>
       <x:c r="S33" s="39" t="str">
-        <x:v>Yes: preflight, rejected-action, completed-refresh, migration, and collision regression tests.</x:v>
+        <x:v>Yes: preflight, rejected-action, completed-refresh, scoped-target, migration, provider, AI, release, and collision regression tests.</x:v>
       </x:c>
       <x:c r="T33" s="39" t="str">
         <x:v>Explicit allowlist and one persistence path keep action policy out of display components; modifying operations remain absent.</x:v>
@@ -3209,13 +3209,13 @@
         <x:v>Yes: native Rust regression coverage.</x:v>
       </x:c>
       <x:c r="V33" s="39" t="str">
-        <x:v>b13de08 source/test output</x:v>
+        <x:v>c0bf758 source/test output</x:v>
       </x:c>
       <x:c r="W33" s="39" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="X33" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y33" s="39" t="str">
         <x:v>Read-only inspect is preflight-only; add modifying actions only with destination-specific permission and post-action verification.</x:v>
@@ -3223,447 +3223,522 @@
     </x:row>
     <x:row r="34" ht="70" customHeight="1">
       <x:c r="A34" s="51" t="str">
-        <x:v>PR-001</x:v>
+        <x:v>HANDOFF-001</x:v>
       </x:c>
       <x:c r="B34" s="39" t="str">
-        <x:v>Pull requests</x:v>
+        <x:v>Workspace handoff</x:v>
       </x:c>
       <x:c r="C34" s="39" t="str">
-        <x:v>Provider lifecycle</x:v>
+        <x:v>Exact workspace / external tools</x:v>
       </x:c>
       <x:c r="D34" s="39" t="str">
-        <x:v>As an operator, I can create or merge a PR only when provider facts and permissions are verifiable.</x:v>
+        <x:v>As an operator, I can open the exact registered workspace in Finder, Terminal, Visual Studio Code, or GitHub Desktop without changing repository state.</x:v>
       </x:c>
       <x:c r="E34" s="39" t="str">
-        <x:v>Provider-connected operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F34" s="39" t="str">
-        <x:v>Provider auth required</x:v>
+        <x:v>macOS local-only</x:v>
       </x:c>
       <x:c r="G34" s="39" t="str">
-        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
+        <x:v>Registered repository and exact workspace ID</x:v>
       </x:c>
       <x:c r="H34" s="39" t="str">
-        <x:v>Desktop + provider API</x:v>
+        <x:v>Desktop + macOS</x:v>
       </x:c>
       <x:c r="I34" s="39" t="str">
-        <x:v>PR creation, review evidence, and merge actions are explicit deferred boundaries.</x:v>
+        <x:v>The handoff command validates repository and workspace identity, accepts only fixed supported tools, and invokes structured macOS open arguments without staging, committing, or mutating registry state.</x:v>
       </x:c>
       <x:c r="J34" s="39" t="str">
-        <x:v>Unknown checks or reviews never become a merge-eligible state.</x:v>
+        <x:v>A handoff opens the intended workspace and rejects unknown targets/tools clearly; it never becomes a hidden Git action.</x:v>
       </x:c>
       <x:c r="K34" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>src-tauri/src/core.rs:5247-5290, 6000-6068; src/renderer/src/components/Drawers.tsx:142-169; /Users/jakyeamos/Downloads/pronto_prd.md:469-487</x:v>
       </x:c>
       <x:c r="L34" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust target/tool regression + desktop interaction check</x:v>
       </x:c>
       <x:c r="M34" s="39" t="str">
-        <x:v>Deferred: provider permission and PR API required</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; open a repository drawer and choose a workspace tool</x:v>
       </x:c>
       <x:c r="N34" s="39" t="str">
-        <x:v>No PR lifecycle implementation is present.</x:v>
+        <x:v>Unknown workspace and unsupported tool are rejected by regression tests; successful macOS launch still requires a live desktop pass.</x:v>
       </x:c>
       <x:c r="O34" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P34" s="39" t="str"/>
       <x:c r="Q34" s="39" t="str">
-        <x:v>Dependency</x:v>
+        <x:v>Environment</x:v>
       </x:c>
       <x:c r="R34" s="39" t="str">
-        <x:v>Requires provider adapter, permission degradation, and action audit.</x:v>
+        <x:v>The local test suite cannot prove Finder, Terminal, VS Code, or GitHub Desktop availability and focus behavior.</x:v>
       </x:c>
       <x:c r="S34" s="39" t="str">
-        <x:v>Deferred with explicit unknown/unavailable semantics.</x:v>
+        <x:v>Added exact workspace lookup, fixed tool allowlist, structured `/usr/bin/open` argument construction, and no registry mutation.</x:v>
       </x:c>
       <x:c r="T34" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: unknown-workspace and unsupported-tool assertions.</x:v>
       </x:c>
       <x:c r="U34" s="39" t="str">
-        <x:v>PR work depends on provider state and cannot be safely inferred from local Git alone.</x:v>
+        <x:v>The target boundary is validated before launch; no arbitrary application or shell string is accepted.</x:v>
       </x:c>
       <x:c r="V34" s="39" t="str">
-        <x:v>pronto_prd.md:555-571, 1185-1189</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:469-487; src-tauri/src/core.rs:5247-5290</x:v>
       </x:c>
       <x:c r="W34" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X34" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y34" s="39" t="str">
-        <x:v>Add provider-backed evidence before adding any merge control.</x:v>
+        <x:v>Verify one successful launch per installed tool on macOS; keep non-macOS mappings deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="70" customHeight="1">
       <x:c r="A35" s="51" t="str">
-        <x:v>REL-001</x:v>
+        <x:v>PR-001</x:v>
       </x:c>
       <x:c r="B35" s="39" t="str">
-        <x:v>Releases</x:v>
+        <x:v>Pull requests</x:v>
       </x:c>
       <x:c r="C35" s="39" t="str">
-        <x:v>Release preparation</x:v>
+        <x:v>Read-only PR evidence</x:v>
       </x:c>
       <x:c r="D35" s="39" t="str">
-        <x:v>As an operator, I can prepare a deterministic release draft without publishing it automatically.</x:v>
+        <x:v>As an operator, I can inspect a matching pull request and see checks, reviews, draft state, mergeability, and freshness without creating or merging it.</x:v>
       </x:c>
       <x:c r="E35" s="39" t="str">
-        <x:v>Release maintainer</x:v>
+        <x:v>Provider-connected operator</x:v>
       </x:c>
       <x:c r="F35" s="39" t="str">
         <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G35" s="39" t="str">
-        <x:v>Published release baseline, configured rule, clean isolated worktree</x:v>
+        <x:v>Known head/base, checks, reviews, and provider identity</x:v>
       </x:c>
       <x:c r="H35" s="39" t="str">
         <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I35" s="39" t="str">
-        <x:v>Release baseline, deterministic rules, isolated worktrees, and draft handoff are deferred.</x:v>
+        <x:v>Preparation matches provider PR snapshots to the selected workspace and preserves unknown checks, reviews, and mergeability; the UI exposes evidence without write controls.</x:v>
       </x:c>
       <x:c r="J35" s="39" t="str">
-        <x:v>No release threshold or version recommendation appears until its configured evidence exists.</x:v>
+        <x:v>Unknown checks or reviews never become a merge-eligible state, and a preview cannot create or merge a PR.</x:v>
       </x:c>
       <x:c r="K35" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>src-tauri/src/core.rs:3374-3465, 6100-6185; src/renderer/src/components/PreparationDrawer.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189</x:v>
       </x:c>
       <x:c r="L35" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust preparation regression + renderer build + authenticated desktop check</x:v>
       </x:c>
       <x:c r="M35" s="39" t="str">
-        <x:v>Deferred: provider, release recipe, and isolated worktree gates required</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; open repository preparation</x:v>
       </x:c>
       <x:c r="N35" s="39" t="str">
-        <x:v>No release preparation or publication path is implemented.</x:v>
+        <x:v>Fixture asserts matching PR number, base branch, commit count, pending checks, and unknown provider detail; live provider refresh remains environment-limited.</x:v>
       </x:c>
       <x:c r="O35" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P35" s="39" t="str"/>
       <x:c r="Q35" s="39" t="str">
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R35" s="39" t="str">
-        <x:v>Requires exact diff review, validation gates, and publication boundary.</x:v>
+        <x:v>Create/merge still require provider write permissions, fresh preflight, exact-target audit, and post-action verification.</x:v>
       </x:c>
       <x:c r="S35" s="39" t="str">
-        <x:v>Phase 3 plan preserves the no-publish rule.</x:v>
+        <x:v>Implemented read-only PR evidence and kept PR creation, approval, and merge outside the action surface.</x:v>
       </x:c>
       <x:c r="T35" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: deterministic preparation fixture.</x:v>
       </x:c>
       <x:c r="U35" s="39" t="str">
-        <x:v>Release automation is intentionally not inferred from local commit counts.</x:v>
+        <x:v>Provider evidence is additive; local branch and dirty state remain independently visible.</x:v>
       </x:c>
       <x:c r="V35" s="39" t="str">
-        <x:v>pronto_prd.md:575-655, 1191-1203</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:555-571, 1185-1189; src-tauri/src/core.rs:3374-3465</x:v>
       </x:c>
       <x:c r="W35" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X35" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y35" s="39" t="str">
-        <x:v>Define recipe state and audit events before implementation.</x:v>
+        <x:v>Add provider-backed write permissions and post-action verification before any PR mutation.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="70" customHeight="1">
       <x:c r="A36" s="51" t="str">
-        <x:v>PROC-001</x:v>
+        <x:v>REL-001</x:v>
       </x:c>
       <x:c r="B36" s="39" t="str">
-        <x:v>Agent workspaces</x:v>
+        <x:v>Releases</x:v>
       </x:c>
       <x:c r="C36" s="39" t="str">
-        <x:v>Process / terminal evidence</x:v>
+        <x:v>Release preparation</x:v>
       </x:c>
       <x:c r="D36" s="39" t="str">
-        <x:v>As an operator, I can tell whether an agent workspace has process evidence without exposing terminal contents.</x:v>
+        <x:v>As an operator, I can inspect a deterministic release candidate, threshold trace, notes, recipe, and version confirmation without executing or publishing it.</x:v>
       </x:c>
       <x:c r="E36" s="39" t="str">
-        <x:v>Local operator</x:v>
+        <x:v>Release maintainer</x:v>
       </x:c>
       <x:c r="F36" s="39" t="str">
-        <x:v>Local permission required</x:v>
+        <x:v>Provider auth required</x:v>
       </x:c>
       <x:c r="G36" s="39" t="str">
-        <x:v>OS process inspection permission and optional manifest</x:v>
+        <x:v>Published release baseline, configured rule, clean workspace, and explicit recipe/version confirmation</x:v>
       </x:c>
       <x:c r="H36" s="39" t="str">
-        <x:v>Desktop + native adapters</x:v>
+        <x:v>Desktop + provider API</x:v>
       </x:c>
       <x:c r="I36" s="39" t="str">
-        <x:v>Process, terminal, and generic agent adapters are deferred; no certainty is claimed from their absence.</x:v>
+        <x:v>Preparation shows published baseline, semantic bump, categorized commits, exact rule trace, the `Configured release threshold met` queue condition when provider context is ready, validated recipe metadata, and a nine-step preview whose actions_performed flag remains false.</x:v>
       </x:c>
       <x:c r="J36" s="39" t="str">
-        <x:v>Unknown process evidence remains unknown rather than being classified as inactive or safe to clean.</x:v>
+        <x:v>A release candidate is explainable and requires explicit version confirmation; no worktree, script, generated file, commit, push, PR, or release publication occurs from preview.</x:v>
       </x:c>
       <x:c r="K36" s="39" t="str">
-        <x:v>docs/implementation-plan.md:51-54; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
+        <x:v>src-tauri/src/core.rs:3110-3369, 3871-4015, 4935-5036, 6179-6291; src/renderer/src/components/PreparationDrawer.tsx; src/renderer/src/components/ReleaseRecipePanel.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203</x:v>
       </x:c>
       <x:c r="L36" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust deterministic preparation regression + renderer build + authenticated desktop check</x:v>
       </x:c>
       <x:c r="M36" s="39" t="str">
-        <x:v>Deferred: OS adapter and permission boundary required</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; configure rule/recipe/version in repository preparation</x:v>
       </x:c>
       <x:c r="N36" s="39" t="str">
-        <x:v>No process or terminal capture is implemented.</x:v>
+        <x:v>Fixture asserts baseline, major candidate, three rule traces, threshold queue condition, stale-version rejection, unsafe recipe rejection, confirmed version, nine steps, and actions_performed=false.</x:v>
       </x:c>
       <x:c r="O36" s="39" t="str">
-        <x:v>Needs-Environment</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P36" s="39" t="str"/>
       <x:c r="Q36" s="39" t="str">
         <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R36" s="39" t="str">
-        <x:v>Cross-platform process APIs and privacy review are required.</x:v>
+        <x:v>Executing the configured recipe still requires a separate worktree/command runner, exact generated-file diff review, commit/push/PR permissions, and release publication authorization.</x:v>
       </x:c>
       <x:c r="S36" s="39" t="str">
-        <x:v>The current slice only models linked worktrees as local workspaces.</x:v>
+        <x:v>Implemented deterministic local release intelligence and safe preparation preview while preserving every external or modifying step as a visible blocked boundary.</x:v>
       </x:c>
       <x:c r="T36" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: release rule, threshold, recipe validation, version confirmation, and preparation regression assertions.</x:v>
       </x:c>
       <x:c r="U36" s="39" t="str">
-        <x:v>Never capture terminal contents, prompts, source text, or keystrokes.</x:v>
+        <x:v>No release automation is inferred from local commit counts; provider freshness and recipe execution remain explicit.</x:v>
       </x:c>
       <x:c r="V36" s="39" t="str">
-        <x:v>pronto_prd.md:489-525</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:575-655, 1191-1203; src-tauri/src/core.rs:3110-3465, 3871-4015</x:v>
       </x:c>
       <x:c r="W36" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X36" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y36" s="39" t="str">
-        <x:v>Add provider-neutral adapters and confidence language in Phase 2.</x:v>
+        <x:v>Define execution audit events and destination-specific publication permissions before enabling any recipe step.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="70" customHeight="1">
       <x:c r="A37" s="51" t="str">
-        <x:v>GROUP-001</x:v>
+        <x:v>PROC-001</x:v>
       </x:c>
       <x:c r="B37" s="39" t="str">
-        <x:v>Products</x:v>
+        <x:v>Agent workspaces</x:v>
       </x:c>
       <x:c r="C37" s="39" t="str">
-        <x:v>Products / groups</x:v>
+        <x:v>Process / terminal evidence</x:v>
       </x:c>
       <x:c r="D37" s="39" t="str">
-        <x:v>As an operator, I can aggregate multiple repositories without hiding repository-level evidence.</x:v>
+        <x:v>As an operator, I can tell whether an agent workspace has process or manifest evidence without exposing terminal contents.</x:v>
       </x:c>
       <x:c r="E37" s="39" t="str">
-        <x:v>Portfolio operator</x:v>
+        <x:v>Local operator</x:v>
       </x:c>
       <x:c r="F37" s="39" t="str">
-        <x:v>Local-only or provider auth</x:v>
+        <x:v>Local permission required</x:v>
       </x:c>
       <x:c r="G37" s="39" t="str">
-        <x:v>Product/group configuration and participating repositories</x:v>
+        <x:v>Linked workspace, optional safe `.pronto/agent.json`, and OS process inspection permission</x:v>
       </x:c>
       <x:c r="H37" s="39" t="str">
-        <x:v>Desktop 1280×800</x:v>
+        <x:v>Desktop + native adapters</x:v>
       </x:c>
       <x:c r="I37" s="39" t="str">
-        <x:v>Products, groups, and coordinated release are deferred; the current portfolio remains repository-first.</x:v>
+        <x:v>Workspace activity combines safe manifest metadata and candidate-process working-directory evidence; unsupported or permission-limited inspection yields `Activity state uncertain` rather than inactive.</x:v>
       </x:c>
       <x:c r="J37" s="39" t="str">
-        <x:v>No aggregate product status is shown until its repository-level provenance and release policy are defined.</x:v>
+        <x:v>Unknown process evidence remains unknown, while active manifest/process signals block integration eligibility; terminal contents, prompts, keystrokes, and source text are never captured.</x:v>
       </x:c>
       <x:c r="K37" s="39" t="str">
-        <x:v>docs/implementation-plan.md:56-60; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>src-tauri/src/core.rs:216-291, 2475-2815, 5959-5982; src/renderer/src/components/Drawers.tsx:116-142; /Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171</x:v>
       </x:c>
       <x:c r="L37" s="39" t="str">
-        <x:v>Boundary review</x:v>
+        <x:v>Rust manifest/activity regression + source review + desktop check</x:v>
       </x:c>
       <x:c r="M37" s="39" t="str">
-        <x:v>Deferred: product model and coordination policy required</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; open a repository workspace with `.pronto/agent.json`</x:v>
       </x:c>
       <x:c r="N37" s="39" t="str">
-        <x:v>No product/group mutation or coordinated release logic is implemented.</x:v>
+        <x:v>Manifest fixture yields Active/High confidence, target evidence, and no terminal content; process correlation remains platform/permission-sensitive.</x:v>
       </x:c>
       <x:c r="O37" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P37" s="39" t="str"/>
       <x:c r="Q37" s="39" t="str">
-        <x:v>Product</x:v>
+        <x:v>Dependency</x:v>
       </x:c>
       <x:c r="R37" s="39" t="str">
-        <x:v>Manual product/group configuration is accepted; implementation still needs the durable state and coordination model.</x:v>
+        <x:v>Cross-platform process APIs and OS permission can still make the activity state uncertain.</x:v>
       </x:c>
       <x:c r="S37" s="39" t="str">
-        <x:v>Repository-first UI avoids a premature inferred aggregate abstraction.</x:v>
+        <x:v>Added safe manifest parsing, platform-specific process working-directory probes, explicit confidence language, and integration blocking for active workspaces.</x:v>
       </x:c>
       <x:c r="T37" s="39" t="str">
-        <x:v>No.</x:v>
+        <x:v>Yes: manifest parsing, privacy, and active-workspace integration-blocking assertions.</x:v>
       </x:c>
       <x:c r="U37" s="39" t="str">
-        <x:v>This is an accepted delivery boundary, not an unresolved product decision.</x:v>
+        <x:v>Activity is evidence, not a cleanup authorization; no terminal capture is introduced.</x:v>
       </x:c>
       <x:c r="V37" s="39" t="str">
-        <x:v>pronto_prd.md:227-238, 659-677</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:489-525, 1165-1171; src-tauri/src/core.rs:2475-2815</x:v>
       </x:c>
       <x:c r="W37" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X37" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y37" s="39" t="str">
-        <x:v>Implement manual product/group configuration after the SQLite contract is stable.</x:v>
+        <x:v>Add more agent manifest schemas only after preserving the same safe-field and uncertainty contract.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
       <x:c r="A38" s="51" t="str">
-        <x:v>AI-001</x:v>
+        <x:v>GROUP-001</x:v>
       </x:c>
       <x:c r="B38" s="39" t="str">
-        <x:v>AI and privacy</x:v>
+        <x:v>Products</x:v>
       </x:c>
       <x:c r="C38" s="39" t="str">
-        <x:v>Privacy boundary</x:v>
+        <x:v>Products / groups</x:v>
       </x:c>
       <x:c r="D38" s="39" t="str">
-        <x:v>As an operator, I can keep AI disabled and prevent uncommitted source from leaving the machine.</x:v>
+        <x:v>As an operator, I can manually configure products and groups with explicit repository membership without hiding repository-level evidence.</x:v>
       </x:c>
       <x:c r="E38" s="39" t="str">
-        <x:v>Privacy-conscious operator</x:v>
+        <x:v>Portfolio operator</x:v>
       </x:c>
       <x:c r="F38" s="39" t="str">
-        <x:v>AI disabled by default</x:v>
+        <x:v>Local-only</x:v>
       </x:c>
       <x:c r="G38" s="39" t="str">
-        <x:v>Explicit provider/model permission and approved payload</x:v>
+        <x:v>Versioned SQLite registry and participating repository IDs</x:v>
       </x:c>
       <x:c r="H38" s="39" t="str">
-        <x:v>Desktop + provider/local model</x:v>
+        <x:v>Desktop 1280×800</x:v>
       </x:c>
       <x:c r="I38" s="39" t="str">
-        <x:v>No AI request path exists in this slice; local snapshots contain metadata and no uncommitted diff content.</x:v>
+        <x:v>Manual product/group create, edit, delete, explicit membership, product release mode, and case-insensitive collection filtering persist locally and remain repository-first.</x:v>
       </x:c>
       <x:c r="J38" s="39" t="str">
-        <x:v>No AI claim or payload is possible until the user opts in and reviews the exact payload categories.</x:v>
+        <x:v>No aggregate product health or coordinated release status is inferred; membership and release policy remain visible configuration.</x:v>
       </x:c>
       <x:c r="K38" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:32-188; src/renderer/src/App.tsx:180-309; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>src-tauri/src/core.rs:44-80, 686-710, 5081-5174, 6865-6963; src/renderer/src/components/PortfolioConfigSurface.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677</x:v>
       </x:c>
       <x:c r="L38" s="39" t="str">
-        <x:v>Static safety review + privacy regression</x:v>
+        <x:v>Rust configuration regression + renderer build + desktop interaction check</x:v>
       </x:c>
       <x:c r="M38" s="39" t="str">
-        <x:v>rg 'diff|filename|content' src-tauri/src/core.rs src/renderer/src; cargo test --manifest-path src-tauri/Cargo.toml</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; open Products/Groups and save a manual configuration</x:v>
       </x:c>
       <x:c r="N38" s="39" t="str">
-        <x:v>No external AI call is implemented; snapshot privacy test passes and UI states the local/private boundary.</x:v>
+        <x:v>Fixture persists product/group membership, release mode, filtering, targeted refresh, and deletion; live form interaction remains an environment check.</x:v>
       </x:c>
       <x:c r="O38" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P38" s="39" t="str"/>
       <x:c r="Q38" s="39" t="str">
         <x:v>Product</x:v>
       </x:c>
       <x:c r="R38" s="39" t="str">
-        <x:v>AI remains disabled by the accepted product direction; payload categories and provider permissions are outside this slice.</x:v>
+        <x:v>Coordinated release, aggregate health, and inferred group membership remain intentionally absent.</x:v>
       </x:c>
       <x:c r="S38" s="39" t="str">
-        <x:v>Deferred AI authority; local metadata-only evidence remains available.</x:v>
+        <x:v>Implemented manual durable product/group configuration and repository-scoped targeting without inventing aggregate health.</x:v>
       </x:c>
       <x:c r="T38" s="39" t="str">
-        <x:v>Yes: snapshot excludes source/diff content.</x:v>
+        <x:v>Yes: product/group/lifecycle/retention persistence regression.</x:v>
       </x:c>
       <x:c r="U38" s="39" t="str">
-        <x:v>AI is not introduced as a shortcut for missing provider evidence.</x:v>
+        <x:v>The accepted manual direction is now implemented; coordinated release remains a separate design and authority gate.</x:v>
       </x:c>
       <x:c r="V38" s="39" t="str">
-        <x:v>pronto_prd.md:679-695, 1205-1211</x:v>
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:227-238, 659-677; src-tauri/src/core.rs:5081-5174</x:v>
       </x:c>
       <x:c r="W38" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="X38" s="39" t="str">
-        <x:v>b13de08</x:v>
+        <x:v>c0bf758</x:v>
       </x:c>
       <x:c r="Y38" s="39" t="str">
-        <x:v>Keep AI disabled until per-repository permissions and payload preview are explicitly designed.</x:v>
+        <x:v>Define coordinated-release semantics before adding any aggregate mutation or publication control.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="70" customHeight="1">
       <x:c r="A39" s="51" t="str">
-        <x:v>HIST-001</x:v>
+        <x:v>AI-001</x:v>
       </x:c>
       <x:c r="B39" s="39" t="str">
-        <x:v>History</x:v>
+        <x:v>AI and privacy</x:v>
       </x:c>
       <x:c r="C39" s="39" t="str">
-        <x:v>Event retention</x:v>
+        <x:v>Privacy boundary</x:v>
       </x:c>
       <x:c r="D39" s="39" t="str">
-        <x:v>As an operator, I can retain bounded transition history without losing current state.</x:v>
+        <x:v>As an operator, I can keep AI disabled or preview an explicitly permitted committed metadata/diff payload before any request.</x:v>
       </x:c>
       <x:c r="E39" s="39" t="str">
-        <x:v>Local operator</x:v>
+        <x:v>Privacy-conscious operator</x:v>
       </x:c>
       <x:c r="F39" s="39" t="str">
-        <x:v>Local-only</x:v>
+        <x:v>AI disabled by default; per-repository permission required for preview</x:v>
       </x:c>
       <x:c r="G39" s="39" t="str">
-        <x:v>Transition events persisted in local store</x:v>
+        <x:v>Explicit repository permission and committed baseline/head</x:v>
       </x:c>
       <x:c r="H39" s="39" t="str">
-        <x:v>Native core</x:v>
+        <x:v>Desktop + provider/local model</x:v>
       </x:c>
       <x:c r="I39" s="39" t="str">
-        <x:v>Events are transition-only with sequence-safe IDs, retained for a default bounded window, and action audits are bounded and pruned independently of current snapshots.</x:v>
+        <x:v>Repository policy supports Disabled, Commit metadata only, and Committed diff allowed; the local preview reports categories, bytes, source references, provider/model trace fields, reasons, and request_performed=false.</x:v>
       </x:c>
       <x:c r="J39" s="39" t="str">
-        <x:v>History is useful without growing indefinitely or becoming a source-content archive.</x:v>
+        <x:v>The exact payload is visible before a request, uncommitted changes are excluded, and no external AI request is made by this slice.</x:v>
       </x:c>
       <x:c r="K39" s="39" t="str">
-        <x:v>src-tauri/src/core.rs:110-149, 1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
+        <x:v>src-tauri/src/core.rs:16-26, 2880-3065, 6340-6375; src/renderer/src/components/AiSummaryPreview.tsx; /Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211</x:v>
       </x:c>
       <x:c r="L39" s="39" t="str">
-        <x:v>Rust repeated-scan regression + source review</x:v>
+        <x:v>Rust privacy regression + renderer build + source safety review</x:v>
       </x:c>
       <x:c r="M39" s="39" t="str">
-        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline; review AI summary preview in repository preparation</x:v>
       </x:c>
       <x:c r="N39" s="39" t="str">
-        <x:v>Transition persistence passes, including same-second IDs; the 90-day default and configurable retention are represented in the core constants/logic for this slice, with action audits bounded to recent records.</x:v>
+        <x:v>Fixture proves disabled, metadata-only, and committed-diff payloads; uncommitted.txt is excluded and request_performed remains false.</x:v>
       </x:c>
       <x:c r="O39" s="39" t="str">
         <x:v>Regression-Covered</x:v>
       </x:c>
       <x:c r="P39" s="39" t="str"/>
-      <x:c r="Q39" s="39" t="str"/>
-      <x:c r="R39" s="39" t="str"/>
+      <x:c r="Q39" s="39" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="R39" s="39" t="str">
+        <x:v>Endpoint/model credential configuration and user-approved external request execution remain intentionally unimplemented.</x:v>
+      </x:c>
       <x:c r="S39" s="39" t="str">
+        <x:v>Implemented local payload preview and per-repository permission without sending data or treating AI as provider evidence.</x:v>
+      </x:c>
+      <x:c r="T39" s="39" t="str">
+        <x:v>Yes: payload privacy and no-request regression assertions.</x:v>
+      </x:c>
+      <x:c r="U39" s="39" t="str">
+        <x:v>AI remains disabled by default and any future request must preserve the preview, permission, and trace contract.</x:v>
+      </x:c>
+      <x:c r="V39" s="39" t="str">
+        <x:v>/Users/jakyeamos/Downloads/pronto_prd.md:679-695, 1205-1211; src-tauri/src/core.rs:2880-3065</x:v>
+      </x:c>
+      <x:c r="W39" s="39" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X39" s="39" t="str">
+        <x:v>c0bf758</x:v>
+      </x:c>
+      <x:c r="Y39" s="39" t="str">
+        <x:v>Keep external AI execution closed until endpoint, credential, approval, and destination-specific audit contracts are explicit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="70" customHeight="1">
+      <x:c r="A40" s="51" t="str">
+        <x:v>HIST-001</x:v>
+      </x:c>
+      <x:c r="B40" s="39" t="str">
+        <x:v>History</x:v>
+      </x:c>
+      <x:c r="C40" s="39" t="str">
+        <x:v>Event retention</x:v>
+      </x:c>
+      <x:c r="D40" s="39" t="str">
+        <x:v>As an operator, I can retain bounded transition history without losing current state.</x:v>
+      </x:c>
+      <x:c r="E40" s="39" t="str">
+        <x:v>Local operator</x:v>
+      </x:c>
+      <x:c r="F40" s="39" t="str">
+        <x:v>Local-only</x:v>
+      </x:c>
+      <x:c r="G40" s="39" t="str">
+        <x:v>Transition events persisted in local store</x:v>
+      </x:c>
+      <x:c r="H40" s="39" t="str">
+        <x:v>Native core</x:v>
+      </x:c>
+      <x:c r="I40" s="39" t="str">
+        <x:v>Events are transition-only with sequence-safe IDs, retained for a default bounded window, and action audits are bounded and pruned independently of current snapshots.</x:v>
+      </x:c>
+      <x:c r="J40" s="39" t="str">
+        <x:v>History is useful without growing indefinitely or becoming a source-content archive.</x:v>
+      </x:c>
+      <x:c r="K40" s="39" t="str">
+        <x:v>src-tauri/src/core.rs:110-149, 1220-1320; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
+      </x:c>
+      <x:c r="L40" s="39" t="str">
+        <x:v>Rust repeated-scan regression + source review</x:v>
+      </x:c>
+      <x:c r="M40" s="39" t="str">
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline</x:v>
+      </x:c>
+      <x:c r="N40" s="39" t="str">
+        <x:v>Transition persistence passes, including same-second IDs; the 90-day default and configurable retention are represented in the core constants/logic for this slice, with action audits bounded to recent records.</x:v>
+      </x:c>
+      <x:c r="O40" s="39" t="str">
+        <x:v>Regression-Covered</x:v>
+      </x:c>
+      <x:c r="P40" s="39" t="str"/>
+      <x:c r="Q40" s="39" t="str"/>
+      <x:c r="R40" s="39" t="str"/>
+      <x:c r="S40" s="39" t="str">
         <x:v>Yes: repeated-scan event regression.</x:v>
       </x:c>
-      <x:c r="T39" s="39" t="str">
+      <x:c r="T40" s="39" t="str">
         <x:v>Bounded event and action-audit history is a small persistence concern; durable configuration remains Phase 2.</x:v>
       </x:c>
-      <x:c r="U39" s="39" t="str">
+      <x:c r="U40" s="39" t="str">
         <x:v>src-tauri/src/core.rs:1671-1695, 1739-1780, 1900-1924; /Users/jakyeamos/Downloads/pronto_prd.md:699-717</x:v>
       </x:c>
-      <x:c r="V39" s="39" t="str">
+      <x:c r="V40" s="39" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W39" s="39" t="str">
-        <x:v>b13de08</x:v>
-      </x:c>
-      <x:c r="X39" s="39" t="str">
+      <x:c r="W40" s="39" t="str">
+        <x:v>c0bf758</x:v>
+      </x:c>
+      <x:c r="X40" s="39" t="str">
         <x:v>Expose retention settings and add date-boundary tests for action audits.</x:v>
       </x:c>
-      <x:c r="Y39" s="39"/>
+      <x:c r="Y40" s="39"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3671,7 +3746,7 @@
     <x:mergeCell ref="A2:Y2"/>
     <x:mergeCell ref="A3:Y3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="O5:O39">
+  <x:conditionalFormatting sqref="O5:O40">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Regression-Covered"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Verified"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Build verified"/>
@@ -3681,13 +3756,13 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="O5:O39">
+    <x:dataValidation type="list" sqref="O5:O40">
       <x:formula1>"Regression-Covered,Verified,Needs-Environment,Needs-Product-Decision,Deferred"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54b1e35410444d39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf6958eba9984929"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3758,10 +3833,10 @@
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E5" s="36" t="str">
-        <x:v>Local roots, recursion, canonical dedup, and linked worktrees are implemented. Provider matching, remote-only, clone, lifecycle confirmation, and submodule promotion remain deferred.</x:v>
+        <x:v>Local roots, recursion, canonical dedup, linked worktrees, submodule summaries, lifecycle confirmation, and privacy-safe snapshots are implemented. Remote-only clone remains deferred.</x:v>
       </x:c>
       <x:c r="F5" s="37" t="str">
-        <x:v>Phase 1 → Phase 2</x:v>
+        <x:v>Live desktop + clone authority gate</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="52" customHeight="1">
@@ -3775,13 +3850,13 @@
         <x:v>PROV-001</x:v>
       </x:c>
       <x:c r="D6" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Read-only verified</x:v>
       </x:c>
       <x:c r="E6" s="39" t="str">
-        <x:v>Requires explicit identity mapping, OS credential storage, provider interface, and permission degradation.</x:v>
+        <x:v>Authenticated GitHub identity, repository, PR, release, locality, and fetched-at snapshots persist through a provider-neutral contract; live gh auth and richer identity scope remain environment-limited.</x:v>
       </x:c>
       <x:c r="F6" s="40" t="str">
-        <x:v>Phase 2</x:v>
+        <x:v>Authenticated desktop refresh</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">
@@ -3792,16 +3867,16 @@
         <x:v>FR-016–026; AC-004–007</x:v>
       </x:c>
       <x:c r="C7" s="39" t="str">
-        <x:v>GIT-001–006</x:v>
+        <x:v>GIT-001–006; REMOTE-001</x:v>
       </x:c>
       <x:c r="D7" s="39" t="str">
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E7" s="39" t="str">
-        <x:v>Local branch, upstream, dirty aggregate, operation markers, and no-implicit-fetch boundary are implemented. Fetch policy and provider freshness remain deferred.</x:v>
+        <x:v>Local branch, upstream, dirty aggregate, operation markers, no-implicit-fetch boundary, provider locality, PR/release snapshots, and freshness are implemented. Fetch policy and clone remain gated.</x:v>
       </x:c>
       <x:c r="F7" s="40" t="str">
-        <x:v>Phase 1 → Phase 2</x:v>
+        <x:v>Freshness policy + clone authority gate</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
@@ -3838,7 +3913,7 @@
         <x:v>Partial / environment</x:v>
       </x:c>
       <x:c r="E9" s="39" t="str">
-        <x:v>Deterministic grouped queue, evidence drawer, expected fingerprints, and distinct no-data/no-match states exist; live interaction still needs a desktop pass.</x:v>
+        <x:v>Deterministic grouped queue, evidence drawer, expected fingerprints, provider-aware threshold condition, and distinct no-data/no-match states exist; live interaction still needs a desktop pass.</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>Phase 1 desktop verification</x:v>
@@ -3852,16 +3927,16 @@
         <x:v>FR-040–057; AC-011–014</x:v>
       </x:c>
       <x:c r="C10" s="39" t="str">
-        <x:v>GIT-005; UI-002</x:v>
+        <x:v>GIT-005; UI-002; HANDOFF-001; PR-001; REL-001</x:v>
       </x:c>
       <x:c r="D10" s="39" t="str">
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E10" s="39" t="str">
-        <x:v>Local workspace/branch evidence and integration heuristics exist. User corrections and safe cleanup actions are deferred.</x:v>
+        <x:v>Local workspace/branch/activity evidence, exact-tool handoff, read-only PR/release preparation, release rules, recipes, and version confirmation exist. Mutating actions remain deferred.</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
-        <x:v>Phase 2</x:v>
+        <x:v>Live desktop + mutation authority gate</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="52" customHeight="1">
@@ -3875,13 +3950,13 @@
         <x:v>PROC-001</x:v>
       </x:c>
       <x:c r="D11" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Read-only verified</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
-        <x:v>Linked worktrees are represented; process, terminal, manifest, and confidence adapters require OS-specific design and permission.</x:v>
+        <x:v>Linked worktrees now include safe manifest metadata, candidate-process signals, confidence, uncertainty, and active-workspace integration blocking; terminal capture remains absent.</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>Phase 2</x:v>
+        <x:v>Cross-platform permission matrix</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
@@ -3915,13 +3990,13 @@
         <x:v>PR-001</x:v>
       </x:c>
       <x:c r="D13" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Partial / environment</x:v>
       </x:c>
       <x:c r="E13" s="39" t="str">
-        <x:v>Provider-backed PR state and merge eligibility are not implemented.</x:v>
+        <x:v>Read-only PR snapshots and preparation evidence preserve unknown checks/reviews/mergeability and match a workspace; create/approve/merge remain outside the action surface.</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
-        <x:v>Phase 3</x:v>
+        <x:v>Provider write permission + post-action audit</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="52" customHeight="1">
@@ -3935,13 +4010,13 @@
         <x:v>REL-001</x:v>
       </x:c>
       <x:c r="D14" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Partial / environment</x:v>
       </x:c>
       <x:c r="E14" s="39" t="str">
-        <x:v>Deterministic release rules, isolated release worktrees, validation, and draft handoff are not implemented.</x:v>
+        <x:v>Published baselines, deterministic notes/bump/rules, threshold queue condition, validated recipe/version confirmation, and nine-step preview are implemented; execution/publication remain blocked.</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>Phase 3</x:v>
+        <x:v>Recipe execution + publication authority</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52" customHeight="1">
@@ -3955,13 +4030,13 @@
         <x:v>GROUP-001</x:v>
       </x:c>
       <x:c r="D15" s="39" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Read-only verified</x:v>
       </x:c>
       <x:c r="E15" s="39" t="str">
-        <x:v>Manual product/group configuration is the accepted direction; aggregation and coordinated release remain deferred until the durable state model is implemented.</x:v>
+        <x:v>Manual product/group configuration, explicit membership, product release mode, local persistence, filtering, targeted refresh, and deletion are implemented; coordinated release/aggregate health remain deferred.</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>Phase 2 design gate</x:v>
+        <x:v>Coordinated-release design gate</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
@@ -3978,10 +4053,10 @@
         <x:v>Privacy boundary</x:v>
       </x:c>
       <x:c r="E16" s="39" t="str">
-        <x:v>AI is disabled by default; local snapshots avoid filenames and diff content. Provider payload preview and per-repository permission remain intentionally absent.</x:v>
+        <x:v>AI is disabled by default; per-repository payload permission and local metadata/committed-diff previews are implemented, with uncommitted content excluded and external request execution absent.</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>Phase 2 decision gate</x:v>
+        <x:v>External AI authority gate</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
@@ -3998,10 +4073,10 @@
         <x:v>Partial / local</x:v>
       </x:c>
       <x:c r="E17" s="39" t="str">
-        <x:v>Transition-only metadata history and bounded action-audit history are implemented and surfaced in Activity; configurable retention and future schema migrations remain deferred.</x:v>
+        <x:v>Transition-only metadata history, bounded action-audit history, configurable retention, and migration-safe SQLite state are implemented and surfaced in Activity; future schema versions remain explicit.</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>Phase 2</x:v>
+        <x:v>Live desktop retention review</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="52" customHeight="1">
@@ -4038,10 +4113,10 @@
         <x:v>Build verified</x:v>
       </x:c>
       <x:c r="E19" s="42" t="str">
-        <x:v>Tauri app and macOS DMG build locally; signing/notarization and cross-platform bundles remain outside this run.</x:v>
+        <x:v>Tauri app and macOS DMG build locally from c0bf758; signing/notarization, live interaction, and cross-platform bundles remain outside this run.</x:v>
       </x:c>
       <x:c r="F19" s="43" t="str">
-        <x:v>Phase 1 build</x:v>
+        <x:v>Live macOS interaction + release signing</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4065,7 +4140,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recb18da0c7d64480"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb685b397b174427d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4106,7 +4181,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Implementation commit: b13de08 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
+        <x:v>Implementation commit: c0bf758 | PRD reviewed: 2026-07-25 | Current slice favors proof of local behavior over unverified provider breadth.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -4148,33 +4223,33 @@
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="61" t="n">
-        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$39)</x:f>
-        <x:v>35</x:v>
+        <x:f>COUNTA('Behavior Inventory'!$A$5:$A$40)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B5" s="62"/>
       <x:c r="C5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Regression-Covered")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$40,"Regression-Covered")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="62"/>
       <x:c r="E5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$39,"Build verified")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$40,"Verified")+COUNTIF('Behavior Inventory'!$O$5:$O$40,"Build verified")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F5" s="62"/>
       <x:c r="G5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Needs-Environment")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$40,"Needs-Environment")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H5" s="62"/>
       <x:c r="I5" s="61" t="n">
-        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$39,"Needs-Product-Decision")</x:f>
+        <x:f>COUNTIF('Behavior Inventory'!$O$5:$O$40,"Needs-Product-Decision")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J5" s="62"/>
       <x:c r="K5" s="63" t="n">
         <x:f>(C5+E5+G5)/(A5)</x:f>
-        <x:v>0.9428571428571428</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L5" s="64"/>
     </x:row>
@@ -4216,16 +4291,16 @@
         <x:v>Local evidence foundation</x:v>
       </x:c>
       <x:c r="C10" s="36" t="str">
-        <x:v>Discovery, structured Git facts, explainable conditions, expected fingerprints, transition history, portfolio UI, truthful local navigation, read-only CLI</x:v>
+        <x:v>Discovery, structured Git facts, explainable conditions, expected fingerprints, transition history, portfolio UI, truthful local navigation, read-only CLI, SQLite persistence</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
-        <x:v>cargo test; typecheck; lint; build:web; CLI smoke; Pre-CR</x:v>
+        <x:v>cargo test; typecheck; lint; build:web; CLI smoke; Pre-CR; Tauri build</x:v>
       </x:c>
       <x:c r="E10" s="36" t="str">
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F10" s="37" t="str">
-        <x:v>Local UX, durable SQLite state, and read-only action audit foundation are implemented at b13de08; workbook review is this iteration.</x:v>
+        <x:v>Local UX, durable state, safe read-only actions, local configuration, and distribution are implemented and regression/build verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -4233,19 +4308,19 @@
         <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="B11" s="39" t="str">
-        <x:v>Provider and safe action expansion</x:v>
+        <x:v>Read-only provider and evidence expansion</x:v>
       </x:c>
       <x:c r="C11" s="39" t="str">
-        <x:v>GitHub identities, fetch/refresh freshness, remote catalog/clone, process adapters, action preflight/audit</x:v>
+        <x:v>GitHub identity/catalog snapshots, PR/release evidence, agent/process signals, exact workspace handoff, products/groups, AI payload previews, release rules/recipe/version preflight</x:v>
       </x:c>
       <x:c r="D11" s="39" t="str">
-        <x:v>Provider permission and action audit design review</x:v>
+        <x:v>Rust regressions; typecheck; lint; renderer/Tauri builds; live provider/desktop review</x:v>
       </x:c>
       <x:c r="E11" s="39" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>Versioned SQLite and the read-only action-audit foundation are complete; read-only GitHub follows explicit identity/freshness contracts; modifying actions remain deferred.</x:v>
+        <x:v>The read-only expansion is implemented through c0bf758. Authenticated provider refresh, native desktop interaction, and OS permission behavior remain environment checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -4253,19 +4328,19 @@
         <x:v>Phase 3</x:v>
       </x:c>
       <x:c r="B12" s="42" t="str">
-        <x:v>Pull requests and releases</x:v>
+        <x:v>Mutations and publication</x:v>
       </x:c>
       <x:c r="C12" s="42" t="str">
-        <x:v>PR evidence, merge eligibility, deterministic release rules, isolated release worktrees, products/groups</x:v>
+        <x:v>Remote clone, PR create/approve/merge, recipe execution, generated-file commit/push, release publication, external AI requests, coordinated release</x:v>
       </x:c>
       <x:c r="D12" s="42" t="str">
-        <x:v>End-to-end provider and release recipe acceptance</x:v>
+        <x:v>Destination-specific authority, fresh preflight, audit, post-action verification, and human approval</x:v>
       </x:c>
       <x:c r="E12" s="42" t="str">
         <x:v>Deferred</x:v>
       </x:c>
       <x:c r="F12" s="43" t="str">
-        <x:v>No publish or merge authority is assumed in Phase 1.</x:v>
+        <x:v>No provider write, shell recipe, worktree, commit, push, merge, publish, or external AI authority is assumed.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -4334,7 +4409,7 @@
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
       <x:c r="A21" s="38" t="str">
-        <x:v>GIT_INDEX_FILE=.git/index pnpm test</x:v>
+        <x:v>pnpm test</x:v>
       </x:c>
       <x:c r="B21" s="39" t="str">
         <x:v>Rust regressions + Vitest</x:v>
@@ -4343,138 +4418,166 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D21" s="40" t="str">
-        <x:v>9 Rust tests; Vitest no test files</x:v>
+        <x:v>20 Rust tests; Vitest no test files pass through</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
       <x:c r="A22" s="38" t="str">
-        <x:v>cargo check --manifest-path src-tauri/Cargo.toml --offline</x:v>
+        <x:v>cargo test --manifest-path src-tauri/Cargo.toml --offline</x:v>
       </x:c>
       <x:c r="B22" s="39" t="str">
-        <x:v>Native compilation</x:v>
+        <x:v>Native behavioral regressions</x:v>
       </x:c>
       <x:c r="C22" s="39" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D22" s="40" t="str">
-        <x:v>Rust 1.97.1</x:v>
+        <x:v>20 tests covering provider, agent, products/groups, actions, AI, and release preparation</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="32" customHeight="1">
       <x:c r="A23" s="38" t="str">
-        <x:v>pnpm cli:json</x:v>
+        <x:v>cargo check --manifest-path src-tauri/Cargo.toml --offline</x:v>
       </x:c>
       <x:c r="B23" s="39" t="str">
-        <x:v>Shared CLI snapshot</x:v>
+        <x:v>Native compilation</x:v>
       </x:c>
       <x:c r="C23" s="39" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D23" s="40" t="str">
-        <x:v>JSON output includes the shared action_audits field</x:v>
+        <x:v>Rust 1.97.1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="32" customHeight="1">
       <x:c r="A24" s="38" t="str">
-        <x:v>pnpm build:web</x:v>
+        <x:v>pnpm cli:json</x:v>
       </x:c>
       <x:c r="B24" s="39" t="str">
-        <x:v>Renderer production build</x:v>
+        <x:v>Shared CLI snapshot</x:v>
       </x:c>
       <x:c r="C24" s="39" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>Vite production bundle emitted with safe action history wiring</x:v>
+        <x:v>JSON output uses the shared snapshot contract with action/provider/release fields</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
       <x:c r="A25" s="38" t="str">
-        <x:v>pnpm build</x:v>
+        <x:v>pnpm build:web</x:v>
       </x:c>
       <x:c r="B25" s="39" t="str">
-        <x:v>Tauri app and DMG</x:v>
+        <x:v>Renderer production build</x:v>
       </x:c>
       <x:c r="C25" s="39" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D25" s="40" t="str">
-        <x:v>Pronto.app and Pronto_0.1.0_aarch64.dmg emitted after the action-audit slice</x:v>
+        <x:v>Vite bundle: 264.96 kB JS / 33.73 kB CSS</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="38" t="str">
+        <x:v>pnpm build</x:v>
+      </x:c>
+      <x:c r="B26" s="39" t="str">
+        <x:v>Tauri app and DMG</x:v>
+      </x:c>
+      <x:c r="C26" s="39" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>Latest source emitted Pronto.app and Pronto_0.1.0_aarch64.dmg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="32" customHeight="1">
+      <x:c r="A27" s="38" t="str">
         <x:v>pre-cr run --json --workspace .</x:v>
       </x:c>
-      <x:c r="B26" s="39" t="str">
+      <x:c r="B27" s="39" t="str">
         <x:v>Commit readiness / anti-slop</x:v>
       </x:c>
-      <x:c r="C26" s="39" t="str">
-        <x:v>Not applicable</x:v>
-      </x:c>
-      <x:c r="D26" s="40" t="str">
-        <x:v>Docs/workbook-only changes are ignored by the configured source surfaces; no changed-line coverage result was produced. Source commit b13de08 passed its commit-time gate.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="32" customHeight="1">
-      <x:c r="A27" s="41" t="str">
+      <x:c r="C27" s="39" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>Source commit c0bf758 passed commit-time Pre-CR; docs-only truth commit had no changed-line source result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="32" customHeight="1">
+      <x:c r="A28" s="38" t="str">
         <x:v>git diff --check</x:v>
       </x:c>
-      <x:c r="B27" s="42" t="str">
+      <x:c r="B28" s="39" t="str">
         <x:v>Whitespace and patch hygiene</x:v>
       </x:c>
-      <x:c r="C27" s="42" t="str">
+      <x:c r="C28" s="39" t="str">
         <x:v>Pass</x:v>
       </x:c>
-      <x:c r="D27" s="43" t="str">
+      <x:c r="D28" s="40" t="str">
         <x:v>No whitespace errors</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="22" customHeight="1">
-      <x:c r="A30" s="66" t="str">
+    <x:row r="29" ht="32" customHeight="1">
+      <x:c r="A29" s="41" t="str">
+        <x:v>Workbook inspect + render</x:v>
+      </x:c>
+      <x:c r="B29" s="42" t="str">
+        <x:v>Canonical PRD evidence artifact</x:v>
+      </x:c>
+      <x:c r="C29" s="42" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="D29" s="43" t="str">
+        <x:v>Three sheets exported; zero formula errors; visual review required before commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="66" t="str">
         <x:v>Review notes</x:v>
       </x:c>
-      <x:c r="B30" s="66"/>
-      <x:c r="C30" s="66"/>
-      <x:c r="D30" s="66"/>
-      <x:c r="E30" s="66"/>
-      <x:c r="F30" s="66"/>
-      <x:c r="G30" s="66"/>
-      <x:c r="H30" s="66"/>
-      <x:c r="I30" s="66"/>
-      <x:c r="J30" s="66"/>
-      <x:c r="K30" s="66"/>
-      <x:c r="L30" s="66"/>
-    </x:row>
-    <x:row r="31" ht="26" customHeight="1">
-      <x:c r="A31" s="8" t="str">
-        <x:v>The accepted direction is now explicit: local UX first, SQLite before provider data, read-only GitHub initially, safe non-destructive local actions, macOS first, AI disabled, and manual products/groups. The local UX, durable-state, and read-only action preflight/audit slices are implemented at b13de08; the next safe expansion is read-only provider context.</x:v>
-      </x:c>
-      <x:c r="B31" s="8"/>
-      <x:c r="C31" s="8"/>
-      <x:c r="D31" s="8"/>
-      <x:c r="E31" s="8"/>
-      <x:c r="F31" s="8"/>
-      <x:c r="G31" s="8"/>
-      <x:c r="H31" s="8"/>
-      <x:c r="I31" s="8"/>
-      <x:c r="J31" s="8"/>
-      <x:c r="K31" s="8"/>
-      <x:c r="L31" s="8"/>
-    </x:row>
-    <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="8"/>
-      <x:c r="B32" s="8"/>
-      <x:c r="C32" s="8"/>
-      <x:c r="D32" s="8"/>
-      <x:c r="E32" s="8"/>
-      <x:c r="F32" s="8"/>
-      <x:c r="G32" s="8"/>
-      <x:c r="H32" s="8"/>
-      <x:c r="I32" s="8"/>
-      <x:c r="J32" s="8"/>
-      <x:c r="K32" s="8"/>
-      <x:c r="L32" s="8"/>
+      <x:c r="B32" s="66"/>
+      <x:c r="C32" s="66"/>
+      <x:c r="D32" s="66"/>
+      <x:c r="E32" s="66"/>
+      <x:c r="F32" s="66"/>
+      <x:c r="G32" s="66"/>
+      <x:c r="H32" s="66"/>
+      <x:c r="I32" s="66"/>
+      <x:c r="J32" s="66"/>
+      <x:c r="K32" s="66"/>
+      <x:c r="L32" s="66"/>
+    </x:row>
+    <x:row r="33" ht="26" customHeight="1">
+      <x:c r="A33" s="8" t="str">
+        <x:v>The accepted direction is now explicit: local UX first, versioned SQLite, read-only GitHub, safe non-destructive local actions, macOS first, AI disabled by default with local payload preview, and manual products/groups. The local and read-only evidence slices are implemented through c0bf758. Remaining boundaries are destination-specific provider writes, recipe execution, worktree/commit/push/PR/release publication, external AI requests, signing, and live desktop/provider verification.</x:v>
+      </x:c>
+      <x:c r="B33" s="8"/>
+      <x:c r="C33" s="8"/>
+      <x:c r="D33" s="8"/>
+      <x:c r="E33" s="8"/>
+      <x:c r="F33" s="8"/>
+      <x:c r="G33" s="8"/>
+      <x:c r="H33" s="8"/>
+      <x:c r="I33" s="8"/>
+      <x:c r="J33" s="8"/>
+      <x:c r="K33" s="8"/>
+      <x:c r="L33" s="8"/>
+    </x:row>
+    <x:row r="34" ht="26" customHeight="1">
+      <x:c r="A34" s="8"/>
+      <x:c r="B34" s="8"/>
+      <x:c r="C34" s="8"/>
+      <x:c r="D34" s="8"/>
+      <x:c r="E34" s="8"/>
+      <x:c r="F34" s="8"/>
+      <x:c r="G34" s="8"/>
+      <x:c r="H34" s="8"/>
+      <x:c r="I34" s="8"/>
+      <x:c r="J34" s="8"/>
+      <x:c r="K34" s="8"/>
+      <x:c r="L34" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4494,8 +4597,8 @@
     <x:mergeCell ref="K5:L5"/>
     <x:mergeCell ref="A8:F8"/>
     <x:mergeCell ref="A16:D16"/>
-    <x:mergeCell ref="A30:L30"/>
-    <x:mergeCell ref="A31:L32"/>
+    <x:mergeCell ref="A32:L32"/>
+    <x:mergeCell ref="A33:L34"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E10:E12">
     <x:cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="Regression-Covered"/>
@@ -4506,7 +4609,7 @@
     <x:cfRule type="containsText" dxfId="19" priority="6" operator="containsText" text="Product decision"/>
     <x:cfRule type="containsText" dxfId="20" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="C18:C27">
+  <x:conditionalFormatting sqref="C18:C29">
     <x:cfRule type="containsText" dxfId="21" priority="8" operator="containsText" text="Regression-Covered"/>
     <x:cfRule type="containsText" dxfId="22" priority="9" operator="containsText" text="Verified"/>
     <x:cfRule type="containsText" dxfId="23" priority="10" operator="containsText" text="Build verified"/>

</xml_diff>